<commit_message>
System FMEA rev 0.9: baseline BL-005, MSR re-rated with the host supervision
BL-005 pins liondriver-dev 1033d98 (panda a55bdfc, opendbc 9a13f60). The
reference build is the default at BL-005, so its panda checks are credited.
Each claim was checked against the code at these pins.

- TSR-621: controlsMismatch within 0.5 s; SFM-015.C2 M 8 -> 6, D 10 -> 8
- TSR-408 + TSR-621: TX arrival then host alert; SFM-005.C2, SFM-011.C2 -> M 6
- TSR-615: pandaTxBlocked on refused frames (SFM-002/008/009, M stays 5)
- TSR-308: cruiseMismatch alert after 1 s; SFM-021 M 9 -> 7
- Reference lock: SFM-032.C1 M 9 -> 8
- SFM-ACT-008/015/018 in progress; msr-plan v0.5, fmea-plan v0.10
- Review pages, workbook and figures regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.8 · draft</t>
+          <t>0.9 · draft</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>BL-004</t>
+          <t>BL-005</t>
         </is>
       </c>
     </row>
@@ -838,11 +838,11 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
+    <row r="10" ht="105" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Scope</t>
@@ -850,7 +850,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>LionDriver as installed on the reference configuration CFG-001 (Corolla E210 · ZRE212 · US, US sedan MY2020-2022) with comma 3X and integrated panda, software BL-004 (structure and failure analysis written at BL-001, risk analysis at BL-004), while the vehicle is driven on public roads by a licensed driver. Functions F1-F7 per fmea-plan.md section 3.1, plus F8 (stock vehicle safety functions are preserved), added because the harness intercepts the stock ADAS camera.</t>
+          <t>LionDriver as installed on the reference configuration CFG-001 (Corolla E210 · ZRE212 · US, US sedan MY2020-2022) with comma 3X and integrated panda, software BL-005 (structure and failure analysis written at BL-001, risk analysis at BL-004, MSR re-rated at BL-005), while the vehicle is driven on public roads by a licensed driver. Functions F1-F7 per fmea-plan.md section 3.1, plus F8 (stock vehicle safety functions are preserved), added because the harness intercepts the stock ADAS camera.</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8272,7 @@
       <c r="R44" s="37" t="inlineStr"/>
       <c r="S44" s="37" t="inlineStr"/>
     </row>
-    <row r="45" ht="195" customHeight="1">
+    <row r="45" ht="222" customHeight="1">
       <c r="A45" s="38" t="n"/>
       <c r="B45" s="38" t="n"/>
       <c r="C45" s="38" t="n"/>
@@ -8330,7 +8330,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• selfdrived raises controlsMismatch (IMMEDIATE_DISABLE) when the panda reports controls not allowed while engaged, but only after 200 frames (2 s at 100 Hz)</t>
+            <t>• selfdrived raises controlsMismatch (IMMEDIATE_DISABLE) when the panda reports controls not allowed while engaged, after 2 consecutive pandaStates samples and at most 0.5 s (BL-005, TSR-621; 200 cumulative frames, about 2 s, at BL-004)</t>
           </r>
           <r>
             <rPr>
@@ -8339,7 +8339,7 @@
               <sz val="8"/>
             </rPr>
             <t xml:space="preserve">
-   openpilot/selfdrive/selfdrived/selfdrived.py:338</t>
+   openpilot/selfdrive/selfdrived/supervision.py</t>
           </r>
         </is>
       </c>
@@ -8351,15 +8351,24 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="008A5A00"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• No pre-release test targets this cause</t>
-          </r>
-        </is>
-      </c>
-      <c r="L45" s="46" t="n">
-        <v>10</v>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• BL-005: test_supervision.py checks the 2-sample and 0.5 s bounds and the 0.3 s engagement grace of controlsMismatch (tests.yaml unit_tests on every push and PR); targeted, not proven by mutation (RT-1 D 8). At BL-004 no test targeted this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/selfdrived/tests/test_supervision.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L45" s="35" t="n">
+        <v>8</v>
       </c>
       <c r="M45" s="36" t="inlineStr">
         <is>
@@ -14689,9 +14698,9 @@
           </r>
         </is>
       </c>
-      <c r="O78" s="48" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="O78" s="50" t="inlineStr">
+        <is>
+          <t>in progress</t>
         </is>
       </c>
       <c r="P78" s="40" t="inlineStr"/>
@@ -15666,7 +15675,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.8 · BL-004&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.9 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -15997,7 +16006,7 @@
       <c r="H7" s="59" t="inlineStr"/>
       <c r="I7" s="59" t="inlineStr"/>
     </row>
-    <row r="8" ht="46.5" customHeight="1">
+    <row r="8" ht="73.5" customHeight="1">
       <c r="A8" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-008</t>
@@ -16020,7 +16029,7 @@
       </c>
       <c r="E8" s="59" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>in progress</t>
         </is>
       </c>
       <c r="F8" s="59" t="inlineStr">
@@ -16030,7 +16039,11 @@
       </c>
       <c r="G8" s="59" t="inlineStr"/>
       <c r="H8" s="59" t="inlineStr"/>
-      <c r="I8" s="59" t="inlineStr"/>
+      <c r="I8" s="59" t="inlineStr">
+        <is>
+          <t>BL-005: the reference build is the default (LionDriver #36), the panda accepts only TOYOTA parameter 73 (reference_lock.h) and pandad configures a car mode only on a reference panda (#41). Fuzzy fingerprint matches are still accepted on the host (SFM-032.C1)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="100.5" customHeight="1">
       <c r="A9" s="59" t="inlineStr">
@@ -16073,7 +16086,7 @@
       <c r="H9" s="59" t="inlineStr"/>
       <c r="I9" s="59" t="inlineStr"/>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10" ht="73.5" customHeight="1">
       <c r="A10" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-010</t>
@@ -16111,7 +16124,7 @@
       <c r="H10" s="59" t="inlineStr"/>
       <c r="I10" s="59" t="inlineStr">
         <is>
-          <t>controlsMismatch debounce cut from 200 cumulative samples (~2 s) to 2 consecutive samples, at most 0.5 s (change-2026-10-13-host-supervision.md); FTTI justification of SOFT_DISABLE reactions open</t>
+          <t>controlsMismatch debounce cut from 200 cumulative samples (~2 s) to 2 consecutive samples, at most 0.5 s (change-2026-10-13-host-supervision.md); credited at BL-005 (SFM-015.C2 M 6). FTTI justification of SOFT_DISABLE reactions open</t>
         </is>
       </c>
     </row>
@@ -16182,7 +16195,7 @@
       <c r="H12" s="59" t="inlineStr"/>
       <c r="I12" s="59" t="inlineStr"/>
     </row>
-    <row r="13" ht="46.5" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-013</t>
@@ -16195,7 +16208,7 @@
       </c>
       <c r="C13" s="59" t="inlineStr">
         <is>
-          <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the BL-004 controlsMismatch counter), with a disable and an alert</t>
+          <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert</t>
         </is>
       </c>
       <c r="D13" s="59" t="inlineStr"/>
@@ -16236,7 +16249,7 @@
       <c r="H14" s="59" t="inlineStr"/>
       <c r="I14" s="59" t="inlineStr"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="87" customHeight="1">
       <c r="A15" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-015</t>
@@ -16255,13 +16268,17 @@
       <c r="D15" s="59" t="inlineStr"/>
       <c r="E15" s="59" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>in progress</t>
         </is>
       </c>
       <c r="F15" s="59" t="inlineStr"/>
       <c r="G15" s="59" t="inlineStr"/>
       <c r="H15" s="59" t="inlineStr"/>
-      <c r="I15" s="59" t="inlineStr"/>
+      <c r="I15" s="59" t="inlineStr">
+        <is>
+          <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="46.5" customHeight="1">
       <c r="A16" s="59" t="inlineStr">
@@ -16317,7 +16334,7 @@
       <c r="H17" s="59" t="inlineStr"/>
       <c r="I17" s="59" t="inlineStr"/>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="73.5" customHeight="1">
       <c r="A18" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-018</t>
@@ -16336,13 +16353,17 @@
       <c r="D18" s="59" t="inlineStr"/>
       <c r="E18" s="59" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>in progress</t>
         </is>
       </c>
       <c r="F18" s="59" t="inlineStr"/>
       <c r="G18" s="59" t="inlineStr"/>
       <c r="H18" s="59" t="inlineStr"/>
-      <c r="I18" s="59" t="inlineStr"/>
+      <c r="I18" s="59" t="inlineStr">
+        <is>
+          <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1; TSR-626)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I18"/>

</xml_diff>

<commit_message>
System FMEA rev 0.10: record the lead's answers DQ-022, DQ-053, DQ-060, DQ-205
- DQ-060: new action SFM-ACT-019 (panda keeps steering authority revoked
  after a rejected frame until re-engagement, TSR-108) on SFM-002.C1/C2/C4
- DQ-053: SFM-ACT-016 behaviour fixed (back off on override, show a cue)
- DQ-022: SFM-020 note (accelerator pauses longitudinal control only)
- DQ-205: SFM-025 note and SFM-ACT-005 (SG-010 ASIL A safe state)
No rating changes: the decided behaviour is not implemented at BL-005.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$82</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -802,7 +802,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.9 · draft</t>
+          <t>0.10 · draft</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>17 (16)</t>
+          <t>18 (17)</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       <c r="R5" s="45" t="inlineStr"/>
       <c r="S5" s="45" t="inlineStr"/>
     </row>
-    <row r="6" ht="100.5" customHeight="1">
+    <row r="6" ht="195" customHeight="1">
       <c r="A6" s="30" t="inlineStr">
         <is>
           <r>
@@ -1926,11 +1926,39 @@
             </rPr>
             <t>Derive steering and acceleration envelopes from measurements on the reference vehicle and set the panda limits from them, independently of the SoC limits (same as SWF-ACT-003, FSC FOI-001)</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-019 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
+          </r>
         </is>
       </c>
       <c r="O6" s="47" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>open
+open</t>
         </is>
       </c>
       <c r="P6" s="33" t="inlineStr"/>
@@ -1938,7 +1966,7 @@
       <c r="R6" s="37" t="inlineStr"/>
       <c r="S6" s="37" t="inlineStr"/>
     </row>
-    <row r="7" ht="168" customHeight="1">
+    <row r="7" ht="276" customHeight="1">
       <c r="A7" s="38" t="n"/>
       <c r="B7" s="38" t="n"/>
       <c r="C7" s="38" t="n"/>
@@ -2053,11 +2081,39 @@
             </rPr>
             <t>Produce SOTIF / ISO PAS 8800 evidence for the neural-network elements (driving model, lead detection, driver monitoring model) per WP-V-02..04, including fault-induced inputs (corrupted or stale frames)</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-019 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
+          </r>
         </is>
       </c>
       <c r="O7" s="47" t="inlineStr">
         <is>
           <t>open
+open
 open</t>
         </is>
       </c>
@@ -2210,7 +2266,7 @@
       <c r="R8" s="37" t="inlineStr"/>
       <c r="S8" s="37" t="inlineStr"/>
     </row>
-    <row r="9" ht="195" customHeight="1">
+    <row r="9" ht="289.5" customHeight="1">
       <c r="A9" s="39" t="n"/>
       <c r="B9" s="39" t="n"/>
       <c r="C9" s="39" t="n"/>
@@ -2360,11 +2416,39 @@
             </rPr>
             <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-019 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
+          </r>
         </is>
       </c>
       <c r="O9" s="48" t="inlineStr">
         <is>
           <t>open
+open
 open</t>
         </is>
       </c>
@@ -11563,7 +11647,7 @@
       <c r="R62" s="45" t="inlineStr"/>
       <c r="S62" s="45" t="inlineStr"/>
     </row>
-    <row r="63" ht="100.5" customHeight="1">
+    <row r="63" ht="114" customHeight="1">
       <c r="A63" s="51" t="inlineStr">
         <is>
           <r>
@@ -11800,7 +11884,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004) and implement the decision</t>
+            <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (ASIL A); the reaction itself is still to be decided</t>
           </r>
         </is>
       </c>
@@ -15675,7 +15759,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.9 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.10 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -15690,7 +15774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15895,7 +15979,7 @@
       <c r="H4" s="59" t="inlineStr"/>
       <c r="I4" s="59" t="inlineStr"/>
     </row>
-    <row r="5" ht="46.5" customHeight="1">
+    <row r="5" ht="73.5" customHeight="1">
       <c r="A5" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-005</t>
@@ -15908,7 +15992,7 @@
       </c>
       <c r="C5" s="59" t="inlineStr">
         <is>
-          <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004) and implement the decision</t>
+          <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (ASIL A); the reaction itself is still to be decided</t>
         </is>
       </c>
       <c r="D5" s="59" t="inlineStr">
@@ -16280,7 +16364,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="46.5" customHeight="1">
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-016</t>
@@ -16293,7 +16377,7 @@
       </c>
       <c r="C16" s="59" t="inlineStr">
         <is>
-          <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304)</t>
+          <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue</t>
         </is>
       </c>
       <c r="D16" s="59" t="inlineStr"/>
@@ -16365,8 +16449,41 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="59" t="inlineStr">
+        <is>
+          <t>SFM-ACT-019</t>
+        </is>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>design change</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr"/>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>SFM-002.C1
+SFM-002.C2
+SFM-002.C4</t>
+        </is>
+      </c>
+      <c r="G19" s="59" t="inlineStr"/>
+      <c r="H19" s="59" t="inlineStr"/>
+      <c r="I19" s="59" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I18"/>
+  <autoFilter ref="A1:I19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
System FMEA rev 0.11: cite the plant-model results as MSR evidence
The closed-loop plant model (assurance/sim, plant 776239d, real panda
safety code in the loop) is cited as evidence on 13 MSR rows, per
msr-plan §4.2 (#116): F-02 on SFM-001.C1/C3, F-01a/F-01b on SFM-002,
F-04b on SFM-005.C2 and SFM-006.C1, F-03 on SFM-006.C2, L-01..L-04 on
SFM-008 and SFM-009. A cross-check of the code-derived times only: no
S/O/D, M or MSR AP change, and no credit for EPS, PCM or driver
behaviour, which are assumptions in the model.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.10 · draft</t>
+          <t>0.11 · draft</t>
         </is>
       </c>
     </row>
@@ -15759,7 +15759,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.10 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.11 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.12: harness-box intercept switch per the DFMEA at BL-005
Taken in from the DFMEA re-baseline (#102, RR-2026-010): the harness-box
"relay" is two DG419LE analog switches, pulled down to pass-through,
powered from the box supply, with no state feedback.
- SFM-034 and SFM-033.C1, SFM-SE-003/004, SFM-ACT-003 reworded
- SFM-034.C1 O 3 -> 4 (inherits DFM-010.C4); SFM-034.C2 D 10 -> 9
  (inherits DFM-011); AP unchanged (H)
- New SFM-033.C3: box supply lost or switch channel open cuts the
  stock camera off (DFM-020, DFM-013; O 5 D 10 AP H, SFM-ACT-003)
- SFM-015.C3 rationale names DFM-020 (box supply loss unpowers the device)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$83</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
@@ -802,7 +802,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.11 · draft</t>
+          <t>0.12 · draft</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16">
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17">
@@ -1057,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S82"/>
+  <dimension ref="A1:S83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2720,7 +2720,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -2829,7 +2829,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3081,7 +3081,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3414,7 +3414,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3550,7 +3550,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3784,7 +3784,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -4862,7 +4862,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -5420,7 +5420,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -5511,7 +5511,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -6015,7 +6015,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -6483,7 +6483,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -6716,7 +6716,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -7079,7 +7079,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -7552,7 +7552,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -8595,7 +8595,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -9242,7 +9242,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -9606,7 +9606,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -9970,7 +9970,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -10221,7 +10221,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -11040,7 +11040,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -12315,7 +12315,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -12658,7 +12658,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -13122,7 +13122,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -14447,7 +14447,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -14906,7 +14906,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Stock ADAS camera messages blocked or replaced by the harness relay</t>
+            <t>Stock ADAS camera messages blocked or replaced by the harness-box intercept</t>
           </r>
         </is>
       </c>
@@ -14954,7 +14954,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Relay intercepts stock camera messages the vehicle needs for AEB</t>
+            <t>The intercept routes the stock camera messages the vehicle needs for AEB through the panda</t>
           </r>
         </is>
       </c>
@@ -14966,7 +14966,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Forwarding keeps stock pre-collision messages (0x283, 0x344) passing the relay (SWF-011); which TSS2 functions remain with openpilot longitudinal is not established</t>
+            <t>• Forwarding keeps stock pre-collision messages (0x283, 0x344) passing the intercept (SWF-011); which TSS2 functions remain with openpilot longitudinal is not established</t>
           </r>
           <r>
             <rPr>
@@ -15035,18 +15035,18 @@
       <c r="S79" s="37" t="inlineStr"/>
     </row>
     <row r="80" ht="100.5" customHeight="1">
-      <c r="A80" s="39" t="n"/>
-      <c r="B80" s="39" t="n"/>
-      <c r="C80" s="39" t="n"/>
-      <c r="D80" s="39" t="n"/>
-      <c r="E80" s="39" t="n"/>
-      <c r="F80" s="39" t="n"/>
-      <c r="G80" s="40" t="inlineStr">
+      <c r="A80" s="38" t="n"/>
+      <c r="B80" s="38" t="n"/>
+      <c r="C80" s="38" t="n"/>
+      <c r="D80" s="38" t="n"/>
+      <c r="E80" s="38" t="n"/>
+      <c r="F80" s="38" t="n"/>
+      <c r="G80" s="33" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="H80" s="41" t="inlineStr">
+      <c r="H80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15067,7 +15067,7 @@
           </r>
         </is>
       </c>
-      <c r="I80" s="41" t="inlineStr">
+      <c r="I80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15088,10 +15088,10 @@
           </r>
         </is>
       </c>
-      <c r="J80" s="42" t="n">
+      <c r="J80" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="K80" s="41" t="inlineStr">
+      <c r="K80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15112,15 +15112,15 @@
           </r>
         </is>
       </c>
-      <c r="L80" s="42" t="n">
+      <c r="L80" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="M80" s="44" t="inlineStr">
+      <c r="M80" s="36" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="N80" s="41" t="inlineStr">
+      <c r="N80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15142,18 +15142,103 @@
           </r>
         </is>
       </c>
-      <c r="O80" s="48" t="inlineStr">
+      <c r="O80" s="47" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="P80" s="40" t="inlineStr"/>
-      <c r="Q80" s="40" t="inlineStr"/>
-      <c r="R80" s="45" t="inlineStr"/>
-      <c r="S80" s="45" t="inlineStr"/>
+      <c r="P80" s="33" t="inlineStr"/>
+      <c r="Q80" s="33" t="inlineStr"/>
+      <c r="R80" s="37" t="inlineStr"/>
+      <c r="S80" s="37" t="inlineStr"/>
     </row>
-    <row r="81" ht="87" customHeight="1">
-      <c r="A81" s="30" t="inlineStr">
+    <row r="81" ht="141" customHeight="1">
+      <c r="A81" s="39" t="n"/>
+      <c r="B81" s="39" t="n"/>
+      <c r="C81" s="39" t="n"/>
+      <c r="D81" s="39" t="n"/>
+      <c r="E81" s="39" t="n"/>
+      <c r="F81" s="39" t="n"/>
+      <c r="G81" s="40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="H81" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The harness box loses its supply (ignition branch or D1 open without comma power, VIN shorted), or a switch channel opens, so the stock camera path through the unpowered or open DG419LE switches is cut (RR-2026-010)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: DFM-020</t>
+          </r>
+        </is>
+      </c>
+      <c r="I81" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Consumer-grade harness box without automotive qualification data available to LionDriver; rated in the DFMEA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/08-analyses/fmea/analyses/dfmea.yaml</t>
+          </r>
+        </is>
+      </c>
+      <c r="J81" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K81" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the DFMEA: no pre-release test of this hardware fault</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/08-analyses/fmea/analyses/dfmea.yaml</t>
+          </r>
+        </is>
+      </c>
+      <c r="L81" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="M81" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N81" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15162,6 +15247,39 @@
               <color rgb="001F4E8C"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">SFM-ACT-003 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+          </r>
+        </is>
+      </c>
+      <c r="O81" s="48" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P81" s="40" t="inlineStr"/>
+      <c r="Q81" s="40" t="inlineStr"/>
+      <c r="R81" s="45" t="inlineStr"/>
+      <c r="S81" s="45" t="inlineStr"/>
+    </row>
+    <row r="82" ht="87" customHeight="1">
+      <c r="A82" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">SFM-SE-001
 </t>
           </r>
@@ -15175,7 +15293,7 @@
           </r>
         </is>
       </c>
-      <c r="B81" s="30" t="inlineStr">
+      <c r="B82" s="30" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15197,7 +15315,7 @@
           </r>
         </is>
       </c>
-      <c r="C81" s="30" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15318,21 +15436,21 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Relay stuck or intermittent; stock camera and item both on bus, or neither</t>
-          </r>
-        </is>
-      </c>
-      <c r="D81" s="31" t="inlineStr">
+            <t>Intercept switch stuck or intermittent: in intercept when released (camera cut off from the car), or in pass-through when driven (stock camera and item both on the bus)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D82" s="31" t="inlineStr">
         <is>
           <t>HZ-011
 HZ-002
 HZ-006</t>
         </is>
       </c>
-      <c r="E81" s="32" t="n">
+      <c r="E82" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="F81" s="30" t="inlineStr">
+      <c r="F82" s="30" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15351,24 +15469,24 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Harness relay fault</t>
-          </r>
-        </is>
-      </c>
-      <c r="G81" s="33" t="inlineStr">
+            <t>Harness-box intercept switch stuck or in the wrong position</t>
+          </r>
+        </is>
+      </c>
+      <c r="G82" s="33" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="H81" s="34" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Relay contact wear or connector fault</t>
+      <c r="H82" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
           </r>
           <r>
             <rPr>
@@ -15381,7 +15499,7 @@
           </r>
         </is>
       </c>
-      <c r="I81" s="34" t="inlineStr">
+      <c r="I82" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15402,10 +15520,10 @@
           </r>
         </is>
       </c>
-      <c r="J81" s="35" t="n">
-        <v>3</v>
-      </c>
-      <c r="K81" s="34" t="inlineStr">
+      <c r="J82" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="K82" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15426,15 +15544,15 @@
           </r>
         </is>
       </c>
-      <c r="L81" s="46" t="n">
+      <c r="L82" s="46" t="n">
         <v>10</v>
       </c>
-      <c r="M81" s="36" t="inlineStr">
+      <c r="M82" s="36" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="N81" s="34" t="inlineStr">
+      <c r="N82" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15451,37 +15569,37 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Hardware fault rated in the DFMEA (DFM-010 O3 D10, DFM-011 O3 D9); this row inherits that rating; relayMalfunction (SWF-012) is the in-field mechanism</t>
-          </r>
-        </is>
-      </c>
-      <c r="O81" s="34" t="inlineStr"/>
-      <c r="P81" s="33" t="inlineStr"/>
-      <c r="Q81" s="33" t="inlineStr"/>
-      <c r="R81" s="37" t="inlineStr"/>
-      <c r="S81" s="37" t="inlineStr"/>
+            <t>Hardware fault rated in the DFMEA (DFM-010.C1-C3 O3 D10, DFM-010.C4 O4 D10); this row inherits the worst. relayMalfunction (SWF-012) is the in-field mechanism; there is no switch-state feedback (RR-2026-010)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O82" s="34" t="inlineStr"/>
+      <c r="P82" s="33" t="inlineStr"/>
+      <c r="Q82" s="33" t="inlineStr"/>
+      <c r="R82" s="37" t="inlineStr"/>
+      <c r="S82" s="37" t="inlineStr"/>
     </row>
-    <row r="82" ht="87" customHeight="1">
-      <c r="A82" s="39" t="n"/>
-      <c r="B82" s="39" t="n"/>
-      <c r="C82" s="39" t="n"/>
-      <c r="D82" s="39" t="n"/>
-      <c r="E82" s="39" t="n"/>
-      <c r="F82" s="39" t="n"/>
-      <c r="G82" s="40" t="inlineStr">
+    <row r="83" ht="102" customHeight="1">
+      <c r="A83" s="39" t="n"/>
+      <c r="B83" s="39" t="n"/>
+      <c r="C83" s="39" t="n"/>
+      <c r="D83" s="39" t="n"/>
+      <c r="E83" s="39" t="n"/>
+      <c r="F83" s="39" t="n"/>
+      <c r="G83" s="40" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="H82" s="41" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Relay drive output fault on panda</t>
+      <c r="H83" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
           </r>
           <r>
             <rPr>
@@ -15494,7 +15612,7 @@
           </r>
         </is>
       </c>
-      <c r="I82" s="41" t="inlineStr">
+      <c r="I83" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15515,10 +15633,10 @@
           </r>
         </is>
       </c>
-      <c r="J82" s="42" t="n">
+      <c r="J83" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="K82" s="41" t="inlineStr">
+      <c r="K83" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15539,15 +15657,15 @@
           </r>
         </is>
       </c>
-      <c r="L82" s="43" t="n">
-        <v>10</v>
-      </c>
-      <c r="M82" s="44" t="inlineStr">
+      <c r="L83" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="M83" s="44" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="N82" s="41" t="inlineStr">
+      <c r="N83" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15564,24 +15682,22 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Hardware fault rated in the DFMEA (DFM-011, DFM-010); this row inherits that rating</t>
-          </r>
-        </is>
-      </c>
-      <c r="O82" s="41" t="inlineStr"/>
-      <c r="P82" s="40" t="inlineStr"/>
-      <c r="Q82" s="40" t="inlineStr"/>
-      <c r="R82" s="45" t="inlineStr"/>
-      <c r="S82" s="45" t="inlineStr"/>
+            <t>Hardware fault rated in the DFMEA (DFM-011.C1 O3 D9, DFM-011.C2 O2 D9); this row inherits the worst</t>
+          </r>
+        </is>
+      </c>
+      <c r="O83" s="41" t="inlineStr"/>
+      <c r="P83" s="40" t="inlineStr"/>
+      <c r="Q83" s="40" t="inlineStr"/>
+      <c r="R83" s="45" t="inlineStr"/>
+      <c r="S83" s="45" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:S82"/>
+  <autoFilter ref="A2:S83"/>
   <mergeCells count="172">
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="E39:E40"/>
-    <mergeCell ref="C79:C80"/>
     <mergeCell ref="A57:A59"/>
-    <mergeCell ref="E79:E80"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="F25:F28"/>
     <mergeCell ref="A51:A52"/>
@@ -15591,7 +15707,6 @@
     <mergeCell ref="C32:C34"/>
     <mergeCell ref="E32:E34"/>
     <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F79:F80"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="D20:D22"/>
     <mergeCell ref="E3:E5"/>
@@ -15600,7 +15715,6 @@
     <mergeCell ref="F29:F31"/>
     <mergeCell ref="F47:F48"/>
     <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F81:F82"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="B37:B38"/>
     <mergeCell ref="C71:C74"/>
@@ -15616,6 +15730,7 @@
     <mergeCell ref="E44:E46"/>
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="C69:C70"/>
+    <mergeCell ref="F79:F81"/>
     <mergeCell ref="D57:D59"/>
     <mergeCell ref="N1:Q1"/>
     <mergeCell ref="D41:D43"/>
@@ -15624,7 +15739,6 @@
     <mergeCell ref="B35:B36"/>
     <mergeCell ref="F10:F13"/>
     <mergeCell ref="D49:D50"/>
-    <mergeCell ref="A79:A80"/>
     <mergeCell ref="E55:E56"/>
     <mergeCell ref="A32:A34"/>
     <mergeCell ref="A14:A16"/>
@@ -15648,37 +15762,38 @@
     <mergeCell ref="D37:D38"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="B55:B56"/>
+    <mergeCell ref="C82:C83"/>
     <mergeCell ref="D55:D56"/>
+    <mergeCell ref="C79:C81"/>
     <mergeCell ref="I1:M1"/>
+    <mergeCell ref="E79:E81"/>
     <mergeCell ref="D39:D40"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="D79:D80"/>
-    <mergeCell ref="E81:E82"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="B29:B31"/>
     <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B81:B82"/>
     <mergeCell ref="D32:D34"/>
     <mergeCell ref="C49:C50"/>
-    <mergeCell ref="D81:D82"/>
     <mergeCell ref="F32:F34"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="E67:E68"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="E51:E52"/>
     <mergeCell ref="C17:C19"/>
+    <mergeCell ref="E82:E83"/>
     <mergeCell ref="E60:E61"/>
     <mergeCell ref="E69:E70"/>
     <mergeCell ref="A25:A28"/>
     <mergeCell ref="B71:B74"/>
+    <mergeCell ref="B82:B83"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="F51:F52"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A64:A66"/>
+    <mergeCell ref="A79:A81"/>
     <mergeCell ref="B41:B43"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="B10:B13"/>
@@ -15725,20 +15840,22 @@
     <mergeCell ref="C25:C28"/>
     <mergeCell ref="A55:A56"/>
     <mergeCell ref="C55:C56"/>
+    <mergeCell ref="B79:B81"/>
     <mergeCell ref="B32:B34"/>
+    <mergeCell ref="D79:D81"/>
     <mergeCell ref="C67:C68"/>
     <mergeCell ref="E17:E19"/>
     <mergeCell ref="D71:D74"/>
     <mergeCell ref="E75:E76"/>
     <mergeCell ref="A47:A48"/>
-    <mergeCell ref="A81:A82"/>
     <mergeCell ref="D17:D19"/>
-    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="F82:F83"/>
     <mergeCell ref="D67:D68"/>
     <mergeCell ref="F67:F68"/>
     <mergeCell ref="B51:B52"/>
     <mergeCell ref="E47:E48"/>
     <mergeCell ref="D51:D52"/>
+    <mergeCell ref="D82:D83"/>
     <mergeCell ref="D60:D61"/>
     <mergeCell ref="F60:F61"/>
     <mergeCell ref="C37:C38"/>
@@ -15747,11 +15864,12 @@
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="F69:F70"/>
     <mergeCell ref="B25:B28"/>
+    <mergeCell ref="A82:A83"/>
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="C6:C9"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15759,7 +15877,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.11 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.12 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -15921,7 +16039,7 @@
       <c r="H3" s="59" t="inlineStr"/>
       <c r="I3" s="59" t="inlineStr"/>
     </row>
-    <row r="4" ht="330" customHeight="1">
+    <row r="4" ht="343.5" customHeight="1">
       <c r="A4" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-003</t>
@@ -15934,7 +16052,7 @@
       </c>
       <c r="C4" s="59" t="inlineStr">
         <is>
-          <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+          <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
         </is>
       </c>
       <c r="D4" s="59" t="inlineStr">
@@ -15972,7 +16090,8 @@
 SFM-026.C2
 SFM-027.C1
 SFM-028.C2
-SFM-031.C1</t>
+SFM-031.C1
+SFM-033.C3</t>
         </is>
       </c>
       <c r="G4" s="59" t="inlineStr"/>

</xml_diff>

<commit_message>
System FMEA rev 0.13: SFM-035, the item sends a frame that alters stock PCS (FTA BE-7.08)
New failure mode SFM-035 under F8, the System FMEA backing the SG-07
fault tree asks for in BE-7.08 (WP-A-04 F-17):
- C1 host QM fault sends 0x344/0x411/DSU IDs or a non-zero 0x283:
  O 6 D 9 AP H; MSR M 5 on the panda per-frame whitelist and content
  check (mutation-tested in both variants), pandaTxBlocked while engaged
- C3 the gate itself lets the frame through: O 5 D 3 AP H; MSR M 10
  (dual point with C1, FTA MCS-07.7)
Links: fta-fmea-map BE-7.08 -> SFM-035; SFM-035 recorded as a tree_gap
for SG-04 (HZ-006) for the FTA owner; hara.yaml HZ-006/HZ-011 sfm_refs
back-links; fta-SG-07-1.svg regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$85</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
@@ -802,7 +802,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.12 · draft</t>
+          <t>0.13 · draft</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15">
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16">
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17">
@@ -1057,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S83"/>
+  <dimension ref="A1:S85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15692,9 +15692,387 @@
       <c r="R83" s="45" t="inlineStr"/>
       <c r="S83" s="45" t="inlineStr"/>
     </row>
+    <row r="84" ht="100.5" customHeight="1">
+      <c r="A84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-SE-001
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-FN-008
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>F8 Stock function preservation: keep stock vehicle safety functions not replaced by the item available</t>
+          </r>
+        </is>
+      </c>
+      <c r="C84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock AEB/FCW degraded while the driver relies on it</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-006: PCS braking triggered by a frame from the item</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock PCS warning or braking suppressed, altered or triggered by the item</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>A PCS-relevant frame from the SoC (0x344 PRE_COLLISION_2, 0x411 PCS_HUD, a DSU-only ID, or 0x283 PRE_COLLISION with a non-zero payload) reaches the car bus</t>
+          </r>
+        </is>
+      </c>
+      <c r="D84" s="31" t="inlineStr">
+        <is>
+          <t>HZ-011
+HZ-006</t>
+        </is>
+      </c>
+      <c r="E84" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-035 · unintended
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Item sends a frame that alters the stock pre-collision function</t>
+          </r>
+        </is>
+      </c>
+      <c r="G84" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Host code (car interface, pandad) emits a PCS-relevant ID or a non-zero PRE_COLLISION payload (QM fault)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream opendbc Toyota port; no carcontroller path builds 0x344, 0x411 or the DSU IDs for the reference car, and 0x283 is sent with a zero payload only; no LionDriver requirements, no field-exposure credit</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   opendbc_repo/opendbc/car/toyota</t>
+          </r>
+        </is>
+      </c>
+      <c r="J84" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="K84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• process_replay over the CI route corpus compares sendcan with the reference commit; a regression check, not designed or proven for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L84" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="M84" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Rationale  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The panda refuses these frames on every frame (SFM-035.C3 is the case where that check fails); no separate action. A compromised SoC sending them on purpose is a TARA topic, out of scope here</t>
+          </r>
+        </is>
+      </c>
+      <c r="O84" s="34" t="inlineStr"/>
+      <c r="P84" s="33" t="inlineStr"/>
+      <c r="Q84" s="33" t="inlineStr"/>
+      <c r="R84" s="37" t="inlineStr"/>
+      <c r="S84" s="37" t="inlineStr"/>
+    </row>
+    <row r="85" ht="100.5" customHeight="1">
+      <c r="A85" s="39" t="n"/>
+      <c r="B85" s="39" t="n"/>
+      <c r="C85" s="39" t="n"/>
+      <c r="D85" s="39" t="n"/>
+      <c r="E85" s="39" t="n"/>
+      <c r="F85" s="39" t="n"/>
+      <c r="G85" s="40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="H85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The TX whitelist or the PRE_COLLISION content check lets a PCS-relevant frame through (table change, or a build that is not the reference build, where 0x411 is allowed by design)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Panda safety code: MISRA C:2012, 100% line coverage, review; reduced whitelist (TSR-705); reference build the default since BL-005 (pandad requires it, TSR-514/619)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   opendbc_repo/opendbc/safety/modes/toyota.h</t>
+          </r>
+        </is>
+      </c>
+      <c r="J85" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• opendbc safety suite with 100% line coverage and mutation tests in both variants, run by CI on every change (proven, early, test-to-fail)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   opendbc_repo/opendbc/safety/tests/test_toyota.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L85" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="M85" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Rationale  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The whitelist is a static table pinned by mutation-proven tests in both variants; the non-reference variant keeps 0x411 by design and cannot configure a car mode with pandad at BL-005. No SW FMEA mode covers the table yet (FTA BE-7.07, for the SW FMEA)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O85" s="41" t="inlineStr"/>
+      <c r="P85" s="40" t="inlineStr"/>
+      <c r="Q85" s="40" t="inlineStr"/>
+      <c r="R85" s="45" t="inlineStr"/>
+      <c r="S85" s="45" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S83"/>
-  <mergeCells count="172">
+  <autoFilter ref="A2:S85"/>
+  <mergeCells count="178">
+    <mergeCell ref="F84:F85"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="E39:E40"/>
     <mergeCell ref="A57:A59"/>
@@ -15754,6 +16132,7 @@
     <mergeCell ref="E6:E9"/>
     <mergeCell ref="B69:B70"/>
     <mergeCell ref="B3:B5"/>
+    <mergeCell ref="B84:B85"/>
     <mergeCell ref="C51:C52"/>
     <mergeCell ref="C60:C61"/>
     <mergeCell ref="C64:C66"/>
@@ -15779,6 +16158,7 @@
     <mergeCell ref="F32:F34"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="E67:E68"/>
+    <mergeCell ref="A84:A85"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="E51:E52"/>
     <mergeCell ref="C17:C19"/>
@@ -15788,6 +16168,8 @@
     <mergeCell ref="A25:A28"/>
     <mergeCell ref="B71:B74"/>
     <mergeCell ref="B82:B83"/>
+    <mergeCell ref="C84:C85"/>
+    <mergeCell ref="E84:E85"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="F51:F52"/>
     <mergeCell ref="C3:C5"/>
@@ -15867,9 +16249,10 @@
     <mergeCell ref="A82:A83"/>
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D84:D85"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15877,7 +16260,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.12 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.13 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.13: SFM-036, the item keeps requesting acceleration during stock PCS (FTA BE-7.13)
The F-17 System FMEA mode for BE-7.13. stockAeb raises only a PERMANENT
alert, so controlsd keeps sending the planner's request while stock PCS
brakes; stock AEB then rests on PCM priority (AOU-04R, unverified).
- C1 design gap, no item reaction: O 8 D 10 AP H; MSR M 8 (alert only)
- C2 PCM does not give PCS priority (AOU-04R): O 3 D 10 AP H; MSR M 10
- SFM-ACT-020 (decision_pending): stand down on a stock PCS event, or
  rely on the AOU-04R test; lead question DQ-300 queued (range 300-319)
Links: fta-fmea-map BE-7.13 -> SFM-036; hara.yaml HZ-011 sfm_refs;
fta-SG-07-1.svg regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$87</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -252,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -389,6 +389,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -880,7 +883,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15">
@@ -890,7 +893,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16">
@@ -900,7 +903,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -931,7 +934,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>18 (17)</t>
+          <t>19 (18)</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S85"/>
+  <dimension ref="A1:S87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16069,9 +16072,342 @@
       <c r="R85" s="45" t="inlineStr"/>
       <c r="S85" s="45" t="inlineStr"/>
     </row>
+    <row r="86" ht="127.5" customHeight="1">
+      <c r="A86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-SE-001
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-FN-008
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>F8 Stock function preservation: keep stock vehicle safety functions not replaced by the item available</t>
+          </r>
+        </is>
+      </c>
+      <c r="C86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock AEB deceleration reduced or delayed if the PCM arbitrates otherwise</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>PCS braking depends on the PCM giving it priority over the item's request (AOU-04R, unverified)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>ACC_CONTROL keeps carrying the planner's acceleration request while the stock camera reports a PCS braking event</t>
+          </r>
+        </is>
+      </c>
+      <c r="D86" s="31" t="inlineStr">
+        <is>
+          <t>HZ-011</t>
+        </is>
+      </c>
+      <c r="E86" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-036 · unintended
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Item keeps requesting acceleration while stock PCS brakes</t>
+          </r>
+        </is>
+      </c>
+      <c r="G86" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The item has no reaction to a stock PCS event on its longitudinal command; controlsd keeps requesting the planner's acceleration (design gap, FTA BE-7.13)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• None in the item: FSR-07.04 places PCS priority in the PCM as an external measure (AOU-04R)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/02-concept/WP-C-04-functional-safety-concept.md</t>
+          </r>
+        </is>
+      </c>
+      <c r="J86" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No pre-release test targets this cause</t>
+          </r>
+        </is>
+      </c>
+      <c r="L86" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="M86" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-020 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
+          </r>
+        </is>
+      </c>
+      <c r="O86" s="58" t="inlineStr">
+        <is>
+          <t>decision pending</t>
+        </is>
+      </c>
+      <c r="P86" s="33" t="inlineStr"/>
+      <c r="Q86" s="33" t="inlineStr"/>
+      <c r="R86" s="37" t="inlineStr"/>
+      <c r="S86" s="37" t="inlineStr"/>
+    </row>
+    <row r="87" ht="100.5" customHeight="1">
+      <c r="A87" s="39" t="n"/>
+      <c r="B87" s="39" t="n"/>
+      <c r="C87" s="39" t="n"/>
+      <c r="D87" s="39" t="n"/>
+      <c r="E87" s="39" t="n"/>
+      <c r="F87" s="39" t="n"/>
+      <c r="G87" s="40" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The PCM does not give stock PCS braking priority over the item's ACC_CONTROL request (AOU-04R not met)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Series-production Toyota ECU; PCS priority over 0x343 assumed (AOU-04R), not verified by LionDriver</t>
+          </r>
+        </is>
+      </c>
+      <c r="J87" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="K87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No pre-release test targets this cause; AOU-04R needs a message review and a PCS target test (WP-C-04)</t>
+          </r>
+        </is>
+      </c>
+      <c r="L87" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="M87" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-006 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Establish on the reference car which stock TSS2 functions (PCS/AEB, FCW) remain available with LionDriver installed and longitudinal control enabled, and verify the stock pre-collision path after installation (PFMEA PFM-014)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O87" s="48" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P87" s="40" t="inlineStr"/>
+      <c r="Q87" s="40" t="inlineStr"/>
+      <c r="R87" s="45" t="inlineStr"/>
+      <c r="S87" s="45" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S85"/>
-  <mergeCells count="178">
+  <autoFilter ref="A2:S87"/>
+  <mergeCells count="184">
     <mergeCell ref="F84:F85"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="E39:E40"/>
@@ -16079,9 +16415,12 @@
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="F25:F28"/>
     <mergeCell ref="A51:A52"/>
+    <mergeCell ref="B86:B87"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="D86:D87"/>
     <mergeCell ref="E23:E24"/>
     <mergeCell ref="F55:F56"/>
+    <mergeCell ref="F86:F87"/>
     <mergeCell ref="C32:C34"/>
     <mergeCell ref="E32:E34"/>
     <mergeCell ref="B23:B24"/>
@@ -16103,6 +16442,7 @@
     <mergeCell ref="C41:C43"/>
     <mergeCell ref="F71:F74"/>
     <mergeCell ref="A10:A13"/>
+    <mergeCell ref="C86:C87"/>
     <mergeCell ref="C44:C46"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="E44:E46"/>
@@ -16176,6 +16516,7 @@
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A64:A66"/>
     <mergeCell ref="A79:A81"/>
+    <mergeCell ref="E86:E87"/>
     <mergeCell ref="B41:B43"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="B10:B13"/>
@@ -16221,6 +16562,7 @@
     <mergeCell ref="B64:B66"/>
     <mergeCell ref="C25:C28"/>
     <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A86:A87"/>
     <mergeCell ref="C55:C56"/>
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="B32:B34"/>
@@ -16252,7 +16594,7 @@
     <mergeCell ref="D84:D85"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16275,7 +16617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16290,79 +16632,79 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="B1" s="58" t="inlineStr">
+      <c r="B1" s="59" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="C1" s="58" t="inlineStr">
+      <c r="C1" s="59" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="58" t="inlineStr">
+      <c r="D1" s="59" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E1" s="58" t="inlineStr">
+      <c r="E1" s="59" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="58" t="inlineStr">
+      <c r="F1" s="59" t="inlineStr">
         <is>
           <t>Causes</t>
         </is>
       </c>
-      <c r="G1" s="58" t="inlineStr">
+      <c r="G1" s="59" t="inlineStr">
         <is>
           <t>Revised S/O/D</t>
         </is>
       </c>
-      <c r="H1" s="58" t="inlineStr">
+      <c r="H1" s="59" t="inlineStr">
         <is>
           <t>Revised AP</t>
         </is>
       </c>
-      <c r="I1" s="58" t="inlineStr">
+      <c r="I1" s="59" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
     </row>
     <row r="2" ht="127.5" customHeight="1">
-      <c r="A2" s="59" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-001</t>
         </is>
       </c>
-      <c r="B2" s="59" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C2" s="59" t="inlineStr">
+      <c r="C2" s="60" t="inlineStr">
         <is>
           <t>Derive steering and acceleration envelopes from measurements on the reference vehicle and set the panda limits from them, independently of the SoC limits (same as SWF-ACT-003, FSC FOI-001)</t>
         </is>
       </c>
-      <c r="D2" s="59" t="inlineStr">
+      <c r="D2" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E2" s="59" t="inlineStr">
+      <c r="E2" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F2" s="59" t="inlineStr">
+      <c r="F2" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
@@ -16375,37 +16717,37 @@
 SFM-029.C2</t>
         </is>
       </c>
-      <c r="G2" s="59" t="inlineStr"/>
-      <c r="H2" s="59" t="inlineStr"/>
-      <c r="I2" s="59" t="inlineStr"/>
+      <c r="G2" s="60" t="inlineStr"/>
+      <c r="H2" s="60" t="inlineStr"/>
+      <c r="I2" s="60" t="inlineStr"/>
     </row>
     <row r="3" ht="127.5" customHeight="1">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-002</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C3" s="59" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
         </is>
       </c>
-      <c r="D3" s="59" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr">
+      <c r="E3" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F3" s="59" t="inlineStr">
+      <c r="F3" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C4
 SFM-004.C3
@@ -16418,37 +16760,37 @@
 SFM-030.C1</t>
         </is>
       </c>
-      <c r="G3" s="59" t="inlineStr"/>
-      <c r="H3" s="59" t="inlineStr"/>
-      <c r="I3" s="59" t="inlineStr"/>
+      <c r="G3" s="60" t="inlineStr"/>
+      <c r="H3" s="60" t="inlineStr"/>
+      <c r="I3" s="60" t="inlineStr"/>
     </row>
     <row r="4" ht="343.5" customHeight="1">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-003</t>
         </is>
       </c>
-      <c r="B4" s="59" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C4" s="59" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
         </is>
       </c>
-      <c r="D4" s="59" t="inlineStr">
+      <c r="D4" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E4" s="59" t="inlineStr">
+      <c r="E4" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F4" s="59" t="inlineStr">
+      <c r="F4" s="60" t="inlineStr">
         <is>
           <t>SFM-003.C1
 SFM-003.C2
@@ -16477,109 +16819,110 @@
 SFM-033.C3</t>
         </is>
       </c>
-      <c r="G4" s="59" t="inlineStr"/>
-      <c r="H4" s="59" t="inlineStr"/>
-      <c r="I4" s="59" t="inlineStr"/>
+      <c r="G4" s="60" t="inlineStr"/>
+      <c r="H4" s="60" t="inlineStr"/>
+      <c r="I4" s="60" t="inlineStr"/>
     </row>
     <row r="5" ht="73.5" customHeight="1">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-005</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C5" s="59" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
         <is>
           <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (ASIL A); the reaction itself is still to be decided</t>
         </is>
       </c>
-      <c r="D5" s="59" t="inlineStr">
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr">
+      <c r="E5" s="60" t="inlineStr">
         <is>
           <t>decision pending</t>
         </is>
       </c>
-      <c r="F5" s="59" t="inlineStr">
+      <c r="F5" s="60" t="inlineStr">
         <is>
           <t>SFM-025.C1</t>
         </is>
       </c>
-      <c r="G5" s="59" t="inlineStr"/>
-      <c r="H5" s="59" t="inlineStr"/>
-      <c r="I5" s="59" t="inlineStr"/>
+      <c r="G5" s="60" t="inlineStr"/>
+      <c r="H5" s="60" t="inlineStr"/>
+      <c r="I5" s="60" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-006</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>Establish on the reference car which stock TSS2 functions (PCS/AEB, FCW) remain available with LionDriver installed and longitudinal control enabled, and verify the stock pre-collision path after installation (PFMEA PFM-014)</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F6" s="59" t="inlineStr">
+      <c r="F6" s="60" t="inlineStr">
         <is>
           <t>SFM-010.C2
 SFM-033.C1
-SFM-033.C2</t>
-        </is>
-      </c>
-      <c r="G6" s="59" t="inlineStr"/>
-      <c r="H6" s="59" t="inlineStr"/>
-      <c r="I6" s="59" t="inlineStr"/>
+SFM-033.C2
+SFM-036.C2</t>
+        </is>
+      </c>
+      <c r="G6" s="60" t="inlineStr"/>
+      <c r="H6" s="60" t="inlineStr"/>
+      <c r="I6" s="60" t="inlineStr"/>
     </row>
     <row r="7" ht="73.5" customHeight="1">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-007</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C7" s="59" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>Supervise the alert channels: treat loss of ui or soundd liveness, or a stale displayed state, as a fault that escalates (audible fallback, disengagement) instead of continuing silently</t>
         </is>
       </c>
-      <c r="D7" s="59" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E7" s="59" t="inlineStr">
+      <c r="E7" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F7" s="59" t="inlineStr">
+      <c r="F7" s="60" t="inlineStr">
         <is>
           <t>SFM-015.C1
 SFM-026.C1
@@ -16588,76 +16931,76 @@
 SFM-028.C1</t>
         </is>
       </c>
-      <c r="G7" s="59" t="inlineStr"/>
-      <c r="H7" s="59" t="inlineStr"/>
-      <c r="I7" s="59" t="inlineStr"/>
+      <c r="G7" s="60" t="inlineStr"/>
+      <c r="H7" s="60" t="inlineStr"/>
+      <c r="I7" s="60" t="inlineStr"/>
     </row>
     <row r="8" ht="73.5" customHeight="1">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-008</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>Allow engagement only when the fingerprint, CarParams and panda safety parameter match the reference configuration AC-001 (refuse fuzzy matches in the reference build); see PFMEA PFM-013</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr">
+      <c r="E8" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F8" s="59" t="inlineStr">
+      <c r="F8" s="60" t="inlineStr">
         <is>
           <t>SFM-032.C1</t>
         </is>
       </c>
-      <c r="G8" s="59" t="inlineStr"/>
-      <c r="H8" s="59" t="inlineStr"/>
-      <c r="I8" s="59" t="inlineStr">
+      <c r="G8" s="60" t="inlineStr"/>
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr">
         <is>
           <t>BL-005: the reference build is the default (LionDriver #36), the panda accepts only TOYOTA parameter 73 (reference_lock.h) and pandad configures a car mode only on a reference panda (#41). Fuzzy fingerprint matches are still accepted on the host (SFM-032.C1)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="100.5" customHeight="1">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-009</t>
         </is>
       </c>
-      <c r="B9" s="59" t="inlineStr">
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t>prevention</t>
         </is>
       </c>
-      <c r="C9" s="59" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>Produce SOTIF / ISO PAS 8800 evidence for the neural-network elements (driving model, lead detection, driver monitoring model) per WP-V-02..04, including fault-induced inputs (corrupted or stale frames)</t>
         </is>
       </c>
-      <c r="D9" s="59" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E9" s="59" t="inlineStr">
+      <c r="E9" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F9" s="59" t="inlineStr">
+      <c r="F9" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C2
 SFM-003.C3
@@ -16668,37 +17011,37 @@
 SFM-022.C2</t>
         </is>
       </c>
-      <c r="G9" s="59" t="inlineStr"/>
-      <c r="H9" s="59" t="inlineStr"/>
-      <c r="I9" s="59" t="inlineStr"/>
+      <c r="G9" s="60" t="inlineStr"/>
+      <c r="H9" s="60" t="inlineStr"/>
+      <c r="I9" s="60" t="inlineStr"/>
     </row>
     <row r="10" ht="73.5" customHeight="1">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-010</t>
         </is>
       </c>
-      <c r="B10" s="59" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C10" s="59" t="inlineStr">
+      <c r="C10" s="60" t="inlineStr">
         <is>
           <t>Justify every SOFT_DISABLE reaction and debounce against the FTTI (WP-S-04) and alert at once when the panda withdraws authority while engaged (controlsMismatch debounce)</t>
         </is>
       </c>
-      <c r="D10" s="59" t="inlineStr">
+      <c r="D10" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E10" s="59" t="inlineStr">
+      <c r="E10" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F10" s="59" t="inlineStr">
+      <c r="F10" s="60" t="inlineStr">
         <is>
           <t>SFM-014.C2
 SFM-015.C2
@@ -16706,286 +17049,317 @@
 SFM-016.C2</t>
         </is>
       </c>
-      <c r="G10" s="59" t="inlineStr"/>
-      <c r="H10" s="59" t="inlineStr"/>
-      <c r="I10" s="59" t="inlineStr">
+      <c r="G10" s="60" t="inlineStr"/>
+      <c r="H10" s="60" t="inlineStr"/>
+      <c r="I10" s="60" t="inlineStr">
         <is>
           <t>controlsMismatch debounce cut from 200 cumulative samples (~2 s) to 2 consecutive samples, at most 0.5 s (change-2026-10-13-host-supervision.md); credited at BL-005 (SFM-015.C2 M 6). FTTI justification of SOFT_DISABLE reactions open</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-011</t>
         </is>
       </c>
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C11" s="59" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
         <is>
           <t>Alert the driver when stock cruise stays engaged while the item is disengaged (cruiseMismatch has no alert at BL-004)</t>
         </is>
       </c>
-      <c r="D11" s="59" t="inlineStr">
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E11" s="60" t="inlineStr">
+      <c r="E11" s="61" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F11" s="59" t="inlineStr">
+      <c r="F11" s="60" t="inlineStr">
         <is>
           <t>SFM-021.C1
 SFM-021.C2</t>
         </is>
       </c>
-      <c r="G11" s="59" t="inlineStr"/>
-      <c r="H11" s="59" t="inlineStr"/>
-      <c r="I11" s="59" t="inlineStr">
+      <c r="G11" s="60" t="inlineStr"/>
+      <c r="H11" s="60" t="inlineStr"/>
+      <c r="I11" s="60" t="inlineStr">
         <is>
           <t>cruiseMismatch now alerts after 1 s (change-2026-10-13-host-supervision.md); see SWF-ACT-034</t>
         </is>
       </c>
     </row>
     <row r="12" ht="73.5" customHeight="1">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-012</t>
         </is>
       </c>
-      <c r="B12" s="59" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C12" s="59" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>Measure on the HIL bench and the reference car (WP-V-05) how the panda reacts to over-limit and not-engaged steering and acceleration frames and to driver brake, gas and cancel inputs, and what the EPS and PCM do when frames are refused; re-rate the MSR rows from code-derived to measured timing</t>
         </is>
       </c>
-      <c r="D12" s="59" t="inlineStr"/>
-      <c r="E12" s="59" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F12" s="59" t="inlineStr"/>
-      <c r="G12" s="59" t="inlineStr"/>
-      <c r="H12" s="59" t="inlineStr"/>
-      <c r="I12" s="59" t="inlineStr"/>
+      <c r="F12" s="60" t="inlineStr"/>
+      <c r="G12" s="60" t="inlineStr"/>
+      <c r="H12" s="60" t="inlineStr"/>
+      <c r="I12" s="60" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-013</t>
         </is>
       </c>
-      <c r="B13" s="59" t="inlineStr">
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C13" s="59" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert</t>
         </is>
       </c>
-      <c r="D13" s="59" t="inlineStr"/>
-      <c r="E13" s="59" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr"/>
+      <c r="E13" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F13" s="59" t="inlineStr"/>
-      <c r="G13" s="59" t="inlineStr"/>
-      <c r="H13" s="59" t="inlineStr"/>
-      <c r="I13" s="59" t="inlineStr"/>
+      <c r="F13" s="60" t="inlineStr"/>
+      <c r="G13" s="60" t="inlineStr"/>
+      <c r="H13" s="60" t="inlineStr"/>
+      <c r="I13" s="60" t="inlineStr"/>
     </row>
     <row r="14" ht="46.5" customHeight="1">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-014</t>
         </is>
       </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C14" s="59" t="inlineStr">
+      <c r="C14" s="60" t="inlineStr">
         <is>
           <t>Specify in the TSC a steering-direction plausibility monitor (commanded torque sign against measured yaw rate and lane-relative lateral motion), or justify its absence against HZ-003</t>
         </is>
       </c>
-      <c r="D14" s="59" t="inlineStr"/>
-      <c r="E14" s="59" t="inlineStr">
+      <c r="D14" s="60" t="inlineStr"/>
+      <c r="E14" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F14" s="59" t="inlineStr"/>
-      <c r="G14" s="59" t="inlineStr"/>
-      <c r="H14" s="59" t="inlineStr"/>
-      <c r="I14" s="59" t="inlineStr"/>
+      <c r="F14" s="60" t="inlineStr"/>
+      <c r="G14" s="60" t="inlineStr"/>
+      <c r="H14" s="60" t="inlineStr"/>
+      <c r="I14" s="60" t="inlineStr"/>
     </row>
     <row r="15" ht="87" customHeight="1">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-015</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>Detect stale commands and inputs within the SG-01 FTTI: command-frame freshness in the MCU with an active zero frame (TSR-408, TSR-109) and frozen-content and age checks on model outputs in controlsd (TSR-602, AIR-17)</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr"/>
-      <c r="E15" s="59" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr"/>
+      <c r="E15" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F15" s="59" t="inlineStr"/>
-      <c r="G15" s="59" t="inlineStr"/>
-      <c r="H15" s="59" t="inlineStr"/>
-      <c r="I15" s="59" t="inlineStr">
+      <c r="F15" s="60" t="inlineStr"/>
+      <c r="G15" s="60" t="inlineStr"/>
+      <c r="H15" s="60" t="inlineStr"/>
+      <c r="I15" s="60" t="inlineStr">
         <is>
           <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="59" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-016</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C16" s="60" t="inlineStr">
         <is>
           <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr"/>
-      <c r="E16" s="59" t="inlineStr">
+      <c r="D16" s="60" t="inlineStr"/>
+      <c r="E16" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F16" s="59" t="inlineStr"/>
-      <c r="G16" s="59" t="inlineStr"/>
-      <c r="H16" s="59" t="inlineStr"/>
-      <c r="I16" s="59" t="inlineStr"/>
+      <c r="F16" s="60" t="inlineStr"/>
+      <c r="G16" s="60" t="inlineStr"/>
+      <c r="H16" s="60" t="inlineStr"/>
+      <c r="I16" s="60" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="59" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-017</t>
         </is>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>Add WP-S-04 FTTI rows for the warning paths without one (insufficient lateral control, late or insufficient braking warnings, SG-008 unintended engagement, driver monitoring), so these mechanisms can be compared with a time budget</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr"/>
-      <c r="E17" s="59" t="inlineStr">
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F17" s="59" t="inlineStr"/>
-      <c r="G17" s="59" t="inlineStr"/>
-      <c r="H17" s="59" t="inlineStr"/>
-      <c r="I17" s="59" t="inlineStr"/>
+      <c r="F17" s="60" t="inlineStr"/>
+      <c r="G17" s="60" t="inlineStr"/>
+      <c r="H17" s="60" t="inlineStr"/>
+      <c r="I17" s="60" t="inlineStr"/>
     </row>
     <row r="18" ht="73.5" customHeight="1">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-018</t>
         </is>
       </c>
-      <c r="B18" s="59" t="inlineStr">
+      <c r="B18" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C18" s="59" t="inlineStr">
+      <c r="C18" s="60" t="inlineStr">
         <is>
           <t>Detect silent loss of the actuation path: report forwarded and refused TX frames from the panda, and compare EPS and PCM acceptance (LKA_STATE, ACC status) with the commands, warning within the SG-02/06 1 s budget</t>
         </is>
       </c>
-      <c r="D18" s="59" t="inlineStr"/>
-      <c r="E18" s="59" t="inlineStr">
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F18" s="59" t="inlineStr"/>
-      <c r="G18" s="59" t="inlineStr"/>
-      <c r="H18" s="59" t="inlineStr"/>
-      <c r="I18" s="59" t="inlineStr">
+      <c r="F18" s="60" t="inlineStr"/>
+      <c r="G18" s="60" t="inlineStr"/>
+      <c r="H18" s="60" t="inlineStr"/>
+      <c r="I18" s="60" t="inlineStr">
         <is>
           <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1; TSR-626)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="59" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-019</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C19" s="59" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
         </is>
       </c>
-      <c r="D19" s="59" t="inlineStr"/>
-      <c r="E19" s="59" t="inlineStr">
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F19" s="59" t="inlineStr">
+      <c r="F19" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
 SFM-002.C4</t>
         </is>
       </c>
-      <c r="G19" s="59" t="inlineStr"/>
-      <c r="H19" s="59" t="inlineStr"/>
-      <c r="I19" s="59" t="inlineStr"/>
+      <c r="G19" s="60" t="inlineStr"/>
+      <c r="H19" s="60" t="inlineStr"/>
+      <c r="I19" s="60" t="inlineStr"/>
+    </row>
+    <row r="20" ht="73.5" customHeight="1">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>SFM-ACT-020</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>design change</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
+        </is>
+      </c>
+      <c r="D20" s="60" t="inlineStr"/>
+      <c r="E20" s="60" t="inlineStr">
+        <is>
+          <t>decision pending</t>
+        </is>
+      </c>
+      <c r="F20" s="60" t="inlineStr">
+        <is>
+          <t>SFM-036.C1</t>
+        </is>
+      </c>
+      <c r="G20" s="60" t="inlineStr"/>
+      <c r="H20" s="60" t="inlineStr"/>
+      <c r="I20" s="60" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:I20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17007,50 +17381,50 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Element</t>
         </is>
       </c>
-      <c r="B1" s="58" t="inlineStr">
+      <c r="B1" s="59" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="58" t="inlineStr">
+      <c r="C1" s="59" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="D1" s="58" t="inlineStr">
+      <c r="D1" s="59" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="E1" s="58" t="inlineStr">
+      <c r="E1" s="59" t="inlineStr">
         <is>
           <t>Functions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="222" customHeight="1">
-      <c r="A2" s="59" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="B2" s="59" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
         </is>
       </c>
-      <c r="C2" s="59" t="inlineStr">
+      <c r="C2" s="60" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D2" s="59" t="inlineStr"/>
-      <c r="E2" s="59" t="inlineStr">
+      <c r="D2" s="60" t="inlineStr"/>
+      <c r="E2" s="60" t="inlineStr">
         <is>
           <t>SFM-FN-001: F1 Lateral control: request steering torque from the EPS to keep the vehicle in its lane while engaged
 SFM-FN-002: F2 Longitudinal control: request acceleration/deceleration to hold set speed and follow leads while engaged
@@ -17064,398 +17438,398 @@
       </c>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">    comma 3X device</t>
         </is>
       </c>
-      <c r="C3" s="59" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="D3" s="59" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr"/>
+      <c r="E3" s="60" t="inlineStr"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-003</t>
         </is>
       </c>
-      <c r="B4" s="59" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Integrated panda (CAN interface and safety model)</t>
         </is>
       </c>
-      <c r="C4" s="59" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>subsystem</t>
         </is>
       </c>
-      <c r="D4" s="59" t="inlineStr">
+      <c r="D4" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E4" s="59" t="inlineStr"/>
+      <c r="E4" s="60" t="inlineStr"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-004</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">    Harness (Toyota A connector, harness box, comma power v3)</t>
         </is>
       </c>
-      <c r="C5" s="59" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
         <is>
           <t>component</t>
         </is>
       </c>
-      <c r="D5" s="59" t="inlineStr">
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr"/>
+      <c r="E5" s="60" t="inlineStr"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-010</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Perception (camerad, modeld)</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-011</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Localization and calibration (locationd, calibrationd, paramsd, torqued)</t>
         </is>
       </c>
-      <c r="C7" s="59" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D7" s="59" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E7" s="59" t="inlineStr"/>
+      <c r="E7" s="60" t="inlineStr"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-012</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Planning (plannerd, radard)</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-013</t>
         </is>
       </c>
-      <c r="B9" s="59" t="inlineStr">
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Control (controlsd, lateral/longitudinal controllers)</t>
         </is>
       </c>
-      <c r="C9" s="59" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D9" s="59" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E9" s="59" t="inlineStr"/>
+      <c r="E9" s="60" t="inlineStr"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-014</t>
         </is>
       </c>
-      <c r="B10" s="59" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Supervision (selfdrived state machine, events, alert manager)</t>
         </is>
       </c>
-      <c r="C10" s="59" t="inlineStr">
+      <c r="C10" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D10" s="59" t="inlineStr">
+      <c r="D10" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E10" s="59" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-015</t>
         </is>
       </c>
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Driver monitoring (dmonitoringmodeld, dmonitoringd)</t>
         </is>
       </c>
-      <c r="C11" s="59" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D11" s="59" t="inlineStr">
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E11" s="59" t="inlineStr"/>
+      <c r="E11" s="60" t="inlineStr"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-016</t>
         </is>
       </c>
-      <c r="B12" s="59" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Car interface (card, car_events, opendbc Toyota port)</t>
         </is>
       </c>
-      <c r="C12" s="59" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D12" s="59" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E12" s="59" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-017</t>
         </is>
       </c>
-      <c r="B13" s="59" t="inlineStr">
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Panda daemon (pandad)</t>
         </is>
       </c>
-      <c r="C13" s="59" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D13" s="59" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E13" s="59" t="inlineStr"/>
+      <c r="E13" s="60" t="inlineStr"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-018</t>
         </is>
       </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        HMI (ui, soundd)</t>
         </is>
       </c>
-      <c r="C14" s="59" t="inlineStr">
+      <c r="C14" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D14" s="59" t="inlineStr">
+      <c r="D14" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E14" s="59" t="inlineStr"/>
+      <c r="E14" s="60" t="inlineStr"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-019</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Platform (manager, messaging, hardwared, OS)</t>
         </is>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E15" s="59" t="inlineStr"/>
+      <c r="E15" s="60" t="inlineStr"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="59" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-030</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>Toyota EPS</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C16" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr"/>
-      <c r="E16" s="59" t="inlineStr"/>
+      <c r="D16" s="60" t="inlineStr"/>
+      <c r="E16" s="60" t="inlineStr"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="59" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-031</t>
         </is>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="60" t="inlineStr">
         <is>
           <t>Toyota powertrain and brake control (receives ACC acceleration requests)</t>
         </is>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr"/>
-      <c r="E17" s="59" t="inlineStr"/>
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="60" t="inlineStr"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-032</t>
         </is>
       </c>
-      <c r="B18" s="59" t="inlineStr">
+      <c r="B18" s="60" t="inlineStr">
         <is>
           <t>Toyota stock ADAS camera (TSS2)</t>
         </is>
       </c>
-      <c r="C18" s="59" t="inlineStr">
+      <c r="C18" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D18" s="59" t="inlineStr"/>
-      <c r="E18" s="59" t="inlineStr"/>
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="60" t="inlineStr"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="59" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-033</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>Vehicle CAN buses and 12 V supply</t>
         </is>
       </c>
-      <c r="C19" s="59" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D19" s="59" t="inlineStr"/>
-      <c r="E19" s="59" t="inlineStr"/>
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="60" t="inlineStr"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="59" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-034</t>
         </is>
       </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="B20" s="60" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C20" s="59" t="inlineStr">
+      <c r="C20" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D20" s="59" t="inlineStr"/>
-      <c r="E20" s="59" t="inlineStr"/>
+      <c r="D20" s="60" t="inlineStr"/>
+      <c r="E20" s="60" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E20"/>

</xml_diff>

<commit_message>
Regenerate the System FMEA review workbook after merging #117 and liondriver-dev
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$83</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
@@ -817,7 +817,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.11 · draft</t>
+          <t>0.12 · draft</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16">
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17">
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S82"/>
+  <dimension ref="A1:S83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2759,7 +2759,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -2868,7 +2868,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3120,7 +3120,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3453,7 +3453,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3589,7 +3589,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -3823,7 +3823,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -4901,7 +4901,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -5459,7 +5459,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -5550,7 +5550,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -6054,7 +6054,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -6522,7 +6522,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -6755,7 +6755,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -7118,7 +7118,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -7591,7 +7591,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -8634,7 +8634,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -9281,7 +9281,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -9645,7 +9645,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -10009,7 +10009,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -10260,7 +10260,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -11079,7 +11079,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -12354,7 +12354,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -12697,7 +12697,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -13161,7 +13161,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -14486,7 +14486,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
           </r>
         </is>
       </c>
@@ -14945,7 +14945,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Stock ADAS camera messages blocked or replaced by the harness relay</t>
+            <t>Stock ADAS camera messages blocked or replaced by the harness-box intercept</t>
           </r>
         </is>
       </c>
@@ -14993,7 +14993,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Relay intercepts stock camera messages the vehicle needs for AEB</t>
+            <t>The intercept routes the stock camera messages the vehicle needs for AEB through the panda</t>
           </r>
         </is>
       </c>
@@ -15005,7 +15005,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Forwarding keeps stock pre-collision messages (0x283, 0x344) passing the relay (SWF-011); which TSS2 functions remain with openpilot longitudinal is not established</t>
+            <t>• Forwarding keeps stock pre-collision messages (0x283, 0x344) passing the intercept (SWF-011); which TSS2 functions remain with openpilot longitudinal is not established</t>
           </r>
           <r>
             <rPr>
@@ -15074,18 +15074,18 @@
       <c r="S79" s="37" t="inlineStr"/>
     </row>
     <row r="80" ht="100.5" customHeight="1">
-      <c r="A80" s="39" t="n"/>
-      <c r="B80" s="39" t="n"/>
-      <c r="C80" s="39" t="n"/>
-      <c r="D80" s="39" t="n"/>
-      <c r="E80" s="39" t="n"/>
-      <c r="F80" s="39" t="n"/>
-      <c r="G80" s="40" t="inlineStr">
+      <c r="A80" s="38" t="n"/>
+      <c r="B80" s="38" t="n"/>
+      <c r="C80" s="38" t="n"/>
+      <c r="D80" s="38" t="n"/>
+      <c r="E80" s="38" t="n"/>
+      <c r="F80" s="38" t="n"/>
+      <c r="G80" s="33" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="H80" s="41" t="inlineStr">
+      <c r="H80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15106,7 +15106,7 @@
           </r>
         </is>
       </c>
-      <c r="I80" s="41" t="inlineStr">
+      <c r="I80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15127,10 +15127,10 @@
           </r>
         </is>
       </c>
-      <c r="J80" s="42" t="n">
+      <c r="J80" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="K80" s="41" t="inlineStr">
+      <c r="K80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15151,15 +15151,15 @@
           </r>
         </is>
       </c>
-      <c r="L80" s="42" t="n">
+      <c r="L80" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="M80" s="44" t="inlineStr">
+      <c r="M80" s="36" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="N80" s="41" t="inlineStr">
+      <c r="N80" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15181,18 +15181,103 @@
           </r>
         </is>
       </c>
-      <c r="O80" s="48" t="inlineStr">
+      <c r="O80" s="47" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="P80" s="40" t="inlineStr"/>
-      <c r="Q80" s="40" t="inlineStr"/>
-      <c r="R80" s="45" t="inlineStr"/>
-      <c r="S80" s="45" t="inlineStr"/>
-    </row>
-    <row r="81" ht="87" customHeight="1">
-      <c r="A81" s="30" t="inlineStr">
+      <c r="P80" s="33" t="inlineStr"/>
+      <c r="Q80" s="33" t="inlineStr"/>
+      <c r="R80" s="37" t="inlineStr"/>
+      <c r="S80" s="37" t="inlineStr"/>
+    </row>
+    <row r="81" ht="141" customHeight="1">
+      <c r="A81" s="39" t="n"/>
+      <c r="B81" s="39" t="n"/>
+      <c r="C81" s="39" t="n"/>
+      <c r="D81" s="39" t="n"/>
+      <c r="E81" s="39" t="n"/>
+      <c r="F81" s="39" t="n"/>
+      <c r="G81" s="40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="H81" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The harness box loses its supply (ignition branch or D1 open without comma power, VIN shorted), or a switch channel opens, so the stock camera path through the unpowered or open DG419LE switches is cut (RR-2026-010)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: DFM-020</t>
+          </r>
+        </is>
+      </c>
+      <c r="I81" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Consumer-grade harness box without automotive qualification data available to LionDriver; rated in the DFMEA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/08-analyses/fmea/analyses/dfmea.yaml</t>
+          </r>
+        </is>
+      </c>
+      <c r="J81" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K81" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the DFMEA: no pre-release test of this hardware fault</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/08-analyses/fmea/analyses/dfmea.yaml</t>
+          </r>
+        </is>
+      </c>
+      <c r="L81" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="M81" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N81" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15201,6 +15286,39 @@
               <color rgb="001F4E8C"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">SFM-ACT-003 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+          </r>
+        </is>
+      </c>
+      <c r="O81" s="48" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P81" s="40" t="inlineStr"/>
+      <c r="Q81" s="40" t="inlineStr"/>
+      <c r="R81" s="45" t="inlineStr"/>
+      <c r="S81" s="45" t="inlineStr"/>
+    </row>
+    <row r="82" ht="87" customHeight="1">
+      <c r="A82" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">SFM-SE-001
 </t>
           </r>
@@ -15214,7 +15332,7 @@
           </r>
         </is>
       </c>
-      <c r="B81" s="30" t="inlineStr">
+      <c r="B82" s="30" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15236,7 +15354,7 @@
           </r>
         </is>
       </c>
-      <c r="C81" s="30" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15357,21 +15475,21 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Relay stuck or intermittent; stock camera and item both on bus, or neither</t>
-          </r>
-        </is>
-      </c>
-      <c r="D81" s="31" t="inlineStr">
+            <t>Intercept switch stuck or intermittent: in intercept when released (camera cut off from the car), or in pass-through when driven (stock camera and item both on the bus)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D82" s="31" t="inlineStr">
         <is>
           <t>HZ-011
 HZ-002
 HZ-006</t>
         </is>
       </c>
-      <c r="E81" s="32" t="n">
+      <c r="E82" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="F81" s="30" t="inlineStr">
+      <c r="F82" s="30" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15390,24 +15508,24 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Harness relay fault</t>
-          </r>
-        </is>
-      </c>
-      <c r="G81" s="33" t="inlineStr">
+            <t>Harness-box intercept switch stuck or in the wrong position</t>
+          </r>
+        </is>
+      </c>
+      <c r="G82" s="33" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="H81" s="34" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Relay contact wear or connector fault</t>
+      <c r="H82" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
           </r>
           <r>
             <rPr>
@@ -15420,7 +15538,7 @@
           </r>
         </is>
       </c>
-      <c r="I81" s="34" t="inlineStr">
+      <c r="I82" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15441,10 +15559,10 @@
           </r>
         </is>
       </c>
-      <c r="J81" s="35" t="n">
-        <v>3</v>
-      </c>
-      <c r="K81" s="34" t="inlineStr">
+      <c r="J82" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="K82" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15465,15 +15583,15 @@
           </r>
         </is>
       </c>
-      <c r="L81" s="46" t="n">
+      <c r="L82" s="46" t="n">
         <v>10</v>
       </c>
-      <c r="M81" s="36" t="inlineStr">
+      <c r="M82" s="36" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="N81" s="34" t="inlineStr">
+      <c r="N82" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15490,37 +15608,37 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Hardware fault rated in the DFMEA (DFM-010 O3 D10, DFM-011 O3 D9); this row inherits that rating; relayMalfunction (SWF-012) is the in-field mechanism</t>
-          </r>
-        </is>
-      </c>
-      <c r="O81" s="34" t="inlineStr"/>
-      <c r="P81" s="33" t="inlineStr"/>
-      <c r="Q81" s="33" t="inlineStr"/>
-      <c r="R81" s="37" t="inlineStr"/>
-      <c r="S81" s="37" t="inlineStr"/>
-    </row>
-    <row r="82" ht="87" customHeight="1">
-      <c r="A82" s="39" t="n"/>
-      <c r="B82" s="39" t="n"/>
-      <c r="C82" s="39" t="n"/>
-      <c r="D82" s="39" t="n"/>
-      <c r="E82" s="39" t="n"/>
-      <c r="F82" s="39" t="n"/>
-      <c r="G82" s="40" t="inlineStr">
+            <t>Hardware fault rated in the DFMEA (DFM-010.C1-C3 O3 D10, DFM-010.C4 O4 D10); this row inherits the worst. relayMalfunction (SWF-012) is the in-field mechanism; there is no switch-state feedback (RR-2026-010)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O82" s="34" t="inlineStr"/>
+      <c r="P82" s="33" t="inlineStr"/>
+      <c r="Q82" s="33" t="inlineStr"/>
+      <c r="R82" s="37" t="inlineStr"/>
+      <c r="S82" s="37" t="inlineStr"/>
+    </row>
+    <row r="83" ht="102" customHeight="1">
+      <c r="A83" s="39" t="n"/>
+      <c r="B83" s="39" t="n"/>
+      <c r="C83" s="39" t="n"/>
+      <c r="D83" s="39" t="n"/>
+      <c r="E83" s="39" t="n"/>
+      <c r="F83" s="39" t="n"/>
+      <c r="G83" s="40" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="H82" s="41" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Relay drive output fault on panda</t>
+      <c r="H83" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
           </r>
           <r>
             <rPr>
@@ -15533,7 +15651,7 @@
           </r>
         </is>
       </c>
-      <c r="I82" s="41" t="inlineStr">
+      <c r="I83" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15554,10 +15672,10 @@
           </r>
         </is>
       </c>
-      <c r="J82" s="42" t="n">
+      <c r="J83" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="K82" s="41" t="inlineStr">
+      <c r="K83" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15578,15 +15696,15 @@
           </r>
         </is>
       </c>
-      <c r="L82" s="43" t="n">
-        <v>10</v>
-      </c>
-      <c r="M82" s="44" t="inlineStr">
+      <c r="L83" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="M83" s="44" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="N82" s="41" t="inlineStr">
+      <c r="N83" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -15603,24 +15721,22 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Hardware fault rated in the DFMEA (DFM-011, DFM-010); this row inherits that rating</t>
-          </r>
-        </is>
-      </c>
-      <c r="O82" s="41" t="inlineStr"/>
-      <c r="P82" s="40" t="inlineStr"/>
-      <c r="Q82" s="40" t="inlineStr"/>
-      <c r="R82" s="45" t="inlineStr"/>
-      <c r="S82" s="45" t="inlineStr"/>
+            <t>Hardware fault rated in the DFMEA (DFM-011.C1 O3 D9, DFM-011.C2 O2 D9); this row inherits the worst</t>
+          </r>
+        </is>
+      </c>
+      <c r="O83" s="41" t="inlineStr"/>
+      <c r="P83" s="40" t="inlineStr"/>
+      <c r="Q83" s="40" t="inlineStr"/>
+      <c r="R83" s="45" t="inlineStr"/>
+      <c r="S83" s="45" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:S82"/>
+  <autoFilter ref="A2:S83"/>
   <mergeCells count="172">
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="E39:E40"/>
-    <mergeCell ref="C79:C80"/>
     <mergeCell ref="A57:A59"/>
-    <mergeCell ref="E79:E80"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="F25:F28"/>
     <mergeCell ref="A51:A52"/>
@@ -15630,7 +15746,6 @@
     <mergeCell ref="C32:C34"/>
     <mergeCell ref="E32:E34"/>
     <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F79:F80"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="D20:D22"/>
     <mergeCell ref="E3:E5"/>
@@ -15639,7 +15754,6 @@
     <mergeCell ref="F29:F31"/>
     <mergeCell ref="F47:F48"/>
     <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F81:F82"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="B37:B38"/>
     <mergeCell ref="C71:C74"/>
@@ -15655,6 +15769,7 @@
     <mergeCell ref="E44:E46"/>
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="C69:C70"/>
+    <mergeCell ref="F79:F81"/>
     <mergeCell ref="D57:D59"/>
     <mergeCell ref="N1:Q1"/>
     <mergeCell ref="D41:D43"/>
@@ -15663,7 +15778,6 @@
     <mergeCell ref="B35:B36"/>
     <mergeCell ref="F10:F13"/>
     <mergeCell ref="D49:D50"/>
-    <mergeCell ref="A79:A80"/>
     <mergeCell ref="E55:E56"/>
     <mergeCell ref="A32:A34"/>
     <mergeCell ref="A14:A16"/>
@@ -15687,37 +15801,38 @@
     <mergeCell ref="D37:D38"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="B55:B56"/>
+    <mergeCell ref="C82:C83"/>
     <mergeCell ref="D55:D56"/>
+    <mergeCell ref="C79:C81"/>
     <mergeCell ref="I1:M1"/>
+    <mergeCell ref="E79:E81"/>
     <mergeCell ref="D39:D40"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="D79:D80"/>
-    <mergeCell ref="E81:E82"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="B29:B31"/>
     <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B81:B82"/>
     <mergeCell ref="D32:D34"/>
     <mergeCell ref="C49:C50"/>
-    <mergeCell ref="D81:D82"/>
     <mergeCell ref="F32:F34"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="E67:E68"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="E51:E52"/>
     <mergeCell ref="C17:C19"/>
+    <mergeCell ref="E82:E83"/>
     <mergeCell ref="E60:E61"/>
     <mergeCell ref="E69:E70"/>
     <mergeCell ref="A25:A28"/>
     <mergeCell ref="B71:B74"/>
+    <mergeCell ref="B82:B83"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="F51:F52"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A64:A66"/>
+    <mergeCell ref="A79:A81"/>
     <mergeCell ref="B41:B43"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="B10:B13"/>
@@ -15764,20 +15879,22 @@
     <mergeCell ref="C25:C28"/>
     <mergeCell ref="A55:A56"/>
     <mergeCell ref="C55:C56"/>
+    <mergeCell ref="B79:B81"/>
     <mergeCell ref="B32:B34"/>
+    <mergeCell ref="D79:D81"/>
     <mergeCell ref="C67:C68"/>
     <mergeCell ref="E17:E19"/>
     <mergeCell ref="D71:D74"/>
     <mergeCell ref="E75:E76"/>
     <mergeCell ref="A47:A48"/>
-    <mergeCell ref="A81:A82"/>
     <mergeCell ref="D17:D19"/>
-    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="F82:F83"/>
     <mergeCell ref="D67:D68"/>
     <mergeCell ref="F67:F68"/>
     <mergeCell ref="B51:B52"/>
     <mergeCell ref="E47:E48"/>
     <mergeCell ref="D51:D52"/>
+    <mergeCell ref="D82:D83"/>
     <mergeCell ref="D60:D61"/>
     <mergeCell ref="F60:F61"/>
     <mergeCell ref="C37:C38"/>
@@ -15786,11 +15903,12 @@
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="F69:F70"/>
     <mergeCell ref="B25:B28"/>
+    <mergeCell ref="A82:A83"/>
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="C6:C9"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15798,7 +15916,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.11 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.12 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -15960,7 +16078,7 @@
       <c r="H3" s="59" t="inlineStr"/>
       <c r="I3" s="59" t="inlineStr"/>
     </row>
-    <row r="4" ht="330" customHeight="1">
+    <row r="4" ht="343.5" customHeight="1">
       <c r="A4" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-003</t>
@@ -15973,7 +16091,7 @@
       </c>
       <c r="C4" s="59" t="inlineStr">
         <is>
-          <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, relay and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
+          <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
         </is>
       </c>
       <c r="D4" s="59" t="inlineStr">
@@ -16011,7 +16129,8 @@
 SFM-026.C2
 SFM-027.C1
 SFM-028.C2
-SFM-031.C1</t>
+SFM-031.C1
+SFM-033.C3</t>
         </is>
       </c>
       <c r="G4" s="59" t="inlineStr"/>
@@ -21019,10 +21138,10 @@
       <c r="O64" s="37" t="inlineStr"/>
       <c r="P64" s="37" t="inlineStr"/>
     </row>
-    <row r="65" ht="33" customHeight="1">
+    <row r="65" ht="73.5" customHeight="1">
       <c r="A65" s="34" t="inlineStr">
         <is>
-          <t>SFM-034 · Harness relay fault</t>
+          <t>SFM-034 · Harness-box intercept switch stuck or in the wrong position</t>
         </is>
       </c>
       <c r="B65" s="35" t="n">
@@ -21035,7 +21154,7 @@
       </c>
       <c r="D65" s="34" t="inlineStr">
         <is>
-          <t>Relay contact wear or connector fault</t>
+          <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
         </is>
       </c>
       <c r="E65" s="62" t="inlineStr">
@@ -21055,10 +21174,10 @@
       <c r="O65" s="37" t="inlineStr"/>
       <c r="P65" s="37" t="inlineStr"/>
     </row>
-    <row r="66" ht="33" customHeight="1">
+    <row r="66" ht="60" customHeight="1">
       <c r="A66" s="34" t="inlineStr">
         <is>
-          <t>SFM-034 · Harness relay fault</t>
+          <t>SFM-034 · Harness-box intercept switch stuck or in the wrong position</t>
         </is>
       </c>
       <c r="B66" s="35" t="n">
@@ -21071,7 +21190,7 @@
       </c>
       <c r="D66" s="34" t="inlineStr">
         <is>
-          <t>Relay drive output fault on panda</t>
+          <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
         </is>
       </c>
       <c r="E66" s="62" t="inlineStr">
@@ -21105,7 +21224,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.11 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.12 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Regenerate the System FMEA review workbook after merging #123 and liondriver-dev
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$87</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$70</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -261,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -398,6 +398,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -817,7 +820,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.12 · draft</t>
+          <t>0.13 · draft</t>
         </is>
       </c>
     </row>
@@ -895,7 +898,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15">
@@ -905,7 +908,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16">
@@ -915,7 +918,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -946,7 +949,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>18 (17)</t>
+          <t>19 (18)</t>
         </is>
       </c>
     </row>
@@ -958,7 +961,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>60 rated, 4 exempt; MSR AP H 60, M 0, L 0 (provisional table)</t>
+          <t>64 rated, 4 exempt; MSR AP H 64, M 0, L 0 (provisional table)</t>
         </is>
       </c>
     </row>
@@ -970,7 +973,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>1–4: 0 · 5–6: 15 · 7–8: 16 · 9–10: 29 (see sheet MSR)</t>
+          <t>1–4: 0 · 5–6: 16 · 7–8: 17 · 9–10: 31 (see sheet MSR)</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S83"/>
+  <dimension ref="A1:S87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15731,18 +15734,732 @@
       <c r="R83" s="45" t="inlineStr"/>
       <c r="S83" s="45" t="inlineStr"/>
     </row>
+    <row r="84" ht="100.5" customHeight="1">
+      <c r="A84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-SE-001
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-FN-008
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>F8 Stock function preservation: keep stock vehicle safety functions not replaced by the item available</t>
+          </r>
+        </is>
+      </c>
+      <c r="C84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock AEB/FCW degraded while the driver relies on it</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-006: PCS braking triggered by a frame from the item</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock PCS warning or braking suppressed, altered or triggered by the item</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>A PCS-relevant frame from the SoC (0x344 PRE_COLLISION_2, 0x411 PCS_HUD, a DSU-only ID, or 0x283 PRE_COLLISION with a non-zero payload) reaches the car bus</t>
+          </r>
+        </is>
+      </c>
+      <c r="D84" s="31" t="inlineStr">
+        <is>
+          <t>HZ-011
+HZ-006</t>
+        </is>
+      </c>
+      <c r="E84" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F84" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-035 · unintended
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Item sends a frame that alters the stock pre-collision function</t>
+          </r>
+        </is>
+      </c>
+      <c r="G84" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Host code (car interface, pandad) emits a PCS-relevant ID or a non-zero PRE_COLLISION payload (QM fault)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream opendbc Toyota port; no carcontroller path builds 0x344, 0x411 or the DSU IDs for the reference car, and 0x283 is sent with a zero payload only; no LionDriver requirements, no field-exposure credit</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   opendbc_repo/opendbc/car/toyota</t>
+          </r>
+        </is>
+      </c>
+      <c r="J84" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="K84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• process_replay over the CI route corpus compares sendcan with the reference commit; a regression check, not designed or proven for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L84" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="M84" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N84" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Rationale  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The panda refuses these frames on every frame (SFM-035.C3 is the case where that check fails); no separate action. A compromised SoC sending them on purpose is a TARA topic, out of scope here</t>
+          </r>
+        </is>
+      </c>
+      <c r="O84" s="34" t="inlineStr"/>
+      <c r="P84" s="33" t="inlineStr"/>
+      <c r="Q84" s="33" t="inlineStr"/>
+      <c r="R84" s="37" t="inlineStr"/>
+      <c r="S84" s="37" t="inlineStr"/>
+    </row>
+    <row r="85" ht="100.5" customHeight="1">
+      <c r="A85" s="39" t="n"/>
+      <c r="B85" s="39" t="n"/>
+      <c r="C85" s="39" t="n"/>
+      <c r="D85" s="39" t="n"/>
+      <c r="E85" s="39" t="n"/>
+      <c r="F85" s="39" t="n"/>
+      <c r="G85" s="40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="H85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The TX whitelist or the PRE_COLLISION content check lets a PCS-relevant frame through (table change, or a build that is not the reference build, where 0x411 is allowed by design)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Panda safety code: MISRA C:2012, 100% line coverage, review; reduced whitelist (TSR-705); reference build the default since BL-005 (pandad requires it, TSR-514/619)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   opendbc_repo/opendbc/safety/modes/toyota.h</t>
+          </r>
+        </is>
+      </c>
+      <c r="J85" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• opendbc safety suite with 100% line coverage and mutation tests in both variants, run by CI on every change (proven, early, test-to-fail)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   opendbc_repo/opendbc/safety/tests/test_toyota.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L85" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="M85" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N85" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Rationale  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The whitelist is a static table pinned by mutation-proven tests in both variants; the non-reference variant keeps 0x411 by design and cannot configure a car mode with pandad at BL-005. No SW FMEA mode covers the table yet (FTA BE-7.07, for the SW FMEA)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O85" s="41" t="inlineStr"/>
+      <c r="P85" s="40" t="inlineStr"/>
+      <c r="Q85" s="40" t="inlineStr"/>
+      <c r="R85" s="45" t="inlineStr"/>
+      <c r="S85" s="45" t="inlineStr"/>
+    </row>
+    <row r="86" ht="127.5" customHeight="1">
+      <c r="A86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-SE-001
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-FN-008
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>F8 Stock function preservation: keep stock vehicle safety functions not replaced by the item available</t>
+          </r>
+        </is>
+      </c>
+      <c r="C86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock AEB deceleration reduced or delayed if the PCM arbitrates otherwise</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>PCS braking depends on the PCM giving it priority over the item's request (AOU-04R, unverified)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>ACC_CONTROL keeps carrying the planner's acceleration request while the stock camera reports a PCS braking event</t>
+          </r>
+        </is>
+      </c>
+      <c r="D86" s="31" t="inlineStr">
+        <is>
+          <t>HZ-011</t>
+        </is>
+      </c>
+      <c r="E86" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F86" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-036 · unintended
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Item keeps requesting acceleration while stock PCS brakes</t>
+          </r>
+        </is>
+      </c>
+      <c r="G86" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The item has no reaction to a stock PCS event on its longitudinal command; controlsd keeps requesting the planner's acceleration (design gap, FTA BE-7.13)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• None in the item: FSR-07.04 places PCS priority in the PCM as an external measure (AOU-04R)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/02-concept/WP-C-04-functional-safety-concept.md</t>
+          </r>
+        </is>
+      </c>
+      <c r="J86" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No pre-release test targets this cause</t>
+          </r>
+        </is>
+      </c>
+      <c r="L86" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="M86" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N86" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-020 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
+          </r>
+        </is>
+      </c>
+      <c r="O86" s="58" t="inlineStr">
+        <is>
+          <t>decision pending</t>
+        </is>
+      </c>
+      <c r="P86" s="33" t="inlineStr"/>
+      <c r="Q86" s="33" t="inlineStr"/>
+      <c r="R86" s="37" t="inlineStr"/>
+      <c r="S86" s="37" t="inlineStr"/>
+    </row>
+    <row r="87" ht="100.5" customHeight="1">
+      <c r="A87" s="39" t="n"/>
+      <c r="B87" s="39" t="n"/>
+      <c r="C87" s="39" t="n"/>
+      <c r="D87" s="39" t="n"/>
+      <c r="E87" s="39" t="n"/>
+      <c r="F87" s="39" t="n"/>
+      <c r="G87" s="40" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The PCM does not give stock PCS braking priority over the item's ACC_CONTROL request (AOU-04R not met)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Series-production Toyota ECU; PCS priority over 0x343 assumed (AOU-04R), not verified by LionDriver</t>
+          </r>
+        </is>
+      </c>
+      <c r="J87" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="K87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No pre-release test targets this cause; AOU-04R needs a message review and a PCS target test (WP-C-04)</t>
+          </r>
+        </is>
+      </c>
+      <c r="L87" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="M87" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N87" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-006 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Establish on the reference car which stock TSS2 functions (PCS/AEB, FCW) remain available with LionDriver installed and longitudinal control enabled, and verify the stock pre-collision path after installation (PFMEA PFM-014)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O87" s="48" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P87" s="40" t="inlineStr"/>
+      <c r="Q87" s="40" t="inlineStr"/>
+      <c r="R87" s="45" t="inlineStr"/>
+      <c r="S87" s="45" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S83"/>
-  <mergeCells count="172">
+  <autoFilter ref="A2:S87"/>
+  <mergeCells count="184">
+    <mergeCell ref="F84:F85"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="E39:E40"/>
     <mergeCell ref="A57:A59"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="F25:F28"/>
     <mergeCell ref="A51:A52"/>
+    <mergeCell ref="B86:B87"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="D86:D87"/>
     <mergeCell ref="E23:E24"/>
     <mergeCell ref="F55:F56"/>
+    <mergeCell ref="F86:F87"/>
     <mergeCell ref="C32:C34"/>
     <mergeCell ref="E32:E34"/>
     <mergeCell ref="B23:B24"/>
@@ -15764,6 +16481,7 @@
     <mergeCell ref="C41:C43"/>
     <mergeCell ref="F71:F74"/>
     <mergeCell ref="A10:A13"/>
+    <mergeCell ref="C86:C87"/>
     <mergeCell ref="C44:C46"/>
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="E44:E46"/>
@@ -15793,6 +16511,7 @@
     <mergeCell ref="E6:E9"/>
     <mergeCell ref="B69:B70"/>
     <mergeCell ref="B3:B5"/>
+    <mergeCell ref="B84:B85"/>
     <mergeCell ref="C51:C52"/>
     <mergeCell ref="C60:C61"/>
     <mergeCell ref="C64:C66"/>
@@ -15818,6 +16537,7 @@
     <mergeCell ref="F32:F34"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="E67:E68"/>
+    <mergeCell ref="A84:A85"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="E51:E52"/>
     <mergeCell ref="C17:C19"/>
@@ -15827,12 +16547,15 @@
     <mergeCell ref="A25:A28"/>
     <mergeCell ref="B71:B74"/>
     <mergeCell ref="B82:B83"/>
+    <mergeCell ref="C84:C85"/>
+    <mergeCell ref="E84:E85"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="F51:F52"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A64:A66"/>
     <mergeCell ref="A79:A81"/>
+    <mergeCell ref="E86:E87"/>
     <mergeCell ref="B41:B43"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="B10:B13"/>
@@ -15878,6 +16601,7 @@
     <mergeCell ref="B64:B66"/>
     <mergeCell ref="C25:C28"/>
     <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A86:A87"/>
     <mergeCell ref="C55:C56"/>
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="B32:B34"/>
@@ -15906,9 +16630,10 @@
     <mergeCell ref="A82:A83"/>
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D84:D85"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15916,7 +16641,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.12 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.13 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -15931,7 +16656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15946,79 +16671,79 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="B1" s="58" t="inlineStr">
+      <c r="B1" s="59" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="C1" s="58" t="inlineStr">
+      <c r="C1" s="59" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="58" t="inlineStr">
+      <c r="D1" s="59" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E1" s="58" t="inlineStr">
+      <c r="E1" s="59" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="58" t="inlineStr">
+      <c r="F1" s="59" t="inlineStr">
         <is>
           <t>Causes</t>
         </is>
       </c>
-      <c r="G1" s="58" t="inlineStr">
+      <c r="G1" s="59" t="inlineStr">
         <is>
           <t>Revised S/O/D</t>
         </is>
       </c>
-      <c r="H1" s="58" t="inlineStr">
+      <c r="H1" s="59" t="inlineStr">
         <is>
           <t>Revised AP</t>
         </is>
       </c>
-      <c r="I1" s="58" t="inlineStr">
+      <c r="I1" s="59" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
     </row>
     <row r="2" ht="127.5" customHeight="1">
-      <c r="A2" s="59" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-001</t>
         </is>
       </c>
-      <c r="B2" s="59" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C2" s="59" t="inlineStr">
+      <c r="C2" s="60" t="inlineStr">
         <is>
           <t>Derive steering and acceleration envelopes from measurements on the reference vehicle and set the panda limits from them, independently of the SoC limits (same as SWF-ACT-003, FSC FOI-001)</t>
         </is>
       </c>
-      <c r="D2" s="59" t="inlineStr">
+      <c r="D2" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E2" s="59" t="inlineStr">
+      <c r="E2" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F2" s="59" t="inlineStr">
+      <c r="F2" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
@@ -16031,37 +16756,37 @@
 SFM-029.C2</t>
         </is>
       </c>
-      <c r="G2" s="59" t="inlineStr"/>
-      <c r="H2" s="59" t="inlineStr"/>
-      <c r="I2" s="59" t="inlineStr"/>
+      <c r="G2" s="60" t="inlineStr"/>
+      <c r="H2" s="60" t="inlineStr"/>
+      <c r="I2" s="60" t="inlineStr"/>
     </row>
     <row r="3" ht="127.5" customHeight="1">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-002</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C3" s="59" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
         </is>
       </c>
-      <c r="D3" s="59" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr">
+      <c r="E3" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F3" s="59" t="inlineStr">
+      <c r="F3" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C4
 SFM-004.C3
@@ -16074,37 +16799,37 @@
 SFM-030.C1</t>
         </is>
       </c>
-      <c r="G3" s="59" t="inlineStr"/>
-      <c r="H3" s="59" t="inlineStr"/>
-      <c r="I3" s="59" t="inlineStr"/>
+      <c r="G3" s="60" t="inlineStr"/>
+      <c r="H3" s="60" t="inlineStr"/>
+      <c r="I3" s="60" t="inlineStr"/>
     </row>
     <row r="4" ht="343.5" customHeight="1">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-003</t>
         </is>
       </c>
-      <c r="B4" s="59" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C4" s="59" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
         </is>
       </c>
-      <c r="D4" s="59" t="inlineStr">
+      <c r="D4" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E4" s="59" t="inlineStr">
+      <c r="E4" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F4" s="59" t="inlineStr">
+      <c r="F4" s="60" t="inlineStr">
         <is>
           <t>SFM-003.C1
 SFM-003.C2
@@ -16133,109 +16858,110 @@
 SFM-033.C3</t>
         </is>
       </c>
-      <c r="G4" s="59" t="inlineStr"/>
-      <c r="H4" s="59" t="inlineStr"/>
-      <c r="I4" s="59" t="inlineStr"/>
+      <c r="G4" s="60" t="inlineStr"/>
+      <c r="H4" s="60" t="inlineStr"/>
+      <c r="I4" s="60" t="inlineStr"/>
     </row>
     <row r="5" ht="73.5" customHeight="1">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-005</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C5" s="59" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
         <is>
           <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (ASIL A); the reaction itself is still to be decided</t>
         </is>
       </c>
-      <c r="D5" s="59" t="inlineStr">
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr">
+      <c r="E5" s="60" t="inlineStr">
         <is>
           <t>decision pending</t>
         </is>
       </c>
-      <c r="F5" s="59" t="inlineStr">
+      <c r="F5" s="60" t="inlineStr">
         <is>
           <t>SFM-025.C1</t>
         </is>
       </c>
-      <c r="G5" s="59" t="inlineStr"/>
-      <c r="H5" s="59" t="inlineStr"/>
-      <c r="I5" s="59" t="inlineStr"/>
+      <c r="G5" s="60" t="inlineStr"/>
+      <c r="H5" s="60" t="inlineStr"/>
+      <c r="I5" s="60" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-006</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>Establish on the reference car which stock TSS2 functions (PCS/AEB, FCW) remain available with LionDriver installed and longitudinal control enabled, and verify the stock pre-collision path after installation (PFMEA PFM-014)</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F6" s="59" t="inlineStr">
+      <c r="F6" s="60" t="inlineStr">
         <is>
           <t>SFM-010.C2
 SFM-033.C1
-SFM-033.C2</t>
-        </is>
-      </c>
-      <c r="G6" s="59" t="inlineStr"/>
-      <c r="H6" s="59" t="inlineStr"/>
-      <c r="I6" s="59" t="inlineStr"/>
+SFM-033.C2
+SFM-036.C2</t>
+        </is>
+      </c>
+      <c r="G6" s="60" t="inlineStr"/>
+      <c r="H6" s="60" t="inlineStr"/>
+      <c r="I6" s="60" t="inlineStr"/>
     </row>
     <row r="7" ht="73.5" customHeight="1">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-007</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C7" s="59" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>Supervise the alert channels: treat loss of ui or soundd liveness, or a stale displayed state, as a fault that escalates (audible fallback, disengagement) instead of continuing silently</t>
         </is>
       </c>
-      <c r="D7" s="59" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E7" s="59" t="inlineStr">
+      <c r="E7" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F7" s="59" t="inlineStr">
+      <c r="F7" s="60" t="inlineStr">
         <is>
           <t>SFM-015.C1
 SFM-026.C1
@@ -16244,76 +16970,76 @@
 SFM-028.C1</t>
         </is>
       </c>
-      <c r="G7" s="59" t="inlineStr"/>
-      <c r="H7" s="59" t="inlineStr"/>
-      <c r="I7" s="59" t="inlineStr"/>
+      <c r="G7" s="60" t="inlineStr"/>
+      <c r="H7" s="60" t="inlineStr"/>
+      <c r="I7" s="60" t="inlineStr"/>
     </row>
     <row r="8" ht="73.5" customHeight="1">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-008</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>Allow engagement only when the fingerprint, CarParams and panda safety parameter match the reference configuration AC-001 (refuse fuzzy matches in the reference build); see PFMEA PFM-013</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr">
+      <c r="E8" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F8" s="59" t="inlineStr">
+      <c r="F8" s="60" t="inlineStr">
         <is>
           <t>SFM-032.C1</t>
         </is>
       </c>
-      <c r="G8" s="59" t="inlineStr"/>
-      <c r="H8" s="59" t="inlineStr"/>
-      <c r="I8" s="59" t="inlineStr">
+      <c r="G8" s="60" t="inlineStr"/>
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr">
         <is>
           <t>BL-005: the reference build is the default (LionDriver #36), the panda accepts only TOYOTA parameter 73 (reference_lock.h) and pandad configures a car mode only on a reference panda (#41). Fuzzy fingerprint matches are still accepted on the host (SFM-032.C1)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="100.5" customHeight="1">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-009</t>
         </is>
       </c>
-      <c r="B9" s="59" t="inlineStr">
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t>prevention</t>
         </is>
       </c>
-      <c r="C9" s="59" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>Produce SOTIF / ISO PAS 8800 evidence for the neural-network elements (driving model, lead detection, driver monitoring model) per WP-V-02..04, including fault-induced inputs (corrupted or stale frames)</t>
         </is>
       </c>
-      <c r="D9" s="59" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E9" s="59" t="inlineStr">
+      <c r="E9" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F9" s="59" t="inlineStr">
+      <c r="F9" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C2
 SFM-003.C3
@@ -16324,37 +17050,37 @@
 SFM-022.C2</t>
         </is>
       </c>
-      <c r="G9" s="59" t="inlineStr"/>
-      <c r="H9" s="59" t="inlineStr"/>
-      <c r="I9" s="59" t="inlineStr"/>
+      <c r="G9" s="60" t="inlineStr"/>
+      <c r="H9" s="60" t="inlineStr"/>
+      <c r="I9" s="60" t="inlineStr"/>
     </row>
     <row r="10" ht="73.5" customHeight="1">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-010</t>
         </is>
       </c>
-      <c r="B10" s="59" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C10" s="59" t="inlineStr">
+      <c r="C10" s="60" t="inlineStr">
         <is>
           <t>Justify every SOFT_DISABLE reaction and debounce against the FTTI (WP-S-04) and alert at once when the panda withdraws authority while engaged (controlsMismatch debounce)</t>
         </is>
       </c>
-      <c r="D10" s="59" t="inlineStr">
+      <c r="D10" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E10" s="59" t="inlineStr">
+      <c r="E10" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F10" s="59" t="inlineStr">
+      <c r="F10" s="60" t="inlineStr">
         <is>
           <t>SFM-014.C2
 SFM-015.C2
@@ -16362,286 +17088,317 @@
 SFM-016.C2</t>
         </is>
       </c>
-      <c r="G10" s="59" t="inlineStr"/>
-      <c r="H10" s="59" t="inlineStr"/>
-      <c r="I10" s="59" t="inlineStr">
+      <c r="G10" s="60" t="inlineStr"/>
+      <c r="H10" s="60" t="inlineStr"/>
+      <c r="I10" s="60" t="inlineStr">
         <is>
           <t>controlsMismatch debounce cut from 200 cumulative samples (~2 s) to 2 consecutive samples, at most 0.5 s (change-2026-10-13-host-supervision.md); credited at BL-005 (SFM-015.C2 M 6). FTTI justification of SOFT_DISABLE reactions open</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-011</t>
         </is>
       </c>
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C11" s="59" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
         <is>
           <t>Alert the driver when stock cruise stays engaged while the item is disengaged (cruiseMismatch has no alert at BL-004)</t>
         </is>
       </c>
-      <c r="D11" s="59" t="inlineStr">
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E11" s="60" t="inlineStr">
+      <c r="E11" s="61" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F11" s="59" t="inlineStr">
+      <c r="F11" s="60" t="inlineStr">
         <is>
           <t>SFM-021.C1
 SFM-021.C2</t>
         </is>
       </c>
-      <c r="G11" s="59" t="inlineStr"/>
-      <c r="H11" s="59" t="inlineStr"/>
-      <c r="I11" s="59" t="inlineStr">
+      <c r="G11" s="60" t="inlineStr"/>
+      <c r="H11" s="60" t="inlineStr"/>
+      <c r="I11" s="60" t="inlineStr">
         <is>
           <t>cruiseMismatch now alerts after 1 s (change-2026-10-13-host-supervision.md); see SWF-ACT-034</t>
         </is>
       </c>
     </row>
     <row r="12" ht="73.5" customHeight="1">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-012</t>
         </is>
       </c>
-      <c r="B12" s="59" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C12" s="59" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>Measure on the HIL bench and the reference car (WP-V-05) how the panda reacts to over-limit and not-engaged steering and acceleration frames and to driver brake, gas and cancel inputs, and what the EPS and PCM do when frames are refused; re-rate the MSR rows from code-derived to measured timing</t>
         </is>
       </c>
-      <c r="D12" s="59" t="inlineStr"/>
-      <c r="E12" s="59" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F12" s="59" t="inlineStr"/>
-      <c r="G12" s="59" t="inlineStr"/>
-      <c r="H12" s="59" t="inlineStr"/>
-      <c r="I12" s="59" t="inlineStr"/>
+      <c r="F12" s="60" t="inlineStr"/>
+      <c r="G12" s="60" t="inlineStr"/>
+      <c r="H12" s="60" t="inlineStr"/>
+      <c r="I12" s="60" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-013</t>
         </is>
       </c>
-      <c r="B13" s="59" t="inlineStr">
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C13" s="59" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert</t>
         </is>
       </c>
-      <c r="D13" s="59" t="inlineStr"/>
-      <c r="E13" s="59" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr"/>
+      <c r="E13" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F13" s="59" t="inlineStr"/>
-      <c r="G13" s="59" t="inlineStr"/>
-      <c r="H13" s="59" t="inlineStr"/>
-      <c r="I13" s="59" t="inlineStr"/>
+      <c r="F13" s="60" t="inlineStr"/>
+      <c r="G13" s="60" t="inlineStr"/>
+      <c r="H13" s="60" t="inlineStr"/>
+      <c r="I13" s="60" t="inlineStr"/>
     </row>
     <row r="14" ht="46.5" customHeight="1">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-014</t>
         </is>
       </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C14" s="59" t="inlineStr">
+      <c r="C14" s="60" t="inlineStr">
         <is>
           <t>Specify in the TSC a steering-direction plausibility monitor (commanded torque sign against measured yaw rate and lane-relative lateral motion), or justify its absence against HZ-003</t>
         </is>
       </c>
-      <c r="D14" s="59" t="inlineStr"/>
-      <c r="E14" s="59" t="inlineStr">
+      <c r="D14" s="60" t="inlineStr"/>
+      <c r="E14" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F14" s="59" t="inlineStr"/>
-      <c r="G14" s="59" t="inlineStr"/>
-      <c r="H14" s="59" t="inlineStr"/>
-      <c r="I14" s="59" t="inlineStr"/>
+      <c r="F14" s="60" t="inlineStr"/>
+      <c r="G14" s="60" t="inlineStr"/>
+      <c r="H14" s="60" t="inlineStr"/>
+      <c r="I14" s="60" t="inlineStr"/>
     </row>
     <row r="15" ht="87" customHeight="1">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-015</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>Detect stale commands and inputs within the SG-01 FTTI: command-frame freshness in the MCU with an active zero frame (TSR-408, TSR-109) and frozen-content and age checks on model outputs in controlsd (TSR-602, AIR-17)</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr"/>
-      <c r="E15" s="59" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr"/>
+      <c r="E15" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F15" s="59" t="inlineStr"/>
-      <c r="G15" s="59" t="inlineStr"/>
-      <c r="H15" s="59" t="inlineStr"/>
-      <c r="I15" s="59" t="inlineStr">
+      <c r="F15" s="60" t="inlineStr"/>
+      <c r="G15" s="60" t="inlineStr"/>
+      <c r="H15" s="60" t="inlineStr"/>
+      <c r="I15" s="60" t="inlineStr">
         <is>
           <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="59" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-016</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C16" s="60" t="inlineStr">
         <is>
           <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr"/>
-      <c r="E16" s="59" t="inlineStr">
+      <c r="D16" s="60" t="inlineStr"/>
+      <c r="E16" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F16" s="59" t="inlineStr"/>
-      <c r="G16" s="59" t="inlineStr"/>
-      <c r="H16" s="59" t="inlineStr"/>
-      <c r="I16" s="59" t="inlineStr"/>
+      <c r="F16" s="60" t="inlineStr"/>
+      <c r="G16" s="60" t="inlineStr"/>
+      <c r="H16" s="60" t="inlineStr"/>
+      <c r="I16" s="60" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="59" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-017</t>
         </is>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>Add WP-S-04 FTTI rows for the warning paths without one (insufficient lateral control, late or insufficient braking warnings, SG-008 unintended engagement, driver monitoring), so these mechanisms can be compared with a time budget</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr"/>
-      <c r="E17" s="59" t="inlineStr">
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F17" s="59" t="inlineStr"/>
-      <c r="G17" s="59" t="inlineStr"/>
-      <c r="H17" s="59" t="inlineStr"/>
-      <c r="I17" s="59" t="inlineStr"/>
+      <c r="F17" s="60" t="inlineStr"/>
+      <c r="G17" s="60" t="inlineStr"/>
+      <c r="H17" s="60" t="inlineStr"/>
+      <c r="I17" s="60" t="inlineStr"/>
     </row>
     <row r="18" ht="73.5" customHeight="1">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-018</t>
         </is>
       </c>
-      <c r="B18" s="59" t="inlineStr">
+      <c r="B18" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C18" s="59" t="inlineStr">
+      <c r="C18" s="60" t="inlineStr">
         <is>
           <t>Detect silent loss of the actuation path: report forwarded and refused TX frames from the panda, and compare EPS and PCM acceptance (LKA_STATE, ACC status) with the commands, warning within the SG-02/06 1 s budget</t>
         </is>
       </c>
-      <c r="D18" s="59" t="inlineStr"/>
-      <c r="E18" s="59" t="inlineStr">
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F18" s="59" t="inlineStr"/>
-      <c r="G18" s="59" t="inlineStr"/>
-      <c r="H18" s="59" t="inlineStr"/>
-      <c r="I18" s="59" t="inlineStr">
+      <c r="F18" s="60" t="inlineStr"/>
+      <c r="G18" s="60" t="inlineStr"/>
+      <c r="H18" s="60" t="inlineStr"/>
+      <c r="I18" s="60" t="inlineStr">
         <is>
           <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1; TSR-626)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="59" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-019</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C19" s="59" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
         </is>
       </c>
-      <c r="D19" s="59" t="inlineStr"/>
-      <c r="E19" s="59" t="inlineStr">
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F19" s="59" t="inlineStr">
+      <c r="F19" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
 SFM-002.C4</t>
         </is>
       </c>
-      <c r="G19" s="59" t="inlineStr"/>
-      <c r="H19" s="59" t="inlineStr"/>
-      <c r="I19" s="59" t="inlineStr"/>
+      <c r="G19" s="60" t="inlineStr"/>
+      <c r="H19" s="60" t="inlineStr"/>
+      <c r="I19" s="60" t="inlineStr"/>
+    </row>
+    <row r="20" ht="73.5" customHeight="1">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>SFM-ACT-020</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>design change</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
+        </is>
+      </c>
+      <c r="D20" s="60" t="inlineStr"/>
+      <c r="E20" s="60" t="inlineStr">
+        <is>
+          <t>decision pending</t>
+        </is>
+      </c>
+      <c r="F20" s="60" t="inlineStr">
+        <is>
+          <t>SFM-036.C1</t>
+        </is>
+      </c>
+      <c r="G20" s="60" t="inlineStr"/>
+      <c r="H20" s="60" t="inlineStr"/>
+      <c r="I20" s="60" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:I20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16663,50 +17420,50 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Element</t>
         </is>
       </c>
-      <c r="B1" s="58" t="inlineStr">
+      <c r="B1" s="59" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="58" t="inlineStr">
+      <c r="C1" s="59" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="D1" s="58" t="inlineStr">
+      <c r="D1" s="59" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="E1" s="58" t="inlineStr">
+      <c r="E1" s="59" t="inlineStr">
         <is>
           <t>Functions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="222" customHeight="1">
-      <c r="A2" s="59" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="B2" s="59" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
         </is>
       </c>
-      <c r="C2" s="59" t="inlineStr">
+      <c r="C2" s="60" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D2" s="59" t="inlineStr"/>
-      <c r="E2" s="59" t="inlineStr">
+      <c r="D2" s="60" t="inlineStr"/>
+      <c r="E2" s="60" t="inlineStr">
         <is>
           <t>SFM-FN-001: F1 Lateral control: request steering torque from the EPS to keep the vehicle in its lane while engaged
 SFM-FN-002: F2 Longitudinal control: request acceleration/deceleration to hold set speed and follow leads while engaged
@@ -16720,398 +17477,398 @@
       </c>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">    comma 3X device</t>
         </is>
       </c>
-      <c r="C3" s="59" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="D3" s="59" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E3" s="59" t="inlineStr"/>
+      <c r="E3" s="60" t="inlineStr"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-003</t>
         </is>
       </c>
-      <c r="B4" s="59" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Integrated panda (CAN interface and safety model)</t>
         </is>
       </c>
-      <c r="C4" s="59" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>subsystem</t>
         </is>
       </c>
-      <c r="D4" s="59" t="inlineStr">
+      <c r="D4" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E4" s="59" t="inlineStr"/>
+      <c r="E4" s="60" t="inlineStr"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-004</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">    Harness (Toyota A connector, harness box, comma power v3)</t>
         </is>
       </c>
-      <c r="C5" s="59" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
         <is>
           <t>component</t>
         </is>
       </c>
-      <c r="D5" s="59" t="inlineStr">
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr"/>
+      <c r="E5" s="60" t="inlineStr"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-010</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Perception (camerad, modeld)</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-011</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Localization and calibration (locationd, calibrationd, paramsd, torqued)</t>
         </is>
       </c>
-      <c r="C7" s="59" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D7" s="59" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E7" s="59" t="inlineStr"/>
+      <c r="E7" s="60" t="inlineStr"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-012</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Planning (plannerd, radard)</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-013</t>
         </is>
       </c>
-      <c r="B9" s="59" t="inlineStr">
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Control (controlsd, lateral/longitudinal controllers)</t>
         </is>
       </c>
-      <c r="C9" s="59" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D9" s="59" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E9" s="59" t="inlineStr"/>
+      <c r="E9" s="60" t="inlineStr"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-014</t>
         </is>
       </c>
-      <c r="B10" s="59" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Supervision (selfdrived state machine, events, alert manager)</t>
         </is>
       </c>
-      <c r="C10" s="59" t="inlineStr">
+      <c r="C10" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D10" s="59" t="inlineStr">
+      <c r="D10" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E10" s="59" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-015</t>
         </is>
       </c>
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Driver monitoring (dmonitoringmodeld, dmonitoringd)</t>
         </is>
       </c>
-      <c r="C11" s="59" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D11" s="59" t="inlineStr">
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E11" s="59" t="inlineStr"/>
+      <c r="E11" s="60" t="inlineStr"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-016</t>
         </is>
       </c>
-      <c r="B12" s="59" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Car interface (card, car_events, opendbc Toyota port)</t>
         </is>
       </c>
-      <c r="C12" s="59" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D12" s="59" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E12" s="59" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-017</t>
         </is>
       </c>
-      <c r="B13" s="59" t="inlineStr">
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Panda daemon (pandad)</t>
         </is>
       </c>
-      <c r="C13" s="59" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D13" s="59" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E13" s="59" t="inlineStr"/>
+      <c r="E13" s="60" t="inlineStr"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-018</t>
         </is>
       </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        HMI (ui, soundd)</t>
         </is>
       </c>
-      <c r="C14" s="59" t="inlineStr">
+      <c r="C14" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D14" s="59" t="inlineStr">
+      <c r="D14" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E14" s="59" t="inlineStr"/>
+      <c r="E14" s="60" t="inlineStr"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-019</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Platform (manager, messaging, hardwared, OS)</t>
         </is>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E15" s="59" t="inlineStr"/>
+      <c r="E15" s="60" t="inlineStr"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="59" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-030</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>Toyota EPS</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C16" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr"/>
-      <c r="E16" s="59" t="inlineStr"/>
+      <c r="D16" s="60" t="inlineStr"/>
+      <c r="E16" s="60" t="inlineStr"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="59" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-031</t>
         </is>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="60" t="inlineStr">
         <is>
           <t>Toyota powertrain and brake control (receives ACC acceleration requests)</t>
         </is>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr"/>
-      <c r="E17" s="59" t="inlineStr"/>
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="60" t="inlineStr"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-032</t>
         </is>
       </c>
-      <c r="B18" s="59" t="inlineStr">
+      <c r="B18" s="60" t="inlineStr">
         <is>
           <t>Toyota stock ADAS camera (TSS2)</t>
         </is>
       </c>
-      <c r="C18" s="59" t="inlineStr">
+      <c r="C18" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D18" s="59" t="inlineStr"/>
-      <c r="E18" s="59" t="inlineStr"/>
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="60" t="inlineStr"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="59" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-033</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>Vehicle CAN buses and 12 V supply</t>
         </is>
       </c>
-      <c r="C19" s="59" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D19" s="59" t="inlineStr"/>
-      <c r="E19" s="59" t="inlineStr"/>
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="60" t="inlineStr"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="59" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-034</t>
         </is>
       </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="B20" s="60" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C20" s="59" t="inlineStr">
+      <c r="C20" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D20" s="59" t="inlineStr"/>
-      <c r="E20" s="59" t="inlineStr"/>
+      <c r="D20" s="60" t="inlineStr"/>
+      <c r="E20" s="60" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E20"/>
@@ -17125,7 +17882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P66"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -17147,7 +17904,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>FMEA-MSR (monitoring and system response, msr-plan.md): S, F, M and MSR AP per rating-tables.md §7 (RT-2). The MSR AP table is provisional until the handbook table is transcribed (decision register DQ-207). Exempt causes are rated in the FMEA named in the reason.</t>
         </is>
@@ -19875,7 +20632,7 @@
           <t>Device power loss (12 V interruption, harness connector)</t>
         </is>
       </c>
-      <c r="E44" s="62" t="inlineStr">
+      <c r="E44" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-012.C1)</t>
         </is>
@@ -20997,7 +21754,7 @@
           <t>Panda MCU hardware fault (see DFMEA/FMEDA)</t>
         </is>
       </c>
-      <c r="E62" s="62" t="inlineStr">
+      <c r="E62" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-001.C1)</t>
         </is>
@@ -21157,7 +21914,7 @@
           <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
         </is>
       </c>
-      <c r="E65" s="62" t="inlineStr">
+      <c r="E65" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-010.C1)</t>
         </is>
@@ -21193,7 +21950,7 @@
           <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
         </is>
       </c>
-      <c r="E66" s="62" t="inlineStr">
+      <c r="E66" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-011.C1)</t>
         </is>
@@ -21210,13 +21967,258 @@
       <c r="O66" s="37" t="inlineStr"/>
       <c r="P66" s="37" t="inlineStr"/>
     </row>
+    <row r="67" ht="73.5" customHeight="1">
+      <c r="A67" s="34" t="inlineStr">
+        <is>
+          <t>SFM-035 · Item sends a frame that alters the stock pre-collision function</t>
+        </is>
+      </c>
+      <c r="B67" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C67" s="33" t="inlineStr">
+        <is>
+          <t>SFM-035.C1</t>
+        </is>
+      </c>
+      <c r="D67" s="34" t="inlineStr">
+        <is>
+          <t>Host code (car interface, pandad) emits a PCS-relevant ID or a non-zero PRE_COLLISION payload (QM fault)</t>
+        </is>
+      </c>
+      <c r="E67" s="34" t="inlineStr">
+        <is>
+          <t>The panda checks every frame from the SoC against the TX whitelist and the 0x283 zero-payload rule before it is sent</t>
+        </is>
+      </c>
+      <c r="F67" s="34" t="inlineStr">
+        <is>
+          <t>Frame refused, the stock PCS path is untouched; while engaged the refusal also gives pandaTxBlocked, an immediate disable with a take-over alert</t>
+        </is>
+      </c>
+      <c r="G67" s="34" t="inlineStr">
+        <is>
+          <t>Stock PCS unaffected. While engaged the item disengages with an alert (controlled handback, S 8), the worst effect left after the response</t>
+        </is>
+      </c>
+      <c r="H67" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="I67" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="J67" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="K67" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L67" s="34" t="inlineStr">
+        <is>
+          <t>SG-07 content (TX gate, block list) · per frame
+0 + 10 ms</t>
+        </is>
+      </c>
+      <c r="M67" s="33" t="inlineStr">
+        <is>
+          <t>code derived</t>
+        </is>
+      </c>
+      <c r="N67" s="34" t="inlineStr"/>
+      <c r="O67" s="37" t="inlineStr"/>
+      <c r="P67" s="37" t="inlineStr"/>
+    </row>
+    <row r="68" ht="73.5" customHeight="1">
+      <c r="A68" s="34" t="inlineStr">
+        <is>
+          <t>SFM-035 · Item sends a frame that alters the stock pre-collision function</t>
+        </is>
+      </c>
+      <c r="B68" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C68" s="33" t="inlineStr">
+        <is>
+          <t>SFM-035.C3</t>
+        </is>
+      </c>
+      <c r="D68" s="34" t="inlineStr">
+        <is>
+          <t>The TX whitelist or the PRE_COLLISION content check lets a PCS-relevant frame through (table change, or a build that is not the reference build, where 0x411 is allowed by design)</t>
+        </is>
+      </c>
+      <c r="E68" s="34" t="inlineStr">
+        <is>
+          <t>None: the gate is itself the monitor that has failed; pandaTxBlocked counts only refused frames</t>
+        </is>
+      </c>
+      <c r="F68" s="34" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G68" s="34" t="inlineStr">
+        <is>
+          <t>Unchanged: the frame reaches the car while the SoC sends it</t>
+        </is>
+      </c>
+      <c r="H68" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I68" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="J68" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K68" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L68" s="34" t="inlineStr"/>
+      <c r="M68" s="33" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N68" s="34" t="inlineStr"/>
+      <c r="O68" s="37" t="inlineStr"/>
+      <c r="P68" s="37" t="inlineStr"/>
+    </row>
+    <row r="69" ht="73.5" customHeight="1">
+      <c r="A69" s="34" t="inlineStr">
+        <is>
+          <t>SFM-036 · Item keeps requesting acceleration while stock PCS brakes</t>
+        </is>
+      </c>
+      <c r="B69" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C69" s="33" t="inlineStr">
+        <is>
+          <t>SFM-036.C1</t>
+        </is>
+      </c>
+      <c r="D69" s="34" t="inlineStr">
+        <is>
+          <t>The item has no reaction to a stock PCS event on its longitudinal command; controlsd keeps requesting the planner's acceleration (design gap, FTA BE-7.13)</t>
+        </is>
+      </c>
+      <c r="E69" s="34" t="inlineStr">
+        <is>
+          <t>stockAeb detects the PCS event from the stock camera's PRE_COLLISION frame and raises an alert</t>
+        </is>
+      </c>
+      <c r="F69" s="34" t="inlineStr">
+        <is>
+          <t>Alert only; the longitudinal request continues until the driver brakes (panda revokes on the brake press)</t>
+        </is>
+      </c>
+      <c r="G69" s="34" t="inlineStr">
+        <is>
+          <t>Unchanged unless the PCM gives PCS priority (AOU-04R): the item may still oppose stock braking</t>
+        </is>
+      </c>
+      <c r="H69" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I69" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="J69" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K69" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L69" s="34" t="inlineStr"/>
+      <c r="M69" s="33" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N69" s="34" t="inlineStr">
+        <is>
+          <t>SFM-ACT-020 · decision pending</t>
+        </is>
+      </c>
+      <c r="O69" s="37" t="inlineStr"/>
+      <c r="P69" s="37" t="inlineStr"/>
+    </row>
+    <row r="70" ht="46.5" customHeight="1">
+      <c r="A70" s="34" t="inlineStr">
+        <is>
+          <t>SFM-036 · Item keeps requesting acceleration while stock PCS brakes</t>
+        </is>
+      </c>
+      <c r="B70" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C70" s="33" t="inlineStr">
+        <is>
+          <t>SFM-036.C2</t>
+        </is>
+      </c>
+      <c r="D70" s="34" t="inlineStr">
+        <is>
+          <t>The PCM does not give stock PCS braking priority over the item's ACC_CONTROL request (AOU-04R not met)</t>
+        </is>
+      </c>
+      <c r="E70" s="34" t="inlineStr">
+        <is>
+          <t>None: the item cannot see how the PCM arbitrates</t>
+        </is>
+      </c>
+      <c r="F70" s="34" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G70" s="34" t="inlineStr">
+        <is>
+          <t>Unchanged: stock braking reduced while the item requests acceleration</t>
+        </is>
+      </c>
+      <c r="H70" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I70" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="J70" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K70" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L70" s="34" t="inlineStr"/>
+      <c r="M70" s="33" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N70" s="34" t="inlineStr">
+        <is>
+          <t>SFM-ACT-020 · decision pending</t>
+        </is>
+      </c>
+      <c r="O70" s="37" t="inlineStr"/>
+      <c r="P70" s="37" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:P66"/>
+  <autoFilter ref="A2:P70"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
+    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O67 O68 O69 O70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -21224,7 +22226,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.12 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.13 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.14: take in WP-C-03 v0.4 (H-09/SG-08, highway-only ODD)
- Scope: driven inside the ODD, limited-access highways only (DQ-023)
- SFM-025 and SFM-ACT-005 cite H-09 and SG-08 (ASIL A); hara-mapping
  already maps HZ-013 -> H-09 and SG-010 -> SG-08
- SFM-013 note: engagement outside the ODD is foreseeable misuse
  (HARA, WP-C-08), not a fault cause
No rating changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -820,7 +820,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.13 · draft</t>
+          <t>0.14 · draft</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="105" customHeight="1">
+    <row r="10" ht="120" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Scope</t>
@@ -868,7 +868,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>LionDriver as installed on the reference configuration CFG-001 (Corolla E210 · ZRE212 · US, US sedan MY2020-2022) with comma 3X and integrated panda, software BL-005 (structure and failure analysis written at BL-001, risk analysis at BL-004, MSR re-rated at BL-005), while the vehicle is driven on public roads by a licensed driver. Functions F1-F7 per fmea-plan.md section 3.1, plus F8 (stock vehicle safety functions are preserved), added because the harness intercepts the stock ADAS camera.</t>
+          <t>LionDriver as installed on the reference configuration CFG-001 (Corolla E210 · ZRE212 · US, US sedan MY2020-2022) with comma 3X and integrated panda, software BL-005 (structure and failure analysis written at BL-001, risk analysis at BL-004, MSR re-rated at BL-005), while the vehicle is driven by a licensed driver inside the ODD: limited-access highways only since WP-C-02 / WP-C-03 v0.4 (DQ-023). Functions F1-F7 per fmea-plan.md section 3.1, plus F8 (stock vehicle safety functions are preserved), added because the harness intercepts the stock ADAS camera.</t>
         </is>
       </c>
     </row>
@@ -11689,7 +11689,7 @@
       <c r="R62" s="45" t="inlineStr"/>
       <c r="S62" s="45" t="inlineStr"/>
     </row>
-    <row r="63" ht="114" customHeight="1">
+    <row r="63" ht="127.5" customHeight="1">
       <c r="A63" s="51" t="inlineStr">
         <is>
           <r>
@@ -11926,7 +11926,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (ASIL A); the reaction itself is still to be decided</t>
+            <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided</t>
           </r>
         </is>
       </c>
@@ -16641,7 +16641,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.13 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.14 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -16875,7 +16875,7 @@
       </c>
       <c r="C5" s="60" t="inlineStr">
         <is>
-          <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (ASIL A); the reaction itself is still to be decided</t>
+          <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided</t>
         </is>
       </c>
       <c r="D5" s="60" t="inlineStr">
@@ -22226,7 +22226,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.13 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.14 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.15: link monitoring actions to their TSRs; compare warning paths with WP-S-04 §3.8
Takes in WP-S-02 v0.22 §12.3a and WP-S-04 v0.7 §3.7/§3.8 (#105).

- SFM-ACT-005/013/015/016/018 cite TSR-630..633, 626(d)/(e), 628, 615.
  SFM-ACT-017 completed.
- SFM-004.C1-C3: M 7 -> 8. steerSaturated (0.4 s) is late for a
  credible 0.5-1.0 m/s² deficit. New SFM-ACT-021.
- SFM-012.C1: M 7 -> 8. Lag detection plus soft disable exceeds the
  1.6 s FCW budget. New SFM-ACT-022.
- SFM-010.C2/C3: FTTI row cited; M 7 kept (FCW onset not derived).
- SFM-013.C1/C2: M 7 -> 5. Panda engage-edge gate, per frame,
  mutation-tested, within the 0.5 s budget.
- msr-plan v0.8 §4.7, fmea-plan v0.12. S, O, D, AP unchanged.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$87</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$70</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
@@ -820,7 +820,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.14 · draft</t>
+          <t>0.15 · draft</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>19 (18)</t>
+          <t>21 (19)</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>1–4: 0 · 5–6: 16 · 7–8: 17 · 9–10: 31 (see sheet MSR)</t>
+          <t>1–4: 0 · 5–6: 18 · 7–8: 15 · 9–10: 31 (see sheet MSR)</t>
         </is>
       </c>
     </row>
@@ -11689,7 +11689,7 @@
       <c r="R62" s="45" t="inlineStr"/>
       <c r="S62" s="45" t="inlineStr"/>
     </row>
-    <row r="63" ht="127.5" customHeight="1">
+    <row r="63" ht="195" customHeight="1">
       <c r="A63" s="51" t="inlineStr">
         <is>
           <r>
@@ -11926,7 +11926,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided</t>
+            <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided. The requirement is TSR-633 (terminal reaction, ASIL A proposed) with TSR-611 (WP-S-02 §12.3a); the reaction is lead decision DQ-340. The H-09 FTTI is not yet set, so the timing rows of WP-S-04 §3.8.4 cannot be compared</t>
           </r>
         </is>
       </c>
@@ -16641,7 +16641,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.14 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.15 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -16656,7 +16656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16862,7 +16862,7 @@
       <c r="H4" s="60" t="inlineStr"/>
       <c r="I4" s="60" t="inlineStr"/>
     </row>
-    <row r="5" ht="73.5" customHeight="1">
+    <row r="5" ht="114" customHeight="1">
       <c r="A5" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-005</t>
@@ -16875,7 +16875,7 @@
       </c>
       <c r="C5" s="60" t="inlineStr">
         <is>
-          <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided</t>
+          <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided. The requirement is TSR-633 (terminal reaction, ASIL A proposed) with TSR-611 (WP-S-02 §12.3a); the reaction is lead decision DQ-340. The H-09 FTTI is not yet set, so the timing rows of WP-S-04 §3.8.4 cannot be compared</t>
         </is>
       </c>
       <c r="D5" s="60" t="inlineStr">
@@ -17163,7 +17163,7 @@
       <c r="H12" s="60" t="inlineStr"/>
       <c r="I12" s="60" t="inlineStr"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="87" customHeight="1">
       <c r="A13" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-013</t>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="C13" s="60" t="inlineStr">
         <is>
-          <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert</t>
+          <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert. The requirement is TSR-630, within 0.3 s (WP-S-02 §12.3a; WP-S-04 T-32, not implemented)</t>
         </is>
       </c>
       <c r="D13" s="60" t="inlineStr"/>
@@ -17217,7 +17217,7 @@
       <c r="H14" s="60" t="inlineStr"/>
       <c r="I14" s="60" t="inlineStr"/>
     </row>
-    <row r="15" ht="87" customHeight="1">
+    <row r="15" ht="100.5" customHeight="1">
       <c r="A15" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-015</t>
@@ -17230,7 +17230,7 @@
       </c>
       <c r="C15" s="60" t="inlineStr">
         <is>
-          <t>Detect stale commands and inputs within the SG-01 FTTI: command-frame freshness in the MCU with an active zero frame (TSR-408, TSR-109) and frozen-content and age checks on model outputs in controlsd (TSR-602, AIR-17)</t>
+          <t>Detect stale commands and inputs within the SG-01 FTTI: command-frame freshness in the MCU with an active zero frame (TSR-408, TSR-109) and frozen-content and age checks on model outputs in controlsd (TSR-602, TSR-631, AIR-17)</t>
         </is>
       </c>
       <c r="D15" s="60" t="inlineStr"/>
@@ -17244,11 +17244,11 @@
       <c r="H15" s="60" t="inlineStr"/>
       <c r="I15" s="60" t="inlineStr">
         <is>
-          <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+          <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3). The frozen-content check is TSR-631, with the age taken from the source timestamp (WP-S-02 §12.3a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="73.5" customHeight="1">
       <c r="A16" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-016</t>
@@ -17261,7 +17261,7 @@
       </c>
       <c r="C16" s="60" t="inlineStr">
         <is>
-          <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue</t>
+          <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue. Requirements: TSR-304 (timing tied to the SG-05 budget) and TSR-628 (WP-S-02 §12.3a)</t>
         </is>
       </c>
       <c r="D16" s="60" t="inlineStr"/>
@@ -17275,7 +17275,7 @@
       <c r="H16" s="60" t="inlineStr"/>
       <c r="I16" s="60" t="inlineStr"/>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="87" customHeight="1">
       <c r="A17" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-017</t>
@@ -17292,17 +17292,21 @@
         </is>
       </c>
       <c r="D17" s="60" t="inlineStr"/>
-      <c r="E17" s="60" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="E17" s="61" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="F17" s="60" t="inlineStr"/>
       <c r="G17" s="60" t="inlineStr"/>
       <c r="H17" s="60" t="inlineStr"/>
-      <c r="I17" s="60" t="inlineStr"/>
-    </row>
-    <row r="18" ht="73.5" customHeight="1">
+      <c r="I17" s="60" t="inlineStr">
+        <is>
+          <t>WP-S-04 v0.7 §3.7 (four rows) and §3.8, with T-30 to T-33. Rev 0.15 compares SFM-004, SFM-010.C2/C3, SFM-012.C1 and SFM-013.C1/C2 with them. Driver monitoring (SFM-022.C3, SFM-025.C1) waits for the H-09 FTTI (§3.8.4); follow-up is SFM-ACT-005. Late warnings found: SFM-ACT-021 (lateral) and SFM-ACT-022 (braking)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="100.5" customHeight="1">
       <c r="A18" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-018</t>
@@ -17329,7 +17333,7 @@
       <c r="H18" s="60" t="inlineStr"/>
       <c r="I18" s="60" t="inlineStr">
         <is>
-          <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1; TSR-626)</t>
+          <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1). Requirements: TSR-632 (per-ID transmitted and refused counts), TSR-626(d)/(e) (EPS and PCM acceptance status) and TSR-615, warning within 1 s (WP-S-02 §12.3a)</t>
         </is>
       </c>
     </row>
@@ -17397,8 +17401,62 @@
       <c r="H20" s="60" t="inlineStr"/>
       <c r="I20" s="60" t="inlineStr"/>
     </row>
+    <row r="21" ht="73.5" customHeight="1">
+      <c r="A21" s="60" t="inlineStr">
+        <is>
+          <t>SFM-ACT-021</t>
+        </is>
+      </c>
+      <c r="B21" s="60" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="C21" s="60" t="inlineStr">
+        <is>
+          <t>Make the insufficient-lateral-control warning timely (WP-S-04 §3.8.1): warn before the deficit has lasted 0.4 s, for example from the planned curvature against the envelope, or keep the deficit at or below about 0.5 m/s² through the steering limits and the ODD curve bound (WP-S-04 OI-2). A change to the ODD bound is a lead decision</t>
+        </is>
+      </c>
+      <c r="D21" s="60" t="inlineStr"/>
+      <c r="E21" s="60" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F21" s="60" t="inlineStr"/>
+      <c r="G21" s="60" t="inlineStr"/>
+      <c r="H21" s="60" t="inlineStr"/>
+      <c r="I21" s="60" t="inlineStr"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>SFM-ACT-022</t>
+        </is>
+      </c>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="C22" s="60" t="inlineStr">
+        <is>
+          <t>Measure the FCW onset after a lead brakes hard (WP-S-04 T-31, M-12) and compare it with the §3.8.2 budget (about 0.6 s at a 1.0 s gap). For pipeline lag (SFM-012.C1), detect it within that budget or show that the FCW path does not depend on the lagging process</t>
+        </is>
+      </c>
+      <c r="D22" s="60" t="inlineStr"/>
+      <c r="E22" s="60" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F22" s="60" t="inlineStr"/>
+      <c r="G22" s="60" t="inlineStr"/>
+      <c r="H22" s="60" t="inlineStr"/>
+      <c r="I22" s="60" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I20"/>
+  <autoFilter ref="A1:I22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18734,7 +18792,7 @@
       </c>
       <c r="G14" s="34" t="inlineStr">
         <is>
-          <t>Driver warned and takes over; no FTTI defined for the warning path</t>
+          <t>Driver warned and takes over; in time only for a deficit of about 0.5 m/s² or less (WP-S-04 §3.8.1)</t>
         </is>
       </c>
       <c r="H14" s="35" t="n">
@@ -18744,22 +18802,28 @@
         <v>6</v>
       </c>
       <c r="J14" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K14" s="36" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="L14" s="34" t="inlineStr"/>
+      <c r="L14" s="34" t="inlineStr">
+        <is>
+          <t>SG-02 insufficient lateral control (warning path, §3.8.1) · 1100 ms
+400 + 100 ms</t>
+        </is>
+      </c>
       <c r="M14" s="33" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>code derived</t>
         </is>
       </c>
       <c r="N14" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-017 · open</t>
+          <t>SFM-ACT-017 · completed
+SFM-ACT-021 · open</t>
         </is>
       </c>
       <c r="O14" s="37" t="inlineStr"/>
@@ -18796,7 +18860,7 @@
       </c>
       <c r="G15" s="34" t="inlineStr">
         <is>
-          <t>Driver warned and takes over; no FTTI defined for the warning path</t>
+          <t>Driver warned and takes over; in time only for a deficit of about 0.5 m/s² or less (WP-S-04 §3.8.1)</t>
         </is>
       </c>
       <c r="H15" s="35" t="n">
@@ -18806,22 +18870,28 @@
         <v>5</v>
       </c>
       <c r="J15" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K15" s="36" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="L15" s="34" t="inlineStr"/>
+      <c r="L15" s="34" t="inlineStr">
+        <is>
+          <t>SG-02 insufficient lateral control (warning path, §3.8.1) · 1100 ms
+400 + 100 ms</t>
+        </is>
+      </c>
       <c r="M15" s="33" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>code derived</t>
         </is>
       </c>
       <c r="N15" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-017 · open</t>
+          <t>SFM-ACT-017 · completed
+SFM-ACT-021 · open</t>
         </is>
       </c>
       <c r="O15" s="37" t="inlineStr"/>
@@ -18858,7 +18928,7 @@
       </c>
       <c r="G16" s="34" t="inlineStr">
         <is>
-          <t>Driver warned and takes over; no FTTI defined for the warning path</t>
+          <t>Driver warned and takes over; in time only for a deficit of about 0.5 m/s² or less (WP-S-04 §3.8.1)</t>
         </is>
       </c>
       <c r="H16" s="35" t="n">
@@ -18868,22 +18938,28 @@
         <v>6</v>
       </c>
       <c r="J16" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K16" s="36" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="L16" s="34" t="inlineStr"/>
+      <c r="L16" s="34" t="inlineStr">
+        <is>
+          <t>SG-02 insufficient lateral control (warning path, §3.8.1) · 1100 ms
+400 + 100 ms</t>
+        </is>
+      </c>
       <c r="M16" s="33" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>code derived</t>
         </is>
       </c>
       <c r="N16" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-017 · open</t>
+          <t>SFM-ACT-017 · completed
+SFM-ACT-021 · open</t>
         </is>
       </c>
       <c r="O16" s="37" t="inlineStr"/>
@@ -19789,7 +19865,7 @@
       <c r="O30" s="37" t="inlineStr"/>
       <c r="P30" s="37" t="inlineStr"/>
     </row>
-    <row r="31" ht="46.5" customHeight="1">
+    <row r="31" ht="73.5" customHeight="1">
       <c r="A31" s="34" t="inlineStr">
         <is>
           <t>SFM-010 · Insufficient deceleration for lead vehicle or stop</t>
@@ -19820,7 +19896,7 @@
       </c>
       <c r="G31" s="34" t="inlineStr">
         <is>
-          <t>Driver warned; no FTTI compared</t>
+          <t>Driver warned; FCW must sound within about 0.6 s of the lead braking at a 1.0 s gap (WP-S-04 §3.8.2), its onset is not derived (T-31, to be measured as M-12)</t>
         </is>
       </c>
       <c r="H31" s="35" t="n">
@@ -19837,7 +19913,11 @@
           <t>H</t>
         </is>
       </c>
-      <c r="L31" s="34" t="inlineStr"/>
+      <c r="L31" s="34" t="inlineStr">
+        <is>
+          <t>SG-06 late or insufficient braking warning (FCW, §3.8.2) · 1600 ms</t>
+        </is>
+      </c>
       <c r="M31" s="33" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -19846,13 +19926,13 @@
       <c r="N31" s="34" t="inlineStr">
         <is>
           <t>SFM-ACT-006 · open
-SFM-ACT-017 · open</t>
+SFM-ACT-022 · open</t>
         </is>
       </c>
       <c r="O31" s="37" t="inlineStr"/>
       <c r="P31" s="37" t="inlineStr"/>
     </row>
-    <row r="32" ht="46.5" customHeight="1">
+    <row r="32" ht="73.5" customHeight="1">
       <c r="A32" s="34" t="inlineStr">
         <is>
           <t>SFM-010 · Insufficient deceleration for lead vehicle or stop</t>
@@ -19883,7 +19963,7 @@
       </c>
       <c r="G32" s="34" t="inlineStr">
         <is>
-          <t>Driver warned; no FTTI compared</t>
+          <t>Driver warned; FCW must sound within about 0.6 s of the lead braking at a 1.0 s gap (WP-S-04 §3.8.2), its onset is not derived (T-31, to be measured as M-12)</t>
         </is>
       </c>
       <c r="H32" s="35" t="n">
@@ -19900,7 +19980,11 @@
           <t>H</t>
         </is>
       </c>
-      <c r="L32" s="34" t="inlineStr"/>
+      <c r="L32" s="34" t="inlineStr">
+        <is>
+          <t>SG-06 late or insufficient braking warning (FCW, §3.8.2) · 1600 ms</t>
+        </is>
+      </c>
       <c r="M32" s="33" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -19909,7 +19993,7 @@
       <c r="N32" s="34" t="inlineStr">
         <is>
           <t>SFM-ACT-003 · open
-SFM-ACT-017 · open</t>
+SFM-ACT-022 · open</t>
         </is>
       </c>
       <c r="O32" s="37" t="inlineStr"/>
@@ -20045,7 +20129,7 @@
       <c r="O34" s="37" t="inlineStr"/>
       <c r="P34" s="37" t="inlineStr"/>
     </row>
-    <row r="35" ht="46.5" customHeight="1">
+    <row r="35" ht="60" customHeight="1">
       <c r="A35" s="34" t="inlineStr">
         <is>
           <t>SFM-012 · Late reaction to lead vehicle braking</t>
@@ -20076,7 +20160,7 @@
       </c>
       <c r="G35" s="34" t="inlineStr">
         <is>
-          <t>Driver warned; no FTTI compared for late reaction</t>
+          <t>Driver warned only after the lag is averaged (about 1 s) and the 3 s soft disable; FCW is the remaining warning</t>
         </is>
       </c>
       <c r="H35" s="35" t="n">
@@ -20086,7 +20170,7 @@
         <v>6</v>
       </c>
       <c r="J35" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K35" s="36" t="inlineStr">
         <is>
@@ -20095,7 +20179,8 @@
       </c>
       <c r="L35" s="34" t="inlineStr">
         <is>
-          <t>1000 + 3000 ms</t>
+          <t>SG-06 late or insufficient braking warning (FCW, §3.8.2) · 1600 ms
+1000 + 3000 ms</t>
         </is>
       </c>
       <c r="M35" s="33" t="inlineStr">
@@ -20105,7 +20190,7 @@
       </c>
       <c r="N35" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-017 · open</t>
+          <t>SFM-ACT-022 · open</t>
         </is>
       </c>
       <c r="O35" s="37" t="inlineStr"/>
@@ -20194,7 +20279,7 @@
       </c>
       <c r="E37" s="34" t="inlineStr">
         <is>
-          <t>Panda grants control only on the PCM cruise engage edge read from the car bus, so a wrong host state alone does not grant actuation; frames are refused on every cycle. WP-S-04 has no FTTI row for SG-008, so the timing is not compared</t>
+          <t>Panda grants control only on the PCM cruise engage edge read from the car bus, so a wrong host state alone does not grant actuation; frames are refused on every cycle; within the 0.5 s unintended-engagement budget (WP-S-04 §3.8.3)</t>
         </is>
       </c>
       <c r="F37" s="34" t="inlineStr">
@@ -20214,7 +20299,7 @@
         <v>6</v>
       </c>
       <c r="J37" s="35" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K37" s="36" t="inlineStr">
         <is>
@@ -20223,7 +20308,8 @@
       </c>
       <c r="L37" s="34" t="inlineStr">
         <is>
-          <t>0 + 10 ms</t>
+          <t>SG-01 / SG-03 unintended engagement (System FMEA SG-008, §3.8.3) · 500 ms
+0 + 10 ms</t>
         </is>
       </c>
       <c r="M37" s="33" t="inlineStr">
@@ -20233,13 +20319,13 @@
       </c>
       <c r="N37" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-017 · open</t>
+          <t>SFM-ACT-013 · open</t>
         </is>
       </c>
       <c r="O37" s="37" t="inlineStr"/>
       <c r="P37" s="37" t="inlineStr"/>
     </row>
-    <row r="38" ht="60" customHeight="1">
+    <row r="38" ht="73.5" customHeight="1">
       <c r="A38" s="34" t="inlineStr">
         <is>
           <t>SFM-013 · Engagement without driver request or with entry conditions not met</t>
@@ -20260,7 +20346,7 @@
       </c>
       <c r="E38" s="34" t="inlineStr">
         <is>
-          <t>Panda parses the PCM cruise state itself and grants control only on its engage edge; a host parsing error does not grant actuation. No SG-008 FTTI row in WP-S-04</t>
+          <t>Panda parses the PCM cruise state itself and grants control only on its engage edge; a host parsing error does not grant actuation; within the 0.5 s unintended-engagement budget (WP-S-04 §3.8.3)</t>
         </is>
       </c>
       <c r="F38" s="34" t="inlineStr">
@@ -20280,7 +20366,7 @@
         <v>6</v>
       </c>
       <c r="J38" s="35" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K38" s="36" t="inlineStr">
         <is>
@@ -20289,7 +20375,8 @@
       </c>
       <c r="L38" s="34" t="inlineStr">
         <is>
-          <t>0 + 10 ms</t>
+          <t>SG-01 / SG-03 unintended engagement (System FMEA SG-008, §3.8.3) · 500 ms
+0 + 10 ms</t>
         </is>
       </c>
       <c r="M38" s="33" t="inlineStr">
@@ -20299,7 +20386,7 @@
       </c>
       <c r="N38" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-017 · open</t>
+          <t>SFM-ACT-013 · open</t>
         </is>
       </c>
       <c r="O38" s="37" t="inlineStr"/>
@@ -21328,7 +21415,7 @@
       </c>
       <c r="G55" s="34" t="inlineStr">
         <is>
-          <t>Driver monitored by wheel touch; no FTTI defined for DM</t>
+          <t>Driver monitored by wheel touch; no FTTI until the H-09 goal has one (WP-S-04 §3.8.4)</t>
         </is>
       </c>
       <c r="H55" s="35" t="n">
@@ -21353,7 +21440,7 @@
       </c>
       <c r="N55" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-017 · open</t>
+          <t>SFM-ACT-005 · decision pending</t>
         </is>
       </c>
       <c r="O55" s="37" t="inlineStr"/>
@@ -22226,7 +22313,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.14 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.15 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.16: inherited rows follow the SW FMEA at BL-005; ODD up to 110 km/h
- SFM-016.C2 (late disengagement, SWF-034.C1): O 8 -> 5, D 10 -> 8.
  The BL-005 controlsMismatch supervision (TSR-621) and its unit tests.
  AP stays H.
- SFM-029.C1 (wrong safety model or parameter, SWF-013.C2): O 8 -> 3,
  D 9 -> 4. The reference build is the default and checked in CI
  (SWF-ACT-009 completed). AP H -> L; MSR F 8 -> 3, M 7 kept.
- Scope: the ODD speed bound of 110 km/h (DQ-260).
- fmea-plan v0.13. Every other inherited row matches its source.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -261,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -399,6 +399,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -820,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.15 · draft</t>
+          <t>0.16 · draft</t>
         </is>
       </c>
     </row>
@@ -868,7 +871,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>LionDriver as installed on the reference configuration CFG-001 (Corolla E210 · ZRE212 · US, US sedan MY2020-2022) with comma 3X and integrated panda, software BL-005 (structure and failure analysis written at BL-001, risk analysis at BL-004, MSR re-rated at BL-005), while the vehicle is driven by a licensed driver inside the ODD: limited-access highways only since WP-C-02 / WP-C-03 v0.4 (DQ-023). Functions F1-F7 per fmea-plan.md section 3.1, plus F8 (stock vehicle safety functions are preserved), added because the harness intercepts the stock ADAS camera.</t>
+          <t>LionDriver as installed on the reference configuration CFG-001 (Corolla E210 · ZRE212 · US, US sedan MY2020-2022) with comma 3X and integrated panda, software BL-005 (structure and failure analysis written at BL-001, risk analysis at BL-004, MSR re-rated at BL-005), while the vehicle is driven by a licensed driver inside the ODD: limited-access highways only since WP-C-02 / WP-C-03 v0.4 (DQ-023), up to 110 km/h (DQ-260). Functions F1-F7 per fmea-plan.md section 3.1, plus F8 (stock vehicle safety functions are preserved), added because the harness intercepts the stock ADAS camera.</t>
         </is>
       </c>
     </row>
@@ -918,7 +921,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17">
@@ -938,7 +941,7 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -8938,7 +8941,7 @@
       <c r="R47" s="37" t="inlineStr"/>
       <c r="S47" s="37" t="inlineStr"/>
     </row>
-    <row r="48" ht="73.5" customHeight="1">
+    <row r="48" ht="100.5" customHeight="1">
       <c r="A48" s="39" t="n"/>
       <c r="B48" s="39" t="n"/>
       <c r="C48" s="39" t="n"/>
@@ -8958,7 +8961,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Debounce/counters too long (e.g. excessive actuation 0.25 s, mismatch counter 200 frames)</t>
+            <t>Debounce or counters too long (e.g. excessive actuation 0.25 s); at BL-005 a defect in the controlsMismatch supervision (2 consecutive samples, at most 0.5 s, TSR-621), which replaced the upstream 200-frame counter</t>
           </r>
           <r>
             <rPr>
@@ -8979,7 +8982,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Upstream threshold; TSR-621 records it as partial</t>
+            <t>• New LionDriver supervision code (#51, TSR-621); rated in the SW FMEA</t>
           </r>
           <r>
             <rPr>
@@ -8988,27 +8991,36 @@
               <sz val="8"/>
             </rPr>
             <t xml:space="preserve">
-   openpilot/selfdrive/selfdrived/selfdrived.py:504-514</t>
+   openpilot/selfdrive/selfdrived/supervision.py</t>
           </r>
         </is>
       </c>
       <c r="J48" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K48" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• test_supervision.py targets the cause (consecutive samples, 0.5 s bound, engagement grace); not run in CI at BL-005 and not proven by mutation (SWF-ACT-055)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/selfdrived/tests/test_supervision.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L48" s="42" t="n">
         <v>8</v>
-      </c>
-      <c r="K48" s="41" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="008A5A00"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• No test targets this cause</t>
-          </r>
-        </is>
-      </c>
-      <c r="L48" s="43" t="n">
-        <v>10</v>
       </c>
       <c r="M48" s="44" t="inlineStr">
         <is>
@@ -13178,7 +13190,7 @@
       <c r="R70" s="45" t="inlineStr"/>
       <c r="S70" s="45" t="inlineStr"/>
     </row>
-    <row r="71" ht="73.5" customHeight="1">
+    <row r="71" ht="114" customHeight="1">
       <c r="A71" s="30" t="inlineStr">
         <is>
           <r>
@@ -13415,7 +13427,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Panda safety code: MISRA C:2012, 100% line coverage, review; rated in the SW FMEA</t>
+            <t>• The openpilot build and the release script select the reference build (LIONDRIVER_REFERENCE=1) by default, and pandad sets a car mode only on a panda that reports it (TSR-619); rated in the SW FMEA</t>
           </r>
           <r>
             <rPr>
@@ -13429,17 +13441,17 @@
         </is>
       </c>
       <c r="J71" s="35" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K71" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="008A5A00"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• As rated in the SW FMEA: no test covers the build configuration</t>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• CI job panda_reference_release_build checks every firmware compile for -DLIONDRIVER_REFERENCE; host test of the reference-build health flag. Checks the build configuration, not the signed release image (PFMEA PFM-001)</t>
           </r>
           <r>
             <rPr>
@@ -13448,16 +13460,16 @@
               <sz val="8"/>
             </rPr>
             <t xml:space="preserve">
-   assurance/08-analyses/fmea/analyses/sw-fmea.yaml</t>
-          </r>
-        </is>
-      </c>
-      <c r="L71" s="46" t="n">
-        <v>9</v>
-      </c>
-      <c r="M71" s="36" t="inlineStr">
-        <is>
-          <t>H</t>
+   .github/workflows/safety.yaml</t>
+          </r>
+        </is>
+      </c>
+      <c r="L71" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="M71" s="58" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="N71" s="34" t="inlineStr">
@@ -13477,7 +13489,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Rated, and actioned where needed, in the SW FMEA (SWF-013.C2 O8 D9, SWF-ACT-009; open LionDriver#36/#41 set and check the reference build); this row inherits that rating</t>
+            <t>Rated, and actioned, in the SW FMEA (SWF-013.C2 O3 D4 at BL-005, SWF-ACT-009 completed); this row inherits that rating</t>
           </r>
         </is>
       </c>
@@ -16343,7 +16355,7 @@
           </r>
         </is>
       </c>
-      <c r="O86" s="58" t="inlineStr">
+      <c r="O86" s="59" t="inlineStr">
         <is>
           <t>decision pending</t>
         </is>
@@ -16641,7 +16653,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.15 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.16 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -16671,79 +16683,79 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="59" t="inlineStr">
+      <c r="A1" s="60" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="B1" s="59" t="inlineStr">
+      <c r="B1" s="60" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="C1" s="59" t="inlineStr">
+      <c r="C1" s="60" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="59" t="inlineStr">
+      <c r="D1" s="60" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E1" s="59" t="inlineStr">
+      <c r="E1" s="60" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="59" t="inlineStr">
+      <c r="F1" s="60" t="inlineStr">
         <is>
           <t>Causes</t>
         </is>
       </c>
-      <c r="G1" s="59" t="inlineStr">
+      <c r="G1" s="60" t="inlineStr">
         <is>
           <t>Revised S/O/D</t>
         </is>
       </c>
-      <c r="H1" s="59" t="inlineStr">
+      <c r="H1" s="60" t="inlineStr">
         <is>
           <t>Revised AP</t>
         </is>
       </c>
-      <c r="I1" s="59" t="inlineStr">
+      <c r="I1" s="60" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
     </row>
     <row r="2" ht="127.5" customHeight="1">
-      <c r="A2" s="60" t="inlineStr">
+      <c r="A2" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-001</t>
         </is>
       </c>
-      <c r="B2" s="60" t="inlineStr">
+      <c r="B2" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C2" s="60" t="inlineStr">
+      <c r="C2" s="61" t="inlineStr">
         <is>
           <t>Derive steering and acceleration envelopes from measurements on the reference vehicle and set the panda limits from them, independently of the SoC limits (same as SWF-ACT-003, FSC FOI-001)</t>
         </is>
       </c>
-      <c r="D2" s="60" t="inlineStr">
+      <c r="D2" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E2" s="60" t="inlineStr">
+      <c r="E2" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F2" s="60" t="inlineStr">
+      <c r="F2" s="61" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
@@ -16756,37 +16768,37 @@
 SFM-029.C2</t>
         </is>
       </c>
-      <c r="G2" s="60" t="inlineStr"/>
-      <c r="H2" s="60" t="inlineStr"/>
-      <c r="I2" s="60" t="inlineStr"/>
+      <c r="G2" s="61" t="inlineStr"/>
+      <c r="H2" s="61" t="inlineStr"/>
+      <c r="I2" s="61" t="inlineStr"/>
     </row>
     <row r="3" ht="127.5" customHeight="1">
-      <c r="A3" s="60" t="inlineStr">
+      <c r="A3" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-002</t>
         </is>
       </c>
-      <c r="B3" s="60" t="inlineStr">
+      <c r="B3" s="61" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C3" s="60" t="inlineStr">
+      <c r="C3" s="61" t="inlineStr">
         <is>
           <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
         </is>
       </c>
-      <c r="D3" s="60" t="inlineStr">
+      <c r="D3" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E3" s="60" t="inlineStr">
+      <c r="E3" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F3" s="60" t="inlineStr">
+      <c r="F3" s="61" t="inlineStr">
         <is>
           <t>SFM-002.C4
 SFM-004.C3
@@ -16799,37 +16811,37 @@
 SFM-030.C1</t>
         </is>
       </c>
-      <c r="G3" s="60" t="inlineStr"/>
-      <c r="H3" s="60" t="inlineStr"/>
-      <c r="I3" s="60" t="inlineStr"/>
+      <c r="G3" s="61" t="inlineStr"/>
+      <c r="H3" s="61" t="inlineStr"/>
+      <c r="I3" s="61" t="inlineStr"/>
     </row>
     <row r="4" ht="343.5" customHeight="1">
-      <c r="A4" s="60" t="inlineStr">
+      <c r="A4" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-003</t>
         </is>
       </c>
-      <c r="B4" s="60" t="inlineStr">
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C4" s="60" t="inlineStr">
+      <c r="C4" s="61" t="inlineStr">
         <is>
           <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
         </is>
       </c>
-      <c r="D4" s="60" t="inlineStr">
+      <c r="D4" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E4" s="60" t="inlineStr">
+      <c r="E4" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F4" s="60" t="inlineStr">
+      <c r="F4" s="61" t="inlineStr">
         <is>
           <t>SFM-003.C1
 SFM-003.C2
@@ -16858,72 +16870,72 @@
 SFM-033.C3</t>
         </is>
       </c>
-      <c r="G4" s="60" t="inlineStr"/>
-      <c r="H4" s="60" t="inlineStr"/>
-      <c r="I4" s="60" t="inlineStr"/>
+      <c r="G4" s="61" t="inlineStr"/>
+      <c r="H4" s="61" t="inlineStr"/>
+      <c r="I4" s="61" t="inlineStr"/>
     </row>
     <row r="5" ht="114" customHeight="1">
-      <c r="A5" s="60" t="inlineStr">
+      <c r="A5" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-005</t>
         </is>
       </c>
-      <c r="B5" s="60" t="inlineStr">
+      <c r="B5" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C5" s="60" t="inlineStr">
+      <c r="C5" s="61" t="inlineStr">
         <is>
           <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided. The requirement is TSR-633 (terminal reaction, ASIL A proposed) with TSR-611 (WP-S-02 §12.3a); the reaction is lead decision DQ-340. The H-09 FTTI is not yet set, so the timing rows of WP-S-04 §3.8.4 cannot be compared</t>
         </is>
       </c>
-      <c r="D5" s="60" t="inlineStr">
+      <c r="D5" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E5" s="60" t="inlineStr">
+      <c r="E5" s="61" t="inlineStr">
         <is>
           <t>decision pending</t>
         </is>
       </c>
-      <c r="F5" s="60" t="inlineStr">
+      <c r="F5" s="61" t="inlineStr">
         <is>
           <t>SFM-025.C1</t>
         </is>
       </c>
-      <c r="G5" s="60" t="inlineStr"/>
-      <c r="H5" s="60" t="inlineStr"/>
-      <c r="I5" s="60" t="inlineStr"/>
+      <c r="G5" s="61" t="inlineStr"/>
+      <c r="H5" s="61" t="inlineStr"/>
+      <c r="I5" s="61" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-006</t>
         </is>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="61" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="61" t="inlineStr">
         <is>
           <t>Establish on the reference car which stock TSS2 functions (PCS/AEB, FCW) remain available with LionDriver installed and longitudinal control enabled, and verify the stock pre-collision path after installation (PFMEA PFM-014)</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E6" s="60" t="inlineStr">
+      <c r="E6" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F6" s="60" t="inlineStr">
+      <c r="F6" s="61" t="inlineStr">
         <is>
           <t>SFM-010.C2
 SFM-033.C1
@@ -16931,37 +16943,37 @@
 SFM-036.C2</t>
         </is>
       </c>
-      <c r="G6" s="60" t="inlineStr"/>
-      <c r="H6" s="60" t="inlineStr"/>
-      <c r="I6" s="60" t="inlineStr"/>
+      <c r="G6" s="61" t="inlineStr"/>
+      <c r="H6" s="61" t="inlineStr"/>
+      <c r="I6" s="61" t="inlineStr"/>
     </row>
     <row r="7" ht="73.5" customHeight="1">
-      <c r="A7" s="60" t="inlineStr">
+      <c r="A7" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-007</t>
         </is>
       </c>
-      <c r="B7" s="60" t="inlineStr">
+      <c r="B7" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C7" s="60" t="inlineStr">
+      <c r="C7" s="61" t="inlineStr">
         <is>
           <t>Supervise the alert channels: treat loss of ui or soundd liveness, or a stale displayed state, as a fault that escalates (audible fallback, disengagement) instead of continuing silently</t>
         </is>
       </c>
-      <c r="D7" s="60" t="inlineStr">
+      <c r="D7" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E7" s="60" t="inlineStr">
+      <c r="E7" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F7" s="60" t="inlineStr">
+      <c r="F7" s="61" t="inlineStr">
         <is>
           <t>SFM-015.C1
 SFM-026.C1
@@ -16970,76 +16982,76 @@
 SFM-028.C1</t>
         </is>
       </c>
-      <c r="G7" s="60" t="inlineStr"/>
-      <c r="H7" s="60" t="inlineStr"/>
-      <c r="I7" s="60" t="inlineStr"/>
+      <c r="G7" s="61" t="inlineStr"/>
+      <c r="H7" s="61" t="inlineStr"/>
+      <c r="I7" s="61" t="inlineStr"/>
     </row>
     <row r="8" ht="73.5" customHeight="1">
-      <c r="A8" s="60" t="inlineStr">
+      <c r="A8" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-008</t>
         </is>
       </c>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="B8" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C8" s="60" t="inlineStr">
+      <c r="C8" s="61" t="inlineStr">
         <is>
           <t>Allow engagement only when the fingerprint, CarParams and panda safety parameter match the reference configuration AC-001 (refuse fuzzy matches in the reference build); see PFMEA PFM-013</t>
         </is>
       </c>
-      <c r="D8" s="60" t="inlineStr">
+      <c r="D8" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E8" s="60" t="inlineStr">
+      <c r="E8" s="61" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F8" s="60" t="inlineStr">
+      <c r="F8" s="61" t="inlineStr">
         <is>
           <t>SFM-032.C1</t>
         </is>
       </c>
-      <c r="G8" s="60" t="inlineStr"/>
-      <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr">
+      <c r="G8" s="61" t="inlineStr"/>
+      <c r="H8" s="61" t="inlineStr"/>
+      <c r="I8" s="61" t="inlineStr">
         <is>
           <t>BL-005: the reference build is the default (LionDriver #36), the panda accepts only TOYOTA parameter 73 (reference_lock.h) and pandad configures a car mode only on a reference panda (#41). Fuzzy fingerprint matches are still accepted on the host (SFM-032.C1)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="100.5" customHeight="1">
-      <c r="A9" s="60" t="inlineStr">
+      <c r="A9" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-009</t>
         </is>
       </c>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>prevention</t>
         </is>
       </c>
-      <c r="C9" s="60" t="inlineStr">
+      <c r="C9" s="61" t="inlineStr">
         <is>
           <t>Produce SOTIF / ISO PAS 8800 evidence for the neural-network elements (driving model, lead detection, driver monitoring model) per WP-V-02..04, including fault-induced inputs (corrupted or stale frames)</t>
         </is>
       </c>
-      <c r="D9" s="60" t="inlineStr">
+      <c r="D9" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E9" s="60" t="inlineStr">
+      <c r="E9" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F9" s="60" t="inlineStr">
+      <c r="F9" s="61" t="inlineStr">
         <is>
           <t>SFM-002.C2
 SFM-003.C3
@@ -17050,37 +17062,37 @@
 SFM-022.C2</t>
         </is>
       </c>
-      <c r="G9" s="60" t="inlineStr"/>
-      <c r="H9" s="60" t="inlineStr"/>
-      <c r="I9" s="60" t="inlineStr"/>
+      <c r="G9" s="61" t="inlineStr"/>
+      <c r="H9" s="61" t="inlineStr"/>
+      <c r="I9" s="61" t="inlineStr"/>
     </row>
     <row r="10" ht="73.5" customHeight="1">
-      <c r="A10" s="60" t="inlineStr">
+      <c r="A10" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-010</t>
         </is>
       </c>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="61" t="inlineStr">
         <is>
           <t>Justify every SOFT_DISABLE reaction and debounce against the FTTI (WP-S-04) and alert at once when the panda withdraws authority while engaged (controlsMismatch debounce)</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
+      <c r="D10" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E10" s="60" t="inlineStr">
+      <c r="E10" s="61" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F10" s="60" t="inlineStr">
+      <c r="F10" s="61" t="inlineStr">
         <is>
           <t>SFM-014.C2
 SFM-015.C2
@@ -17088,372 +17100,372 @@
 SFM-016.C2</t>
         </is>
       </c>
-      <c r="G10" s="60" t="inlineStr"/>
-      <c r="H10" s="60" t="inlineStr"/>
-      <c r="I10" s="60" t="inlineStr">
+      <c r="G10" s="61" t="inlineStr"/>
+      <c r="H10" s="61" t="inlineStr"/>
+      <c r="I10" s="61" t="inlineStr">
         <is>
           <t>controlsMismatch debounce cut from 200 cumulative samples (~2 s) to 2 consecutive samples, at most 0.5 s (change-2026-10-13-host-supervision.md); credited at BL-005 (SFM-015.C2 M 6). FTTI justification of SOFT_DISABLE reactions open</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="60" t="inlineStr">
+      <c r="A11" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-011</t>
         </is>
       </c>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C11" s="60" t="inlineStr">
+      <c r="C11" s="61" t="inlineStr">
         <is>
           <t>Alert the driver when stock cruise stays engaged while the item is disengaged (cruiseMismatch has no alert at BL-004)</t>
         </is>
       </c>
-      <c r="D11" s="60" t="inlineStr">
+      <c r="D11" s="61" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E11" s="61" t="inlineStr">
+      <c r="E11" s="62" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F11" s="60" t="inlineStr">
+      <c r="F11" s="61" t="inlineStr">
         <is>
           <t>SFM-021.C1
 SFM-021.C2</t>
         </is>
       </c>
-      <c r="G11" s="60" t="inlineStr"/>
-      <c r="H11" s="60" t="inlineStr"/>
-      <c r="I11" s="60" t="inlineStr">
+      <c r="G11" s="61" t="inlineStr"/>
+      <c r="H11" s="61" t="inlineStr"/>
+      <c r="I11" s="61" t="inlineStr">
         <is>
           <t>cruiseMismatch now alerts after 1 s (change-2026-10-13-host-supervision.md); see SWF-ACT-034</t>
         </is>
       </c>
     </row>
     <row r="12" ht="73.5" customHeight="1">
-      <c r="A12" s="60" t="inlineStr">
+      <c r="A12" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-012</t>
         </is>
       </c>
-      <c r="B12" s="60" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C12" s="61" t="inlineStr">
         <is>
           <t>Measure on the HIL bench and the reference car (WP-V-05) how the panda reacts to over-limit and not-engaged steering and acceleration frames and to driver brake, gas and cancel inputs, and what the EPS and PCM do when frames are refused; re-rate the MSR rows from code-derived to measured timing</t>
         </is>
       </c>
-      <c r="D12" s="60" t="inlineStr"/>
-      <c r="E12" s="60" t="inlineStr">
+      <c r="D12" s="61" t="inlineStr"/>
+      <c r="E12" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F12" s="60" t="inlineStr"/>
-      <c r="G12" s="60" t="inlineStr"/>
-      <c r="H12" s="60" t="inlineStr"/>
-      <c r="I12" s="60" t="inlineStr"/>
+      <c r="F12" s="61" t="inlineStr"/>
+      <c r="G12" s="61" t="inlineStr"/>
+      <c r="H12" s="61" t="inlineStr"/>
+      <c r="I12" s="61" t="inlineStr"/>
     </row>
     <row r="13" ht="87" customHeight="1">
-      <c r="A13" s="60" t="inlineStr">
+      <c r="A13" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-013</t>
         </is>
       </c>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C13" s="60" t="inlineStr">
+      <c r="C13" s="61" t="inlineStr">
         <is>
           <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert. The requirement is TSR-630, within 0.3 s (WP-S-02 §12.3a; WP-S-04 T-32, not implemented)</t>
         </is>
       </c>
-      <c r="D13" s="60" t="inlineStr"/>
-      <c r="E13" s="60" t="inlineStr">
+      <c r="D13" s="61" t="inlineStr"/>
+      <c r="E13" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F13" s="60" t="inlineStr"/>
-      <c r="G13" s="60" t="inlineStr"/>
-      <c r="H13" s="60" t="inlineStr"/>
-      <c r="I13" s="60" t="inlineStr"/>
+      <c r="F13" s="61" t="inlineStr"/>
+      <c r="G13" s="61" t="inlineStr"/>
+      <c r="H13" s="61" t="inlineStr"/>
+      <c r="I13" s="61" t="inlineStr"/>
     </row>
     <row r="14" ht="46.5" customHeight="1">
-      <c r="A14" s="60" t="inlineStr">
+      <c r="A14" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-014</t>
         </is>
       </c>
-      <c r="B14" s="60" t="inlineStr">
+      <c r="B14" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C14" s="60" t="inlineStr">
+      <c r="C14" s="61" t="inlineStr">
         <is>
           <t>Specify in the TSC a steering-direction plausibility monitor (commanded torque sign against measured yaw rate and lane-relative lateral motion), or justify its absence against HZ-003</t>
         </is>
       </c>
-      <c r="D14" s="60" t="inlineStr"/>
-      <c r="E14" s="60" t="inlineStr">
+      <c r="D14" s="61" t="inlineStr"/>
+      <c r="E14" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F14" s="60" t="inlineStr"/>
-      <c r="G14" s="60" t="inlineStr"/>
-      <c r="H14" s="60" t="inlineStr"/>
-      <c r="I14" s="60" t="inlineStr"/>
+      <c r="F14" s="61" t="inlineStr"/>
+      <c r="G14" s="61" t="inlineStr"/>
+      <c r="H14" s="61" t="inlineStr"/>
+      <c r="I14" s="61" t="inlineStr"/>
     </row>
     <row r="15" ht="100.5" customHeight="1">
-      <c r="A15" s="60" t="inlineStr">
+      <c r="A15" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-015</t>
         </is>
       </c>
-      <c r="B15" s="60" t="inlineStr">
+      <c r="B15" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C15" s="60" t="inlineStr">
+      <c r="C15" s="61" t="inlineStr">
         <is>
           <t>Detect stale commands and inputs within the SG-01 FTTI: command-frame freshness in the MCU with an active zero frame (TSR-408, TSR-109) and frozen-content and age checks on model outputs in controlsd (TSR-602, TSR-631, AIR-17)</t>
         </is>
       </c>
-      <c r="D15" s="60" t="inlineStr"/>
-      <c r="E15" s="60" t="inlineStr">
+      <c r="D15" s="61" t="inlineStr"/>
+      <c r="E15" s="61" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F15" s="60" t="inlineStr"/>
-      <c r="G15" s="60" t="inlineStr"/>
-      <c r="H15" s="60" t="inlineStr"/>
-      <c r="I15" s="60" t="inlineStr">
+      <c r="F15" s="61" t="inlineStr"/>
+      <c r="G15" s="61" t="inlineStr"/>
+      <c r="H15" s="61" t="inlineStr"/>
+      <c r="I15" s="61" t="inlineStr">
         <is>
           <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3). The frozen-content check is TSR-631, with the age taken from the source timestamp (WP-S-02 §12.3a)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="73.5" customHeight="1">
-      <c r="A16" s="60" t="inlineStr">
+      <c r="A16" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-016</t>
         </is>
       </c>
-      <c r="B16" s="60" t="inlineStr">
+      <c r="B16" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C16" s="60" t="inlineStr">
+      <c r="C16" s="61" t="inlineStr">
         <is>
           <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue. Requirements: TSR-304 (timing tied to the SG-05 budget) and TSR-628 (WP-S-02 §12.3a)</t>
         </is>
       </c>
-      <c r="D16" s="60" t="inlineStr"/>
-      <c r="E16" s="60" t="inlineStr">
+      <c r="D16" s="61" t="inlineStr"/>
+      <c r="E16" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F16" s="60" t="inlineStr"/>
-      <c r="G16" s="60" t="inlineStr"/>
-      <c r="H16" s="60" t="inlineStr"/>
-      <c r="I16" s="60" t="inlineStr"/>
+      <c r="F16" s="61" t="inlineStr"/>
+      <c r="G16" s="61" t="inlineStr"/>
+      <c r="H16" s="61" t="inlineStr"/>
+      <c r="I16" s="61" t="inlineStr"/>
     </row>
     <row r="17" ht="87" customHeight="1">
-      <c r="A17" s="60" t="inlineStr">
+      <c r="A17" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-017</t>
         </is>
       </c>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C17" s="60" t="inlineStr">
+      <c r="C17" s="61" t="inlineStr">
         <is>
           <t>Add WP-S-04 FTTI rows for the warning paths without one (insufficient lateral control, late or insufficient braking warnings, SG-008 unintended engagement, driver monitoring), so these mechanisms can be compared with a time budget</t>
         </is>
       </c>
-      <c r="D17" s="60" t="inlineStr"/>
-      <c r="E17" s="61" t="inlineStr">
+      <c r="D17" s="61" t="inlineStr"/>
+      <c r="E17" s="62" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F17" s="60" t="inlineStr"/>
-      <c r="G17" s="60" t="inlineStr"/>
-      <c r="H17" s="60" t="inlineStr"/>
-      <c r="I17" s="60" t="inlineStr">
+      <c r="F17" s="61" t="inlineStr"/>
+      <c r="G17" s="61" t="inlineStr"/>
+      <c r="H17" s="61" t="inlineStr"/>
+      <c r="I17" s="61" t="inlineStr">
         <is>
           <t>WP-S-04 v0.7 §3.7 (four rows) and §3.8, with T-30 to T-33. Rev 0.15 compares SFM-004, SFM-010.C2/C3, SFM-012.C1 and SFM-013.C1/C2 with them. Driver monitoring (SFM-022.C3, SFM-025.C1) waits for the H-09 FTTI (§3.8.4); follow-up is SFM-ACT-005. Late warnings found: SFM-ACT-021 (lateral) and SFM-ACT-022 (braking)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="100.5" customHeight="1">
-      <c r="A18" s="60" t="inlineStr">
+      <c r="A18" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-018</t>
         </is>
       </c>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C18" s="60" t="inlineStr">
+      <c r="C18" s="61" t="inlineStr">
         <is>
           <t>Detect silent loss of the actuation path: report forwarded and refused TX frames from the panda, and compare EPS and PCM acceptance (LKA_STATE, ACC status) with the commands, warning within the SG-02/06 1 s budget</t>
         </is>
       </c>
-      <c r="D18" s="60" t="inlineStr"/>
-      <c r="E18" s="60" t="inlineStr">
+      <c r="D18" s="61" t="inlineStr"/>
+      <c r="E18" s="61" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F18" s="60" t="inlineStr"/>
-      <c r="G18" s="60" t="inlineStr"/>
-      <c r="H18" s="60" t="inlineStr"/>
-      <c r="I18" s="60" t="inlineStr">
+      <c r="F18" s="61" t="inlineStr"/>
+      <c r="G18" s="61" t="inlineStr"/>
+      <c r="H18" s="61" t="inlineStr"/>
+      <c r="I18" s="61" t="inlineStr">
         <is>
           <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1). Requirements: TSR-632 (per-ID transmitted and refused counts), TSR-626(d)/(e) (EPS and PCM acceptance status) and TSR-615, warning within 1 s (WP-S-02 §12.3a)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="60" t="inlineStr">
+      <c r="A19" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-019</t>
         </is>
       </c>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="61" t="inlineStr">
         <is>
           <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
         </is>
       </c>
-      <c r="D19" s="60" t="inlineStr"/>
-      <c r="E19" s="60" t="inlineStr">
+      <c r="D19" s="61" t="inlineStr"/>
+      <c r="E19" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F19" s="60" t="inlineStr">
+      <c r="F19" s="61" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
 SFM-002.C4</t>
         </is>
       </c>
-      <c r="G19" s="60" t="inlineStr"/>
-      <c r="H19" s="60" t="inlineStr"/>
-      <c r="I19" s="60" t="inlineStr"/>
+      <c r="G19" s="61" t="inlineStr"/>
+      <c r="H19" s="61" t="inlineStr"/>
+      <c r="I19" s="61" t="inlineStr"/>
     </row>
     <row r="20" ht="73.5" customHeight="1">
-      <c r="A20" s="60" t="inlineStr">
+      <c r="A20" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-020</t>
         </is>
       </c>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
+      <c r="C20" s="61" t="inlineStr">
         <is>
           <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
         </is>
       </c>
-      <c r="D20" s="60" t="inlineStr"/>
-      <c r="E20" s="60" t="inlineStr">
+      <c r="D20" s="61" t="inlineStr"/>
+      <c r="E20" s="61" t="inlineStr">
         <is>
           <t>decision pending</t>
         </is>
       </c>
-      <c r="F20" s="60" t="inlineStr">
+      <c r="F20" s="61" t="inlineStr">
         <is>
           <t>SFM-036.C1</t>
         </is>
       </c>
-      <c r="G20" s="60" t="inlineStr"/>
-      <c r="H20" s="60" t="inlineStr"/>
-      <c r="I20" s="60" t="inlineStr"/>
+      <c r="G20" s="61" t="inlineStr"/>
+      <c r="H20" s="61" t="inlineStr"/>
+      <c r="I20" s="61" t="inlineStr"/>
     </row>
     <row r="21" ht="73.5" customHeight="1">
-      <c r="A21" s="60" t="inlineStr">
+      <c r="A21" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-021</t>
         </is>
       </c>
-      <c r="B21" s="60" t="inlineStr">
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C21" s="60" t="inlineStr">
+      <c r="C21" s="61" t="inlineStr">
         <is>
           <t>Make the insufficient-lateral-control warning timely (WP-S-04 §3.8.1): warn before the deficit has lasted 0.4 s, for example from the planned curvature against the envelope, or keep the deficit at or below about 0.5 m/s² through the steering limits and the ODD curve bound (WP-S-04 OI-2). A change to the ODD bound is a lead decision</t>
         </is>
       </c>
-      <c r="D21" s="60" t="inlineStr"/>
-      <c r="E21" s="60" t="inlineStr">
+      <c r="D21" s="61" t="inlineStr"/>
+      <c r="E21" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F21" s="60" t="inlineStr"/>
-      <c r="G21" s="60" t="inlineStr"/>
-      <c r="H21" s="60" t="inlineStr"/>
-      <c r="I21" s="60" t="inlineStr"/>
+      <c r="F21" s="61" t="inlineStr"/>
+      <c r="G21" s="61" t="inlineStr"/>
+      <c r="H21" s="61" t="inlineStr"/>
+      <c r="I21" s="61" t="inlineStr"/>
     </row>
     <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="60" t="inlineStr">
+      <c r="A22" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-022</t>
         </is>
       </c>
-      <c r="B22" s="60" t="inlineStr">
+      <c r="B22" s="61" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C22" s="60" t="inlineStr">
+      <c r="C22" s="61" t="inlineStr">
         <is>
           <t>Measure the FCW onset after a lead brakes hard (WP-S-04 T-31, M-12) and compare it with the §3.8.2 budget (about 0.6 s at a 1.0 s gap). For pipeline lag (SFM-012.C1), detect it within that budget or show that the FCW path does not depend on the lagging process</t>
         </is>
       </c>
-      <c r="D22" s="60" t="inlineStr"/>
-      <c r="E22" s="60" t="inlineStr">
+      <c r="D22" s="61" t="inlineStr"/>
+      <c r="E22" s="61" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F22" s="60" t="inlineStr"/>
-      <c r="G22" s="60" t="inlineStr"/>
-      <c r="H22" s="60" t="inlineStr"/>
-      <c r="I22" s="60" t="inlineStr"/>
+      <c r="F22" s="61" t="inlineStr"/>
+      <c r="G22" s="61" t="inlineStr"/>
+      <c r="H22" s="61" t="inlineStr"/>
+      <c r="I22" s="61" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I22"/>
@@ -17478,50 +17490,50 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="59" t="inlineStr">
+      <c r="A1" s="60" t="inlineStr">
         <is>
           <t>Element</t>
         </is>
       </c>
-      <c r="B1" s="59" t="inlineStr">
+      <c r="B1" s="60" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="59" t="inlineStr">
+      <c r="C1" s="60" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="D1" s="59" t="inlineStr">
+      <c r="D1" s="60" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="E1" s="59" t="inlineStr">
+      <c r="E1" s="60" t="inlineStr">
         <is>
           <t>Functions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="222" customHeight="1">
-      <c r="A2" s="60" t="inlineStr">
+      <c r="A2" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="B2" s="60" t="inlineStr">
+      <c r="B2" s="61" t="inlineStr">
         <is>
           <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
         </is>
       </c>
-      <c r="C2" s="60" t="inlineStr">
+      <c r="C2" s="61" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D2" s="60" t="inlineStr"/>
-      <c r="E2" s="60" t="inlineStr">
+      <c r="D2" s="61" t="inlineStr"/>
+      <c r="E2" s="61" t="inlineStr">
         <is>
           <t>SFM-FN-001: F1 Lateral control: request steering torque from the EPS to keep the vehicle in its lane while engaged
 SFM-FN-002: F2 Longitudinal control: request acceleration/deceleration to hold set speed and follow leads while engaged
@@ -17535,398 +17547,398 @@
       </c>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="60" t="inlineStr">
+      <c r="A3" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="B3" s="60" t="inlineStr">
+      <c r="B3" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">    comma 3X device</t>
         </is>
       </c>
-      <c r="C3" s="60" t="inlineStr">
+      <c r="C3" s="61" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="D3" s="60" t="inlineStr">
+      <c r="D3" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E3" s="60" t="inlineStr"/>
+      <c r="E3" s="61" t="inlineStr"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="60" t="inlineStr">
+      <c r="A4" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-003</t>
         </is>
       </c>
-      <c r="B4" s="60" t="inlineStr">
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Integrated panda (CAN interface and safety model)</t>
         </is>
       </c>
-      <c r="C4" s="60" t="inlineStr">
+      <c r="C4" s="61" t="inlineStr">
         <is>
           <t>subsystem</t>
         </is>
       </c>
-      <c r="D4" s="60" t="inlineStr">
+      <c r="D4" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E4" s="60" t="inlineStr"/>
+      <c r="E4" s="61" t="inlineStr"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="60" t="inlineStr">
+      <c r="A5" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-004</t>
         </is>
       </c>
-      <c r="B5" s="60" t="inlineStr">
+      <c r="B5" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">    Harness (Toyota A connector, harness box, comma power v3)</t>
         </is>
       </c>
-      <c r="C5" s="60" t="inlineStr">
+      <c r="C5" s="61" t="inlineStr">
         <is>
           <t>component</t>
         </is>
       </c>
-      <c r="D5" s="60" t="inlineStr">
+      <c r="D5" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E5" s="60" t="inlineStr"/>
+      <c r="E5" s="61" t="inlineStr"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-010</t>
         </is>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Perception (camerad, modeld)</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E6" s="60" t="inlineStr"/>
+      <c r="E6" s="61" t="inlineStr"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="60" t="inlineStr">
+      <c r="A7" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-011</t>
         </is>
       </c>
-      <c r="B7" s="60" t="inlineStr">
+      <c r="B7" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Localization and calibration (locationd, calibrationd, paramsd, torqued)</t>
         </is>
       </c>
-      <c r="C7" s="60" t="inlineStr">
+      <c r="C7" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D7" s="60" t="inlineStr">
+      <c r="D7" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E7" s="60" t="inlineStr"/>
+      <c r="E7" s="61" t="inlineStr"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="60" t="inlineStr">
+      <c r="A8" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-012</t>
         </is>
       </c>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="B8" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Planning (plannerd, radard)</t>
         </is>
       </c>
-      <c r="C8" s="60" t="inlineStr">
+      <c r="C8" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D8" s="60" t="inlineStr">
+      <c r="D8" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E8" s="60" t="inlineStr"/>
+      <c r="E8" s="61" t="inlineStr"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="60" t="inlineStr">
+      <c r="A9" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-013</t>
         </is>
       </c>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Control (controlsd, lateral/longitudinal controllers)</t>
         </is>
       </c>
-      <c r="C9" s="60" t="inlineStr">
+      <c r="C9" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D9" s="60" t="inlineStr">
+      <c r="D9" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E9" s="60" t="inlineStr"/>
+      <c r="E9" s="61" t="inlineStr"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="60" t="inlineStr">
+      <c r="A10" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-014</t>
         </is>
       </c>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Supervision (selfdrived state machine, events, alert manager)</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
+      <c r="D10" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E10" s="60" t="inlineStr"/>
+      <c r="E10" s="61" t="inlineStr"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="60" t="inlineStr">
+      <c r="A11" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-015</t>
         </is>
       </c>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Driver monitoring (dmonitoringmodeld, dmonitoringd)</t>
         </is>
       </c>
-      <c r="C11" s="60" t="inlineStr">
+      <c r="C11" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D11" s="60" t="inlineStr">
+      <c r="D11" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E11" s="60" t="inlineStr"/>
+      <c r="E11" s="61" t="inlineStr"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="60" t="inlineStr">
+      <c r="A12" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-016</t>
         </is>
       </c>
-      <c r="B12" s="60" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Car interface (card, car_events, opendbc Toyota port)</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C12" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D12" s="60" t="inlineStr">
+      <c r="D12" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E12" s="60" t="inlineStr"/>
+      <c r="E12" s="61" t="inlineStr"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="60" t="inlineStr">
+      <c r="A13" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-017</t>
         </is>
       </c>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Panda daemon (pandad)</t>
         </is>
       </c>
-      <c r="C13" s="60" t="inlineStr">
+      <c r="C13" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D13" s="60" t="inlineStr">
+      <c r="D13" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E13" s="60" t="inlineStr"/>
+      <c r="E13" s="61" t="inlineStr"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="60" t="inlineStr">
+      <c r="A14" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-018</t>
         </is>
       </c>
-      <c r="B14" s="60" t="inlineStr">
+      <c r="B14" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        HMI (ui, soundd)</t>
         </is>
       </c>
-      <c r="C14" s="60" t="inlineStr">
+      <c r="C14" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D14" s="60" t="inlineStr">
+      <c r="D14" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E14" s="60" t="inlineStr"/>
+      <c r="E14" s="61" t="inlineStr"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="60" t="inlineStr">
+      <c r="A15" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-019</t>
         </is>
       </c>
-      <c r="B15" s="60" t="inlineStr">
+      <c r="B15" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">        Platform (manager, messaging, hardwared, OS)</t>
         </is>
       </c>
-      <c r="C15" s="60" t="inlineStr">
+      <c r="C15" s="61" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D15" s="60" t="inlineStr">
+      <c r="D15" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E15" s="60" t="inlineStr"/>
+      <c r="E15" s="61" t="inlineStr"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="60" t="inlineStr">
+      <c r="A16" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-030</t>
         </is>
       </c>
-      <c r="B16" s="60" t="inlineStr">
+      <c r="B16" s="61" t="inlineStr">
         <is>
           <t>Toyota EPS</t>
         </is>
       </c>
-      <c r="C16" s="60" t="inlineStr">
+      <c r="C16" s="61" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D16" s="60" t="inlineStr"/>
-      <c r="E16" s="60" t="inlineStr"/>
+      <c r="D16" s="61" t="inlineStr"/>
+      <c r="E16" s="61" t="inlineStr"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="60" t="inlineStr">
+      <c r="A17" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-031</t>
         </is>
       </c>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>Toyota powertrain and brake control (receives ACC acceleration requests)</t>
         </is>
       </c>
-      <c r="C17" s="60" t="inlineStr">
+      <c r="C17" s="61" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D17" s="60" t="inlineStr"/>
-      <c r="E17" s="60" t="inlineStr"/>
+      <c r="D17" s="61" t="inlineStr"/>
+      <c r="E17" s="61" t="inlineStr"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="60" t="inlineStr">
+      <c r="A18" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-032</t>
         </is>
       </c>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t>Toyota stock ADAS camera (TSS2)</t>
         </is>
       </c>
-      <c r="C18" s="60" t="inlineStr">
+      <c r="C18" s="61" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D18" s="60" t="inlineStr"/>
-      <c r="E18" s="60" t="inlineStr"/>
+      <c r="D18" s="61" t="inlineStr"/>
+      <c r="E18" s="61" t="inlineStr"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="60" t="inlineStr">
+      <c r="A19" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-033</t>
         </is>
       </c>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t>Vehicle CAN buses and 12 V supply</t>
         </is>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="61" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D19" s="60" t="inlineStr"/>
-      <c r="E19" s="60" t="inlineStr"/>
+      <c r="D19" s="61" t="inlineStr"/>
+      <c r="E19" s="61" t="inlineStr"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="60" t="inlineStr">
+      <c r="A20" s="61" t="inlineStr">
         <is>
           <t>SFM-SE-034</t>
         </is>
       </c>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
+      <c r="C20" s="61" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D20" s="60" t="inlineStr"/>
-      <c r="E20" s="60" t="inlineStr"/>
+      <c r="D20" s="61" t="inlineStr"/>
+      <c r="E20" s="61" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E20"/>
@@ -17962,7 +17974,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>FMEA-MSR (monitoring and system response, msr-plan.md): S, F, M and MSR AP per rating-tables.md §7 (RT-2). The MSR AP table is provisional until the handbook table is transcribed (decision register DQ-207). Exempt causes are rated in the FMEA named in the reason.</t>
         </is>
@@ -20719,7 +20731,7 @@
           <t>Device power loss (12 V interruption, harness connector)</t>
         </is>
       </c>
-      <c r="E44" s="63" t="inlineStr">
+      <c r="E44" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-012.C1)</t>
         </is>
@@ -21732,7 +21744,7 @@
         <v>8</v>
       </c>
       <c r="I60" s="35" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J60" s="35" t="n">
         <v>7</v>
@@ -21841,7 +21853,7 @@
           <t>Panda MCU hardware fault (see DFMEA/FMEDA)</t>
         </is>
       </c>
-      <c r="E62" s="63" t="inlineStr">
+      <c r="E62" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-001.C1)</t>
         </is>
@@ -22001,7 +22013,7 @@
           <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
         </is>
       </c>
-      <c r="E65" s="63" t="inlineStr">
+      <c r="E65" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-010.C1)</t>
         </is>
@@ -22037,7 +22049,7 @@
           <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
         </is>
       </c>
-      <c r="E66" s="63" t="inlineStr">
+      <c r="E66" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-011.C1)</t>
         </is>
@@ -22313,7 +22325,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.15 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.16 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.17: link 17 host-software causes to the SW FMEA P2/P3 rows
The SW FMEA now rates the P2/P3 host elements at BL-005 (#111, #112).
Causes that describe the same fault link to those rows and inherit
their O and D: packer (SWF-059), learned parameters (SWF-076),
calibration (SWF-075), carState decoding (SWF-057), frozen modelV2
(SWF-072), planner (SWF-065), missed lead (SWF-070), DM escalation
(SWF-061) and fingerprint (SWF-058).

O falls on 6 causes and rises on SFM-008.C1; D 8 -> 9 on 11. MSR F
follows O. Every AP stays H. Partial matches are not linked.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.16 · draft</t>
+          <t>0.17 · draft</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       <c r="R4" s="37" t="inlineStr"/>
       <c r="S4" s="37" t="inlineStr"/>
     </row>
-    <row r="5" ht="100.5" customHeight="1">
+    <row r="5" ht="235.5" customHeight="1">
       <c r="A5" s="39" t="n"/>
       <c r="B5" s="39" t="n"/>
       <c r="C5" s="39" t="n"/>
@@ -1650,6 +1650,15 @@
             </rPr>
             <t>Steering message packed with non-zero torque/request bit while latActive is false</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-059</t>
+          </r>
         </is>
       </c>
       <c r="I5" s="41" t="inlineStr">
@@ -1674,7 +1683,7 @@
         </is>
       </c>
       <c r="J5" s="42" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K5" s="41" t="inlineStr">
         <is>
@@ -1684,7 +1693,7 @@
               <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
-            <t>• process_replay over the CI route corpus compares outputs with the reference commit (CI 'process replay'); a regression check, not designed or proven for this cause</t>
+            <t>• As rated in the SW FMEA (SWF-059.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause; it compares sendcan</t>
           </r>
           <r>
             <rPr>
@@ -1695,6 +1704,32 @@
             <t xml:space="preserve">
    openpilot/selfdrive/test/process_replay/test_processes.py</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• process_replay over the CI route corpus compares outputs with the reference commit (CI 'process replay'); a regression check, not designed or proven for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
         </is>
       </c>
       <c r="L5" s="43" t="n">
@@ -1722,7 +1757,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>The panda refuses steering torque while controls are not allowed (SWF-002, D 3), so this cause leads to the end effect only together with SFM-001.C2; no separate action</t>
+            <t>Rated in the SW FMEA (SWF-059.C1, O 4 D 9 at BL-005); this row inherits that rating. The panda refuses steering torque while controls are not allowed (SWF-002, D 3), so this cause leads to the end effect only together with SFM-001.C2; no separate action</t>
           </r>
         </is>
       </c>
@@ -2333,6 +2368,15 @@
             </rPr>
             <t>Wrong vehicle parameters (steer ratio, lateral accel factor, torque offsets) from online learners</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-076</t>
+          </r>
         </is>
       </c>
       <c r="I9" s="41" t="inlineStr">
@@ -2383,17 +2427,17 @@
         </is>
       </c>
       <c r="J9" s="42" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K9" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• paramsd and torqued unit tests (estimate bounds and convergence); targeted, not proven by fault injection</t>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-076.C1, D 9 at BL-005): test_paramsd.py (CI) checks the saved-parameter handling; not designed for out-of-bound use</t>
           </r>
           <r>
             <rPr>
@@ -2404,10 +2448,36 @@
             <t xml:space="preserve">
    openpilot/selfdrive/locationd/test/test_paramsd.py</t>
           </r>
-        </is>
-      </c>
-      <c r="L9" s="42" t="n">
-        <v>8</v>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• paramsd and torqued unit tests (estimate bounds and convergence); targeted, not proven by fault injection</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/locationd/test/test_paramsd.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L9" s="43" t="n">
+        <v>9</v>
       </c>
       <c r="M9" s="44" t="inlineStr">
         <is>
@@ -2666,6 +2736,15 @@
             </rPr>
             <t>Calibration (camera extrinsics) wrong or not converged</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-075</t>
+          </r>
         </is>
       </c>
       <c r="I10" s="34" t="inlineStr">
@@ -2716,10 +2795,36 @@
         </is>
       </c>
       <c r="J10" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K10" s="34" t="inlineStr">
         <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-075.C1, D 8 at BL-005): test_calibrationd.py (CI) checks status transitions on synthetic data; targeted at the thresholds, not proven</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/locationd/test/test_calibrationd.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
           <r>
             <rPr>
               <rFont val="Calibri"/>
@@ -2779,7 +2884,7 @@
       <c r="R10" s="37" t="inlineStr"/>
       <c r="S10" s="37" t="inlineStr"/>
     </row>
-    <row r="11" ht="141" customHeight="1">
+    <row r="11" ht="235.5" customHeight="1">
       <c r="A11" s="38" t="n"/>
       <c r="B11" s="38" t="n"/>
       <c r="C11" s="38" t="n"/>
@@ -2801,6 +2906,15 @@
             </rPr>
             <t>Sign convention error in steering signal parse or pack for this car</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-057</t>
+          </r>
         </is>
       </c>
       <c r="I11" s="34" t="inlineStr">
@@ -2832,7 +2946,33 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-057.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• opendbc car tests check carState against the panda safety model on recorded routes (test_models); targeted at parse and pack consistency, not proven by fault injection, and run only where the route corpus is available</t>
@@ -2848,8 +2988,8 @@
           </r>
         </is>
       </c>
-      <c r="L11" s="35" t="n">
-        <v>8</v>
+      <c r="L11" s="46" t="n">
+        <v>9</v>
       </c>
       <c r="M11" s="36" t="inlineStr">
         <is>
@@ -4323,6 +4463,15 @@
             </rPr>
             <t>modeld output frozen (stale frame) but still published as valid</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-072</t>
+          </r>
         </is>
       </c>
       <c r="I21" s="34" t="inlineStr">
@@ -4373,10 +4522,27 @@
         </is>
       </c>
       <c r="J21" s="35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K21" s="34" t="inlineStr">
         <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-072.C2, D 10 at BL-005): modeld has no unit tests, is excluded from process replay (EXCLUDED_PROCS) and from test_fuzzy, and model_replay is not run in LionDriver CI; test_onroad timing checks are device-only</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
           <r>
             <rPr>
               <rFont val="Calibri"/>
@@ -4921,7 +5087,7 @@
       <c r="R24" s="45" t="inlineStr"/>
       <c r="S24" s="45" t="inlineStr"/>
     </row>
-    <row r="25" ht="181.5" customHeight="1">
+    <row r="25" ht="195" customHeight="1">
       <c r="A25" s="30" t="inlineStr">
         <is>
           <r>
@@ -5085,6 +5251,15 @@
             </rPr>
             <t>Planner targets higher speed (missed lead, wrong set speed)</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-065</t>
+          </r>
         </is>
       </c>
       <c r="I25" s="34" t="inlineStr">
@@ -5135,14 +5310,40 @@
         </is>
       </c>
       <c r="J25" s="35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K25" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-065.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• Unit test of the longitudinal plan's following distance and set-speed behaviour; targeted, not proven</t>
@@ -5158,8 +5359,8 @@
           </r>
         </is>
       </c>
-      <c r="L25" s="35" t="n">
-        <v>8</v>
+      <c r="L25" s="46" t="n">
+        <v>9</v>
       </c>
       <c r="M25" s="36" t="inlineStr">
         <is>
@@ -5344,7 +5545,7 @@
       <c r="R26" s="37" t="inlineStr"/>
       <c r="S26" s="37" t="inlineStr"/>
     </row>
-    <row r="27" ht="181.5" customHeight="1">
+    <row r="27" ht="249" customHeight="1">
       <c r="A27" s="38" t="n"/>
       <c r="B27" s="38" t="n"/>
       <c r="C27" s="38" t="n"/>
@@ -5366,6 +5567,15 @@
             </rPr>
             <t>Wrong scaling of acceleration request for this car</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-059</t>
+          </r>
         </is>
       </c>
       <c r="I27" s="34" t="inlineStr">
@@ -5416,14 +5626,40 @@
         </is>
       </c>
       <c r="J27" s="35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K27" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-059.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause; it compares sendcan</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• opendbc car tests check carState against the panda safety model on recorded routes (test_models); targeted at parse and pack consistency, not proven by fault injection, and run only where the route corpus is available</t>
@@ -5439,8 +5675,8 @@
           </r>
         </is>
       </c>
-      <c r="L27" s="35" t="n">
-        <v>8</v>
+      <c r="L27" s="46" t="n">
+        <v>9</v>
       </c>
       <c r="M27" s="36" t="inlineStr">
         <is>
@@ -5965,7 +6201,7 @@
       <c r="R30" s="37" t="inlineStr"/>
       <c r="S30" s="37" t="inlineStr"/>
     </row>
-    <row r="31" ht="141" customHeight="1">
+    <row r="31" ht="235.5" customHeight="1">
       <c r="A31" s="39" t="n"/>
       <c r="B31" s="39" t="n"/>
       <c r="C31" s="39" t="n"/>
@@ -5987,6 +6223,15 @@
             </rPr>
             <t>Wrong vEgo/aEgo from CAN parse</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-057</t>
+          </r>
         </is>
       </c>
       <c r="I31" s="41" t="inlineStr">
@@ -6018,7 +6263,33 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-057.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• opendbc car tests check carState against the panda safety model on recorded routes (test_models); targeted at parse and pack consistency, not proven by fault injection, and run only where the route corpus is available</t>
@@ -6034,8 +6305,8 @@
           </r>
         </is>
       </c>
-      <c r="L31" s="42" t="n">
-        <v>8</v>
+      <c r="L31" s="43" t="n">
+        <v>9</v>
       </c>
       <c r="M31" s="44" t="inlineStr">
         <is>
@@ -6238,6 +6509,15 @@
             </rPr>
             <t>Lead missed due to radar/vision fusion fault</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-070</t>
+          </r>
         </is>
       </c>
       <c r="I32" s="34" t="inlineStr">
@@ -6292,6 +6572,32 @@
       </c>
       <c r="K32" s="34" t="inlineStr">
         <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-070.C1, D 8 at BL-005): test_stopped_vehicle test_radar_only_stationary_target reproduces the gap and is marked expectedFailure (CI)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/stopped_vehicle/test_stopped_vehicle.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
           <r>
             <rPr>
               <rFont val="Calibri"/>
@@ -9059,7 +9365,7 @@
       <c r="R48" s="45" t="inlineStr"/>
       <c r="S48" s="45" t="inlineStr"/>
     </row>
-    <row r="49" ht="141" customHeight="1">
+    <row r="49" ht="235.5" customHeight="1">
       <c r="A49" s="30" t="inlineStr">
         <is>
           <r>
@@ -9223,6 +9529,15 @@
             </rPr>
             <t>brakePressed parsed wrong or CAN signal missing</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-057</t>
+          </r>
         </is>
       </c>
       <c r="I49" s="34" t="inlineStr">
@@ -9254,7 +9569,33 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-057.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• opendbc car tests check carState against the panda safety model on recorded routes (test_models); targeted at parse and pack consistency, not proven by fault injection, and run only where the route corpus is available</t>
@@ -9270,8 +9611,8 @@
           </r>
         </is>
       </c>
-      <c r="L49" s="35" t="n">
-        <v>8</v>
+      <c r="L49" s="46" t="n">
+        <v>9</v>
       </c>
       <c r="M49" s="36" t="inlineStr">
         <is>
@@ -9423,7 +9764,7 @@
       <c r="R50" s="45" t="inlineStr"/>
       <c r="S50" s="45" t="inlineStr"/>
     </row>
-    <row r="51" ht="141" customHeight="1">
+    <row r="51" ht="235.5" customHeight="1">
       <c r="A51" s="30" t="inlineStr">
         <is>
           <r>
@@ -9587,6 +9928,15 @@
             </rPr>
             <t>Driver torque threshold too high or signal parsed wrong</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-057</t>
+          </r>
         </is>
       </c>
       <c r="I51" s="34" t="inlineStr">
@@ -9618,7 +9968,33 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-057.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• opendbc car tests check carState against the panda safety model on recorded routes (test_models); targeted at parse and pack consistency, not proven by fault injection, and run only where the route corpus is available</t>
@@ -9634,8 +10010,8 @@
           </r>
         </is>
       </c>
-      <c r="L51" s="35" t="n">
-        <v>8</v>
+      <c r="L51" s="46" t="n">
+        <v>9</v>
       </c>
       <c r="M51" s="36" t="inlineStr">
         <is>
@@ -9787,7 +10163,7 @@
       <c r="R52" s="45" t="inlineStr"/>
       <c r="S52" s="45" t="inlineStr"/>
     </row>
-    <row r="53" ht="141" customHeight="1">
+    <row r="53" ht="235.5" customHeight="1">
       <c r="A53" s="51" t="inlineStr">
         <is>
           <r>
@@ -9951,6 +10327,15 @@
             </rPr>
             <t>Button message parsed wrong or missing</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-057</t>
+          </r>
         </is>
       </c>
       <c r="I53" s="41" t="inlineStr">
@@ -9982,7 +10367,33 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-057.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• opendbc car tests check carState against the panda safety model on recorded routes (test_models); targeted at parse and pack consistency, not proven by fault injection, and run only where the route corpus is available</t>
@@ -9998,8 +10409,8 @@
           </r>
         </is>
       </c>
-      <c r="L53" s="42" t="n">
-        <v>8</v>
+      <c r="L53" s="43" t="n">
+        <v>9</v>
       </c>
       <c r="M53" s="44" t="inlineStr">
         <is>
@@ -10038,7 +10449,7 @@
       <c r="R53" s="45" t="inlineStr"/>
       <c r="S53" s="45" t="inlineStr"/>
     </row>
-    <row r="54" ht="141" customHeight="1">
+    <row r="54" ht="235.5" customHeight="1">
       <c r="A54" s="51" t="inlineStr">
         <is>
           <r>
@@ -10202,6 +10613,15 @@
             </rPr>
             <t>gasPressed parsed wrong or missing</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-057</t>
+          </r>
         </is>
       </c>
       <c r="I54" s="41" t="inlineStr">
@@ -10233,7 +10653,33 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-057.C1, D 9 at BL-005): process_replay (CI) replays the TOYOTA3 Corolla TSS2 segment and compares with reference logs made from the same code, so it cannot find a defect already present at the baseline; not designed for this cause</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/process_replay/test_processes.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• opendbc car tests check carState against the panda safety model on recorded routes (test_models); targeted at parse and pack consistency, not proven by fault injection, and run only where the route corpus is available</t>
@@ -10249,8 +10695,8 @@
           </r>
         </is>
       </c>
-      <c r="L54" s="42" t="n">
-        <v>8</v>
+      <c r="L54" s="43" t="n">
+        <v>9</v>
       </c>
       <c r="M54" s="44" t="inlineStr">
         <is>
@@ -10873,7 +11319,7 @@
       <c r="R57" s="37" t="inlineStr"/>
       <c r="S57" s="37" t="inlineStr"/>
     </row>
-    <row r="58" ht="100.5" customHeight="1">
+    <row r="58" ht="195" customHeight="1">
       <c r="A58" s="38" t="n"/>
       <c r="B58" s="38" t="n"/>
       <c r="C58" s="38" t="n"/>
@@ -10895,6 +11341,15 @@
             </rPr>
             <t>Pose thresholds/calibration wrong for driver or mount</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-061</t>
+          </r>
         </is>
       </c>
       <c r="I58" s="34" t="inlineStr">
@@ -10923,6 +11378,32 @@
       </c>
       <c r="K58" s="34" t="inlineStr">
         <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-061.C2, D 8 at BL-005): test_monitoring.py scenarios (distracted, invisible, uncertain, last-second responder) in CI; targeted at the policy, not proven by mutation</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/monitoring/test_monitoring.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
           <r>
             <rPr>
               <rFont val="Calibri"/>
@@ -11108,7 +11589,7 @@
       <c r="R59" s="45" t="inlineStr"/>
       <c r="S59" s="45" t="inlineStr"/>
     </row>
-    <row r="60" ht="100.5" customHeight="1">
+    <row r="60" ht="195" customHeight="1">
       <c r="A60" s="30" t="inlineStr">
         <is>
           <r>
@@ -11272,6 +11753,15 @@
             </rPr>
             <t>Policy timers or recovery factor misconfigured</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-061</t>
+          </r>
         </is>
       </c>
       <c r="I60" s="34" t="inlineStr">
@@ -11300,6 +11790,32 @@
       </c>
       <c r="K60" s="34" t="inlineStr">
         <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-061.C2, D 8 at BL-005): test_monitoring.py scenarios (distracted, invisible, uncertain, last-second responder) in CI; targeted at the policy, not proven by mutation</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/monitoring/test_monitoring.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
           <r>
             <rPr>
               <rFont val="Calibri"/>
@@ -11359,7 +11875,7 @@
       <c r="R60" s="37" t="inlineStr"/>
       <c r="S60" s="37" t="inlineStr"/>
     </row>
-    <row r="61" ht="100.5" customHeight="1">
+    <row r="61" ht="181.5" customHeight="1">
       <c r="A61" s="39" t="n"/>
       <c r="B61" s="39" t="n"/>
       <c r="C61" s="39" t="n"/>
@@ -11381,6 +11897,15 @@
             </rPr>
             <t>Low-speed or always-on exemption applied incorrectly</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-061</t>
+          </r>
         </is>
       </c>
       <c r="I61" s="41" t="inlineStr">
@@ -11412,10 +11937,10 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• Driver-monitoring policy unit tests (alert timing, awareness recovery, exemptions) on synthetic inputs; targeted, not proven by fault injection; the model itself is not tested</t>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-061.C3, D 9 at BL-005): test_monitoring.py covers the wheel-touch fallback; not designed for this cause</t>
           </r>
           <r>
             <rPr>
@@ -11426,10 +11951,36 @@
             <t xml:space="preserve">
    openpilot/selfdrive/monitoring/test_monitoring.py</t>
           </r>
-        </is>
-      </c>
-      <c r="L61" s="42" t="n">
-        <v>8</v>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Driver-monitoring policy unit tests (alert timing, awareness recovery, exemptions) on synthetic inputs; targeted, not proven by fault injection; the model itself is not tested</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/monitoring/test_monitoring.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L61" s="43" t="n">
+        <v>9</v>
       </c>
       <c r="M61" s="44" t="inlineStr">
         <is>
@@ -14733,6 +15284,15 @@
             </rPr>
             <t>Fuzzy fingerprint matches a similar platform</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-058</t>
+          </r>
         </is>
       </c>
       <c r="I78" s="41" t="inlineStr">
@@ -14783,14 +15343,31 @@
         </is>
       </c>
       <c r="J78" s="42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K78" s="41" t="inlineStr">
         <is>
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-058.C1, D 9 at BL-005): opendbc test_fw_fingerprint exists but is not run by LionDriver CI</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
             <t>• Fingerprinting unit tests (FW and CAN fingerprint); targeted, not proven by fault injection</t>
@@ -14806,8 +15383,8 @@
           </r>
         </is>
       </c>
-      <c r="L78" s="42" t="n">
-        <v>8</v>
+      <c r="L78" s="43" t="n">
+        <v>9</v>
       </c>
       <c r="M78" s="44" t="inlineStr">
         <is>
@@ -16653,7 +17230,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.16 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.17 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -18229,7 +18806,7 @@
         <v>4</v>
       </c>
       <c r="I5" s="35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J5" s="35" t="n">
         <v>5</v>
@@ -18496,7 +19073,7 @@
         <v>10</v>
       </c>
       <c r="I9" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" s="35" t="n">
         <v>5</v>
@@ -18563,7 +19140,7 @@
         <v>10</v>
       </c>
       <c r="I10" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" s="46" t="n">
         <v>10</v>
@@ -19274,7 +19851,7 @@
         <v>10</v>
       </c>
       <c r="I21" s="35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J21" s="46" t="n">
         <v>9</v>
@@ -19398,7 +19975,7 @@
         <v>10</v>
       </c>
       <c r="I23" s="35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J23" s="46" t="n">
         <v>9</v>
@@ -19528,7 +20105,7 @@
         <v>10</v>
       </c>
       <c r="I25" s="35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J25" s="35" t="n">
         <v>5</v>
@@ -21966,7 +22543,7 @@
         <v>10</v>
       </c>
       <c r="I64" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J64" s="35" t="n">
         <v>8</v>
@@ -22325,7 +22902,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.16 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.17 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.18: link SFM-025.C1 to SWF-062.C1
The SW FMEA now rates the driver-monitoring terminal-state design gap
at O 8 (#144), the same as the System FMEA. SFM-025.C1 links to it
and takes its detection: D 10 -> 9 (test_longitudinal and
test_monitoring run in CI, not designed for FSR-040). O 8 and AP H
unchanged. fmea-plan v0.15.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.17 · draft</t>
+          <t>0.18 · draft</t>
         </is>
       </c>
     </row>
@@ -12416,6 +12416,15 @@
             </rPr>
             <t>driverDistracted3 / driverUnresponsive3 mapped only to ET.PERMANENT (no disable reaction)</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-062</t>
+          </r>
         </is>
       </c>
       <c r="I63" s="41" t="inlineStr">
@@ -12450,6 +12459,32 @@
               <color rgb="008A5A00"/>
               <sz val="10"/>
             </rPr>
+            <t>• As rated in the SW FMEA (SWF-062.C1, D 9 at BL-005): test_longitudinal runs the force_decel maneuver in CI and test_monitoring checks the alert levels; neither checks that the reaction meets FSR-040</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/test/longitudinal_maneuvers/test_longitudinal.py</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
             <t>• Present by design and known; no test, because no requirement says what the reaction should be</t>
           </r>
           <r>
@@ -12464,7 +12499,7 @@
         </is>
       </c>
       <c r="L63" s="43" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M63" s="44" t="inlineStr">
         <is>
@@ -17230,7 +17265,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.17 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.18 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -22902,7 +22937,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.17 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.18 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.19: steering-override and N-3 simulation evidence
WP-S-04 v0.11 §3.9 (#145) adds two simulation results that bear on
System FMEA rows. Both are cited as MSR evidence with no rating credit
(msr-plan §4.2):
- SFM-018.C1/C2 (driver override): the host drops LKA within the 0.2 s
  SG-05 budget in 18 of 36 runs and never in 8 (override-l2.md).
- SFM-004.C1-C3 (insufficient lateral control): N-3 saturates at the
  ODD curve bound and reaches the 3.0 m lane line after 4.09 s.
No rating changes. fmea-plan v0.16.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.18 · draft</t>
+          <t>0.19 · draft</t>
         </is>
       </c>
     </row>
@@ -17265,7 +17265,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.18 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.19 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -22937,7 +22937,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.18 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.19 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.20: HZ-013 end effects on SFM-026 and SFM-027
The driver-monitoring escalation goes through the same HMI path as the
take-over alerts, so a missing (SFM-026) or late or masked (SFM-027)
alert also contributes to HZ-013, as SWF-082 and SWF-035 now say
(#146). HARA HZ-013 sfm_refs gain both; FTA finding F-37 marked
resolved for the System FMEA part. Severity stays 10; no rating
changes. Based on liondriver-dev, independent of #149 and #150.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.17 · draft</t>
+          <t>0.20 · draft</t>
         </is>
       </c>
     </row>
@@ -12609,6 +12609,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-013: driver-monitoring escalation alerts not shown or played, so an inattentive driver is not told; the forced deceleration does not depend on them (as SWF-082)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -12650,7 +12676,8 @@
       <c r="D64" s="31" t="inlineStr">
         <is>
           <t>HZ-012
-HZ-006</t>
+HZ-006
+HZ-013</t>
         </is>
       </c>
       <c r="E64" s="32" t="n">
@@ -13115,6 +13142,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-013: a driver-monitoring escalation presented late, or hidden behind a higher-priority alert, so the inattentive driver is told late (as SWF-035)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -13155,7 +13208,8 @@
       </c>
       <c r="D67" s="31" t="inlineStr">
         <is>
-          <t>HZ-012</t>
+          <t>HZ-012
+HZ-013</t>
         </is>
       </c>
       <c r="E67" s="32" t="n">
@@ -17230,7 +17284,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.17 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -22902,7 +22956,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.17 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Regenerate the FMEA review README, figure 4-1 and the System FMEA workbook after merging #149 and liondriver-dev
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.18 · draft</t>
+          <t>0.19 · draft</t>
         </is>
       </c>
     </row>
@@ -17265,7 +17265,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.18 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.19 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -22937,7 +22937,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.18 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.19 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.21: hazard end effects the fault trees rely on
The fta-fmea-map linter warned that SG-03 and SG-05 cite System FMEA
modes whose effects did not name the goal's hazard. Where the effect is
real, it is added:
- HZ-005: SFM-013 (unintended engagement), SFM-017 (brake does not
  disengage), SFM-034 (intercept in pass-through).
- HZ-008: SFM-021 (stock cruise survives the cancel), SFM-028
  (displayed state says released).
HARA sfm_refs updated. Severity stays 10; no rating changes.
SFM-005 (SG-06), SFM-006 (SG-03) and SFM-020 (SG-05) are tree mapping
questions for the FTA owner and are not changed here.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.20 · draft</t>
+          <t>0.21 · draft</t>
         </is>
       </c>
     </row>
@@ -7633,6 +7633,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-005: positive acceleration requested after an engagement the driver did not ask for</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -7673,7 +7699,8 @@
       </c>
       <c r="D39" s="31" t="inlineStr">
         <is>
-          <t>HZ-010</t>
+          <t>HZ-010
+HZ-005</t>
         </is>
       </c>
       <c r="E39" s="32" t="n">
@@ -9445,6 +9472,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-005: the item keeps requesting acceleration while the driver brakes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -9485,7 +9538,8 @@
       </c>
       <c r="D49" s="31" t="inlineStr">
         <is>
-          <t>HZ-008</t>
+          <t>HZ-008
+HZ-005</t>
         </is>
       </c>
       <c r="E49" s="32" t="n">
@@ -10815,6 +10869,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-008: the driver cancels but stock cruise keeps longitudinal control</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -10855,7 +10935,8 @@
       </c>
       <c r="D55" s="31" t="inlineStr">
         <is>
-          <t>HZ-012</t>
+          <t>HZ-012
+HZ-008</t>
         </is>
       </c>
       <c r="E55" s="32" t="n">
@@ -13524,6 +13605,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-008: the driver believes control was released by the brake or cancel while the item still acts</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -13564,7 +13671,8 @@
       </c>
       <c r="D69" s="31" t="inlineStr">
         <is>
-          <t>HZ-012</t>
+          <t>HZ-012
+HZ-008</t>
         </is>
       </c>
       <c r="E69" s="32" t="n">
@@ -16087,6 +16195,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-005: stock ACC and item acceleration requests combine on the bus</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -16129,7 +16263,8 @@
         <is>
           <t>HZ-011
 HZ-002
-HZ-006</t>
+HZ-006
+HZ-005</t>
         </is>
       </c>
       <c r="E82" s="32" t="n">
@@ -16264,7 +16399,7 @@
       <c r="R82" s="37" t="inlineStr"/>
       <c r="S82" s="37" t="inlineStr"/>
     </row>
-    <row r="83" ht="102" customHeight="1">
+    <row r="83" ht="142.5" customHeight="1">
       <c r="A83" s="39" t="n"/>
       <c r="B83" s="39" t="n"/>
       <c r="C83" s="39" t="n"/>
@@ -17284,7 +17419,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.21 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -22956,7 +23091,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.21 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.22: SFM-037, longitudinal command frozen at last value
The counterpart of SFM-006 that the SG-03 tree lacked (fta-fmea-map
BE-1.19 note: no System FMEA mode for a frozen longitudinal request).
End effects HZ-005 and HZ-007.
- C1 controlsd hangs (SWF-047.C1, O 6 D 10): panda revokes within
  0.11 s of the last ACC_CONTROL (TSR-408), but the PCM reaction to
  missing frames is unknown: M 7.
- C2 plannerd stops (SWF-068.C1, O 4 D 9): 0.5 s liveness plus 3 s
  soft disable exceeds the 1 s FTTI: M 8.
- C3 stale data with fresh timestamps (O 5 D 10): M 9.
All AP H; existing actions SFM-ACT-002 and SFM-ACT-015. HARA sfm_refs
updated; not_in_fta tree_gap rows for SG-03 and SG-06 for the FTA owner.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$90</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$73</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.21 · draft</t>
+          <t>0.22 · draft</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16">
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17">
@@ -964,7 +964,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>64 rated, 4 exempt; MSR AP H 64, M 0, L 0 (provisional table)</t>
+          <t>67 rated, 4 exempt; MSR AP H 67, M 0, L 0 (provisional table)</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>1–4: 0 · 5–6: 18 · 7–8: 15 · 9–10: 31 (see sheet MSR)</t>
+          <t>1–4: 0 · 5–6: 18 · 7–8: 17 · 9–10: 32 (see sheet MSR)</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S87"/>
+  <dimension ref="A1:S90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17222,9 +17222,496 @@
       <c r="R87" s="45" t="inlineStr"/>
       <c r="S87" s="45" t="inlineStr"/>
     </row>
+    <row r="88" ht="100.5" customHeight="1">
+      <c r="A88" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-SE-001
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B88" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-FN-002
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>F2 Longitudinal control: request acceleration/deceleration to hold set speed and follow leads while engaged</t>
+          </r>
+        </is>
+      </c>
+      <c r="C88" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Unintended acceleration when the frozen request is positive</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Insufficient deceleration when the lead brakes and the frozen request is not braking</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Vehicle holds a constant acceleration or deceleration request</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Same acceleration request repeated regardless of lead, set speed or road</t>
+          </r>
+        </is>
+      </c>
+      <c r="D88" s="31" t="inlineStr">
+        <is>
+          <t>HZ-005
+HZ-007</t>
+        </is>
+      </c>
+      <c r="E88" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F88" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-037 · stuck
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Longitudinal command frozen at last value</t>
+          </r>
+        </is>
+      </c>
+      <c r="G88" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H88" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>controlsd hangs while card keeps sending the last carControl</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-047</t>
+          </r>
+        </is>
+      </c>
+      <c r="I88" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream review, ruff, ty; rated in the SW FMEA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/08-analyses/fmea/analyses/sw-fmea.yaml</t>
+          </r>
+        </is>
+      </c>
+      <c r="J88" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="K88" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-047.C1, D 10 at BL-005): no test injects the exception that stops controlsd</t>
+          </r>
+        </is>
+      </c>
+      <c r="L88" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="M88" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N88" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-002 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O88" s="47" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P88" s="33" t="inlineStr"/>
+      <c r="Q88" s="33" t="inlineStr"/>
+      <c r="R88" s="37" t="inlineStr"/>
+      <c r="S88" s="37" t="inlineStr"/>
+    </row>
+    <row r="89" ht="100.5" customHeight="1">
+      <c r="A89" s="38" t="n"/>
+      <c r="B89" s="38" t="n"/>
+      <c r="C89" s="38" t="n"/>
+      <c r="D89" s="38" t="n"/>
+      <c r="E89" s="38" t="n"/>
+      <c r="F89" s="38" t="n"/>
+      <c r="G89" s="33" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H89" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>plannerd stops or runs late while engaged, so controlsd keeps using the last longitudinalPlan</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-068</t>
+          </r>
+        </is>
+      </c>
+      <c r="I89" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream openpilot code with upstream review; rated in the SW FMEA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/08-analyses/fmea/analyses/sw-fmea.yaml</t>
+          </r>
+        </is>
+      </c>
+      <c r="J89" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="K89" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• As rated in the SW FMEA (SWF-068.C1, D 9 at BL-005): no test targets an exception in the planner loop</t>
+          </r>
+        </is>
+      </c>
+      <c r="L89" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="M89" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N89" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-002 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O89" s="47" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P89" s="33" t="inlineStr"/>
+      <c r="Q89" s="33" t="inlineStr"/>
+      <c r="R89" s="37" t="inlineStr"/>
+      <c r="S89" s="37" t="inlineStr"/>
+    </row>
+    <row r="90" ht="100.5" customHeight="1">
+      <c r="A90" s="39" t="n"/>
+      <c r="B90" s="39" t="n"/>
+      <c r="C90" s="39" t="n"/>
+      <c r="D90" s="39" t="n"/>
+      <c r="E90" s="39" t="n"/>
+      <c r="F90" s="39" t="n"/>
+      <c r="G90" s="40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="H90" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Messaging delivers a stale longitudinal plan or command with fresh timestamps</t>
+          </r>
+        </is>
+      </c>
+      <c r="I90" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• msgq/cereal stamp logMonoTime at publication; SubMaster tracks arrival time and frequency</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/cereal/messaging/__init__.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="J90" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K90" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No pre-release test targets this cause</t>
+          </r>
+        </is>
+      </c>
+      <c r="L90" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="M90" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N90" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-002 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
+          </r>
+        </is>
+      </c>
+      <c r="O90" s="48" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P90" s="40" t="inlineStr"/>
+      <c r="Q90" s="40" t="inlineStr"/>
+      <c r="R90" s="45" t="inlineStr"/>
+      <c r="S90" s="45" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S87"/>
-  <mergeCells count="184">
+  <autoFilter ref="A2:S90"/>
+  <mergeCells count="190">
     <mergeCell ref="F84:F85"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="E39:E40"/>
@@ -17272,6 +17759,7 @@
     <mergeCell ref="F41:F43"/>
     <mergeCell ref="D10:D13"/>
     <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B88:B90"/>
     <mergeCell ref="F10:F13"/>
     <mergeCell ref="D49:D50"/>
     <mergeCell ref="E55:E56"/>
@@ -17291,6 +17779,7 @@
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="B84:B85"/>
     <mergeCell ref="C51:C52"/>
+    <mergeCell ref="A88:A90"/>
     <mergeCell ref="C60:C61"/>
     <mergeCell ref="C64:C66"/>
     <mergeCell ref="D25:D28"/>
@@ -17303,6 +17792,8 @@
     <mergeCell ref="C79:C81"/>
     <mergeCell ref="I1:M1"/>
     <mergeCell ref="E79:E81"/>
+    <mergeCell ref="C88:C90"/>
+    <mergeCell ref="E88:E90"/>
     <mergeCell ref="D39:D40"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="A3:A5"/>
@@ -17384,6 +17875,8 @@
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="B32:B34"/>
     <mergeCell ref="D79:D81"/>
+    <mergeCell ref="D88:D90"/>
+    <mergeCell ref="F88:F90"/>
     <mergeCell ref="C67:C68"/>
     <mergeCell ref="E17:E19"/>
     <mergeCell ref="D71:D74"/>
@@ -17411,7 +17904,7 @@
     <mergeCell ref="D84:D85"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87 R88 R89 R90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17419,7 +17912,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.21 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.22 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -17538,7 +18031,7 @@
       <c r="H2" s="61" t="inlineStr"/>
       <c r="I2" s="61" t="inlineStr"/>
     </row>
-    <row r="3" ht="127.5" customHeight="1">
+    <row r="3" ht="168" customHeight="1">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-002</t>
@@ -17574,7 +18067,10 @@
 SFM-008.C1
 SFM-023.C1
 SFM-023.C2
-SFM-030.C1</t>
+SFM-030.C1
+SFM-037.C1
+SFM-037.C2
+SFM-037.C3</t>
         </is>
       </c>
       <c r="G3" s="61" t="inlineStr"/>
@@ -18718,7 +19214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -23077,13 +23573,208 @@
       <c r="O70" s="37" t="inlineStr"/>
       <c r="P70" s="37" t="inlineStr"/>
     </row>
+    <row r="71" ht="100.5" customHeight="1">
+      <c r="A71" s="34" t="inlineStr">
+        <is>
+          <t>SFM-037 · Longitudinal command frozen at last value</t>
+        </is>
+      </c>
+      <c r="B71" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C71" s="33" t="inlineStr">
+        <is>
+          <t>SFM-037.C1</t>
+        </is>
+      </c>
+      <c r="D71" s="34" t="inlineStr">
+        <is>
+          <t>controlsd hangs while card keeps sending the last carControl</t>
+        </is>
+      </c>
+      <c r="E71" s="34" t="inlineStr">
+        <is>
+          <t>card stops sending once carControl is 0.1 s old (T-13); the panda then revokes authority within 0.11 s of the last ACC_CONTROL frame (TSR-408, T-34) and selfdrived raises controlsMismatch within 0.5 s (TSR-621)</t>
+        </is>
+      </c>
+      <c r="F71" s="34" t="inlineStr">
+        <is>
+          <t>controlsMismatch IMMEDIATE_DISABLE with alert; no ACC_CONTROL frame follows the stall and there is no active zero request (TSR-109), so what the PCM does with the last request after the frames stop is not known (AOU, not measured)</t>
+        </is>
+      </c>
+      <c r="G71" s="34" t="inlineStr">
+        <is>
+          <t>Last request held about 0.2 s, then frames stop; the PCM reaction to missing ACC_CONTROL is not established</t>
+        </is>
+      </c>
+      <c r="H71" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I71" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="J71" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="K71" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L71" s="34" t="inlineStr">
+        <is>
+          <t>SG-03/04 · 1000 ms</t>
+        </is>
+      </c>
+      <c r="M71" s="33" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N71" s="34" t="inlineStr">
+        <is>
+          <t>SFM-ACT-015 · in progress</t>
+        </is>
+      </c>
+      <c r="O71" s="37" t="inlineStr"/>
+      <c r="P71" s="37" t="inlineStr"/>
+    </row>
+    <row r="72" ht="46.5" customHeight="1">
+      <c r="A72" s="34" t="inlineStr">
+        <is>
+          <t>SFM-037 · Longitudinal command frozen at last value</t>
+        </is>
+      </c>
+      <c r="B72" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C72" s="33" t="inlineStr">
+        <is>
+          <t>SFM-037.C2</t>
+        </is>
+      </c>
+      <c r="D72" s="34" t="inlineStr">
+        <is>
+          <t>plannerd stops or runs late while engaged, so controlsd keeps using the last longitudinalPlan</t>
+        </is>
+      </c>
+      <c r="E72" s="34" t="inlineStr">
+        <is>
+          <t>selfdrived liveness check on longitudinalPlan (10 missed periods at 20 Hz, 0.5 s, T-14)</t>
+        </is>
+      </c>
+      <c r="F72" s="34" t="inlineStr">
+        <is>
+          <t>commIssue SOFT_DISABLE; actuation continues for the 3 s countdown (T-16) on the last plan</t>
+        </is>
+      </c>
+      <c r="G72" s="34" t="inlineStr">
+        <is>
+          <t>Frozen request held up to about 3.5 s before the item disengages</t>
+        </is>
+      </c>
+      <c r="H72" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I72" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="J72" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K72" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L72" s="34" t="inlineStr">
+        <is>
+          <t>SG-03/04 · 1000 ms
+500 + 3000 ms</t>
+        </is>
+      </c>
+      <c r="M72" s="33" t="inlineStr">
+        <is>
+          <t>code derived</t>
+        </is>
+      </c>
+      <c r="N72" s="34" t="inlineStr">
+        <is>
+          <t>SFM-ACT-015 · in progress</t>
+        </is>
+      </c>
+      <c r="O72" s="37" t="inlineStr"/>
+      <c r="P72" s="37" t="inlineStr"/>
+    </row>
+    <row r="73" ht="46.5" customHeight="1">
+      <c r="A73" s="34" t="inlineStr">
+        <is>
+          <t>SFM-037 · Longitudinal command frozen at last value</t>
+        </is>
+      </c>
+      <c r="B73" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C73" s="33" t="inlineStr">
+        <is>
+          <t>SFM-037.C3</t>
+        </is>
+      </c>
+      <c r="D73" s="34" t="inlineStr">
+        <is>
+          <t>Messaging delivers a stale longitudinal plan or command with fresh timestamps</t>
+        </is>
+      </c>
+      <c r="E73" s="34" t="inlineStr">
+        <is>
+          <t>Liveness checks use arrival and timestamps, so stale data with fresh timestamps passes them</t>
+        </is>
+      </c>
+      <c r="F73" s="34" t="inlineStr">
+        <is>
+          <t>None until another check trips</t>
+        </is>
+      </c>
+      <c r="G73" s="34" t="inlineStr">
+        <is>
+          <t>Unchanged: longitudinal control acts on stale data</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I73" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="J73" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="K73" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L73" s="34" t="inlineStr"/>
+      <c r="M73" s="33" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N73" s="34" t="inlineStr">
+        <is>
+          <t>SFM-ACT-015 · in progress</t>
+        </is>
+      </c>
+      <c r="O73" s="37" t="inlineStr"/>
+      <c r="P73" s="37" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:P70"/>
+  <autoFilter ref="A2:P73"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O67 O68 O69 O70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
+    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O67 O68 O69 O70 O71 O72 O73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -23091,7 +23782,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.21 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.22 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.23: SFM-038, lateral-control warning late, silent or missing
Backs FTA SG-02 BE-2.08 and BE-2.24, which had no FMEA mode (F-28):
- C1: a temporary EPS fault within 1.5 s of driver steering raises
  only the silent steerTempUnavailableSilent warning, latched while
  the fault lasts (car_events.py:162-177; GAP-03).
- C2: pandad publishes epsFault and requestsRejected, but no SoC
  process reads them (txRateExceeded is read, TSR-615).
- C3: steerSaturated conditions make the warning late for a gradual
  deficit (selfdrived.py:465-479, WP-S-04 §3.8.1).
O 8 (design gaps), AP H; msr_exempt, since the warning timing is
rated in the MSR rows of SFM-004 and SFM-005. New SFM-ACT-023; C3 uses
SFM-ACT-021. HARA HZ-004 sfm_refs and the two FTA events updated.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$93</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$76</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.22 · draft</t>
+          <t>0.23 · draft</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16">
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17">
@@ -952,7 +952,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>21 (19)</t>
+          <t>22 (20)</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>67 rated, 4 exempt; MSR AP H 67, M 0, L 0 (provisional table)</t>
+          <t>67 rated, 7 exempt; MSR AP H 67, M 0, L 0 (provisional table)</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S90"/>
+  <dimension ref="A1:S93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17709,9 +17709,460 @@
       <c r="R90" s="45" t="inlineStr"/>
       <c r="S90" s="45" t="inlineStr"/>
     </row>
+    <row r="91" ht="114" customHeight="1">
+      <c r="A91" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-SE-001
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B91" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-FN-006
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>F6 Alerting: inform the driver of engagement state, takeover requests and faults (visual and audible)</t>
+          </r>
+        </is>
+      </c>
+      <c r="C91" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Driver unaware of the loss or limit; lane departure</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Driver not prompted to take over while lateral control is lost or limited</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>steerTempUnavailable shown silently, steerSaturated raised late or not at all, or the panda's EPS-fault flag not acted on</t>
+          </r>
+        </is>
+      </c>
+      <c r="D91" s="31" t="inlineStr">
+        <is>
+          <t>HZ-004</t>
+        </is>
+      </c>
+      <c r="E91" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F91" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-038 · late
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Warning of a lateral-control fault or limit late, silent or missing</t>
+          </r>
+        </is>
+      </c>
+      <c r="G91" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H91" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>After any driver steering input in the last 1.5 s, a temporary EPS fault raises only steerTempUnavailableSilent (a small WARNING with no soft disable), and the warning stays silent for as long as the fault lasts (car_events.py:162-177; T-25, GAP-03)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I91" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream openpilot design choice (a softer alert after an override); no LionDriver requirement on it</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/car/car_events.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="J91" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K91" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No LionDriver test targets this cause</t>
+          </r>
+        </is>
+      </c>
+      <c r="L91" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="M91" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N91" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-023 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Warn audibly and with a take-over request on every EPS fault while engaged, with no silent variant after a recent override (car_events.py steerTempUnavailableSilent), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+          </r>
+        </is>
+      </c>
+      <c r="O91" s="47" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P91" s="33" t="inlineStr"/>
+      <c r="Q91" s="33" t="inlineStr"/>
+      <c r="R91" s="37" t="inlineStr"/>
+      <c r="S91" s="37" t="inlineStr"/>
+    </row>
+    <row r="92" ht="114" customHeight="1">
+      <c r="A92" s="38" t="n"/>
+      <c r="B92" s="38" t="n"/>
+      <c r="C92" s="38" t="n"/>
+      <c r="D92" s="38" t="n"/>
+      <c r="E92" s="38" t="n"/>
+      <c r="F92" s="38" t="n"/>
+      <c r="G92" s="33" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H92" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>pandad publishes the panda fields epsFault and requestsRejected (pandad.cc:137-138), but no SoC process reads them (txRateExceeded is read, TSR-615), so a panda-side EPS-fault refusal reaches the driver only through the panda siren and the stock EPS path (SW FMEA SWF-025 notes)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I92" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• None; the fields were added for the panda siren and logging</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/pandad/pandad.cc</t>
+          </r>
+        </is>
+      </c>
+      <c r="J92" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K92" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No test targets this cause</t>
+          </r>
+        </is>
+      </c>
+      <c r="L92" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="M92" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N92" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-023 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Warn audibly and with a take-over request on every EPS fault while engaged, with no silent variant after a recent override (car_events.py steerTempUnavailableSilent), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+          </r>
+        </is>
+      </c>
+      <c r="O92" s="47" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P92" s="33" t="inlineStr"/>
+      <c r="Q92" s="33" t="inlineStr"/>
+      <c r="R92" s="37" t="inlineStr"/>
+      <c r="S92" s="37" t="inlineStr"/>
+    </row>
+    <row r="93" ht="127.5" customHeight="1">
+      <c r="A93" s="39" t="n"/>
+      <c r="B93" s="39" t="n"/>
+      <c r="C93" s="39" t="n"/>
+      <c r="D93" s="39" t="n"/>
+      <c r="E93" s="39" t="n"/>
+      <c r="F93" s="39" t="n"/>
+      <c r="G93" s="40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="H93" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>steerSaturated needs the controller saturated, a desired lateral acceleration above 1.0 m/s², an undershoot above 1.2x and no steering input for 2 s (selfdrived.py:465-479), and the controller reports saturation only after 0.4 s (latcontrol.py, T-30); a gradual deficit therefore warns late or not at all (WP-S-04 §3.8.1)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I93" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream openpilot code with upstream review; ruff and type checks in CI (static analysis job)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   scripts/lint/lint.sh</t>
+          </r>
+        </is>
+      </c>
+      <c r="J93" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="K93" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Lateral controller unit tests (saturation detection); targeted at nominal behaviour, not proven</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/controls/tests/test_latcontrol.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L93" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="M93" s="44" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N93" s="41" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SFM-ACT-021 · monitoring
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Make the insufficient-lateral-control warning timely (WP-S-04 §3.8.1): warn before the deficit has lasted 0.4 s, for example from the planned curvature against the envelope, or keep the deficit at or below about 0.5 m/s² through the steering limits and the ODD curve bound (WP-S-04 OI-2). A change to the ODD bound is a lead decision</t>
+          </r>
+        </is>
+      </c>
+      <c r="O93" s="48" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P93" s="40" t="inlineStr"/>
+      <c r="Q93" s="40" t="inlineStr"/>
+      <c r="R93" s="45" t="inlineStr"/>
+      <c r="S93" s="45" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S90"/>
-  <mergeCells count="190">
+  <autoFilter ref="A2:S93"/>
+  <mergeCells count="196">
     <mergeCell ref="F84:F85"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="E39:E40"/>
@@ -17830,6 +18281,7 @@
     <mergeCell ref="B10:B13"/>
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B91:B93"/>
     <mergeCell ref="C20:C22"/>
     <mergeCell ref="C14:C16"/>
     <mergeCell ref="E20:E22"/>
@@ -17842,7 +18294,9 @@
     <mergeCell ref="F49:F50"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B75:B76"/>
+    <mergeCell ref="D91:D93"/>
     <mergeCell ref="F20:F22"/>
+    <mergeCell ref="F91:F93"/>
     <mergeCell ref="B44:B46"/>
     <mergeCell ref="A67:A68"/>
     <mergeCell ref="E71:E74"/>
@@ -17852,7 +18306,9 @@
     <mergeCell ref="E57:E59"/>
     <mergeCell ref="A69:A70"/>
     <mergeCell ref="D6:D9"/>
+    <mergeCell ref="A91:A93"/>
     <mergeCell ref="F6:F9"/>
+    <mergeCell ref="C91:C93"/>
     <mergeCell ref="D64:D66"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="E41:E43"/>
@@ -17866,6 +18322,7 @@
     <mergeCell ref="E35:E36"/>
     <mergeCell ref="A75:A76"/>
     <mergeCell ref="C75:C76"/>
+    <mergeCell ref="E91:E93"/>
     <mergeCell ref="F57:F59"/>
     <mergeCell ref="B64:B66"/>
     <mergeCell ref="C25:C28"/>
@@ -17904,7 +18361,7 @@
     <mergeCell ref="D84:D85"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87 R88 R89 R90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87 R88 R89 R90 R91 R92 R93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17912,7 +18369,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.22 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.23 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -17927,7 +18384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18697,7 +19154,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="F21" s="61" t="inlineStr"/>
+      <c r="F21" s="61" t="inlineStr">
+        <is>
+          <t>SFM-038.C3</t>
+        </is>
+      </c>
       <c r="G21" s="61" t="inlineStr"/>
       <c r="H21" s="61" t="inlineStr"/>
       <c r="I21" s="61" t="inlineStr"/>
@@ -18729,8 +19190,40 @@
       <c r="H22" s="61" t="inlineStr"/>
       <c r="I22" s="61" t="inlineStr"/>
     </row>
+    <row r="23" ht="73.5" customHeight="1">
+      <c r="A23" s="61" t="inlineStr">
+        <is>
+          <t>SFM-ACT-023</t>
+        </is>
+      </c>
+      <c r="B23" s="61" t="inlineStr">
+        <is>
+          <t>design change</t>
+        </is>
+      </c>
+      <c r="C23" s="61" t="inlineStr">
+        <is>
+          <t>Warn audibly and with a take-over request on every EPS fault while engaged, with no silent variant after a recent override (car_events.py steerTempUnavailableSilent), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+        </is>
+      </c>
+      <c r="D23" s="61" t="inlineStr"/>
+      <c r="E23" s="61" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F23" s="61" t="inlineStr">
+        <is>
+          <t>SFM-038.C1
+SFM-038.C2</t>
+        </is>
+      </c>
+      <c r="G23" s="61" t="inlineStr"/>
+      <c r="H23" s="61" t="inlineStr"/>
+      <c r="I23" s="61" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19214,7 +19707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P73"/>
+  <dimension ref="A1:P76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -23768,13 +24261,121 @@
       <c r="O73" s="37" t="inlineStr"/>
       <c r="P73" s="37" t="inlineStr"/>
     </row>
+    <row r="74" ht="100.5" customHeight="1">
+      <c r="A74" s="34" t="inlineStr">
+        <is>
+          <t>SFM-038 · Warning of a lateral-control fault or limit late, silent or missing</t>
+        </is>
+      </c>
+      <c r="B74" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C74" s="33" t="inlineStr">
+        <is>
+          <t>SFM-038.C1</t>
+        </is>
+      </c>
+      <c r="D74" s="34" t="inlineStr">
+        <is>
+          <t>After any driver steering input in the last 1.5 s, a temporary EPS fault raises only steerTempUnavailableSilent (a small WARNING with no soft disable), and the warning stays silent for as long as the fault lasts (car_events.py:162-177; T-25, GAP-03)</t>
+        </is>
+      </c>
+      <c r="E74" s="64" t="inlineStr">
+        <is>
+          <t>Exempt: The cause is a defect of the warning path itself; its effect on detecting the lateral loss is rated in the MSR rows of SFM-004.C2 and SFM-005 (msr-plan §3)</t>
+        </is>
+      </c>
+      <c r="F74" s="34" t="inlineStr"/>
+      <c r="G74" s="34" t="inlineStr"/>
+      <c r="H74" s="35" t="inlineStr"/>
+      <c r="I74" s="35" t="inlineStr"/>
+      <c r="J74" s="35" t="inlineStr"/>
+      <c r="K74" s="33" t="inlineStr"/>
+      <c r="L74" s="34" t="inlineStr"/>
+      <c r="M74" s="33" t="inlineStr"/>
+      <c r="N74" s="34" t="inlineStr"/>
+      <c r="O74" s="37" t="inlineStr"/>
+      <c r="P74" s="37" t="inlineStr"/>
+    </row>
+    <row r="75" ht="114" customHeight="1">
+      <c r="A75" s="34" t="inlineStr">
+        <is>
+          <t>SFM-038 · Warning of a lateral-control fault or limit late, silent or missing</t>
+        </is>
+      </c>
+      <c r="B75" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C75" s="33" t="inlineStr">
+        <is>
+          <t>SFM-038.C2</t>
+        </is>
+      </c>
+      <c r="D75" s="34" t="inlineStr">
+        <is>
+          <t>pandad publishes the panda fields epsFault and requestsRejected (pandad.cc:137-138), but no SoC process reads them (txRateExceeded is read, TSR-615), so a panda-side EPS-fault refusal reaches the driver only through the panda siren and the stock EPS path (SW FMEA SWF-025 notes)</t>
+        </is>
+      </c>
+      <c r="E75" s="64" t="inlineStr">
+        <is>
+          <t>Exempt: The cause is a defect of the warning path itself; the panda siren that remains is rated on SFM-005 and in the DFMEA (msr-plan §3)</t>
+        </is>
+      </c>
+      <c r="F75" s="34" t="inlineStr"/>
+      <c r="G75" s="34" t="inlineStr"/>
+      <c r="H75" s="35" t="inlineStr"/>
+      <c r="I75" s="35" t="inlineStr"/>
+      <c r="J75" s="35" t="inlineStr"/>
+      <c r="K75" s="33" t="inlineStr"/>
+      <c r="L75" s="34" t="inlineStr"/>
+      <c r="M75" s="33" t="inlineStr"/>
+      <c r="N75" s="34" t="inlineStr"/>
+      <c r="O75" s="37" t="inlineStr"/>
+      <c r="P75" s="37" t="inlineStr"/>
+    </row>
+    <row r="76" ht="127.5" customHeight="1">
+      <c r="A76" s="34" t="inlineStr">
+        <is>
+          <t>SFM-038 · Warning of a lateral-control fault or limit late, silent or missing</t>
+        </is>
+      </c>
+      <c r="B76" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="C76" s="33" t="inlineStr">
+        <is>
+          <t>SFM-038.C3</t>
+        </is>
+      </c>
+      <c r="D76" s="34" t="inlineStr">
+        <is>
+          <t>steerSaturated needs the controller saturated, a desired lateral acceleration above 1.0 m/s², an undershoot above 1.2x and no steering input for 2 s (selfdrived.py:465-479), and the controller reports saturation only after 0.4 s (latcontrol.py, T-30); a gradual deficit therefore warns late or not at all (WP-S-04 §3.8.1)</t>
+        </is>
+      </c>
+      <c r="E76" s="64" t="inlineStr">
+        <is>
+          <t>Exempt: The cause is the timing of the warning itself; it is rated as M 8 in the MSR rows of SFM-004.C1-C3 (rev 0.15, WP-S-04 §3.8.1)</t>
+        </is>
+      </c>
+      <c r="F76" s="34" t="inlineStr"/>
+      <c r="G76" s="34" t="inlineStr"/>
+      <c r="H76" s="35" t="inlineStr"/>
+      <c r="I76" s="35" t="inlineStr"/>
+      <c r="J76" s="35" t="inlineStr"/>
+      <c r="K76" s="33" t="inlineStr"/>
+      <c r="L76" s="34" t="inlineStr"/>
+      <c r="M76" s="33" t="inlineStr"/>
+      <c r="N76" s="34" t="inlineStr"/>
+      <c r="O76" s="37" t="inlineStr"/>
+      <c r="P76" s="37" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:P73"/>
+  <autoFilter ref="A2:P76"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O67 O68 O69 O70 O71 O72 O73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
+    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O67 O68 O69 O70 O71 O72 O73 O74 O75 O76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -23782,7 +24383,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.22 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.23 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Regenerate the FMEA review outputs and figures after merging liondriver-dev (#150)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.19 · draft</t>
+          <t>0.20 · draft</t>
         </is>
       </c>
     </row>
@@ -12644,6 +12644,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-013: driver-monitoring escalation alerts not shown or played, so an inattentive driver is not told; the forced deceleration does not depend on them (as SWF-082)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -12685,7 +12711,8 @@
       <c r="D64" s="31" t="inlineStr">
         <is>
           <t>HZ-012
-HZ-006</t>
+HZ-006
+HZ-013</t>
         </is>
       </c>
       <c r="E64" s="32" t="n">
@@ -13150,6 +13177,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-013: a driver-monitoring escalation presented late, or hidden behind a higher-priority alert, so the inattentive driver is told late (as SWF-035)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -13190,7 +13243,8 @@
       </c>
       <c r="D67" s="31" t="inlineStr">
         <is>
-          <t>HZ-012</t>
+          <t>HZ-012
+HZ-013</t>
         </is>
       </c>
       <c r="E67" s="32" t="n">
@@ -17265,7 +17319,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.19 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -22937,7 +22991,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.19 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Regenerate the FMEA review outputs and figures after merging the updated base
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.20 · draft</t>
+          <t>0.21 · draft</t>
         </is>
       </c>
     </row>
@@ -7633,6 +7633,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-005: positive acceleration requested after an engagement the driver did not ask for</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -7673,7 +7699,8 @@
       </c>
       <c r="D39" s="31" t="inlineStr">
         <is>
-          <t>HZ-010</t>
+          <t>HZ-010
+HZ-005</t>
         </is>
       </c>
       <c r="E39" s="32" t="n">
@@ -9445,6 +9472,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-005: the item keeps requesting acceleration while the driver brakes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -9485,7 +9538,8 @@
       </c>
       <c r="D49" s="31" t="inlineStr">
         <is>
-          <t>HZ-008</t>
+          <t>HZ-008
+HZ-005</t>
         </is>
       </c>
       <c r="E49" s="32" t="n">
@@ -10815,6 +10869,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-008: the driver cancels but stock cruise keeps longitudinal control</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -10855,7 +10935,8 @@
       </c>
       <c r="D55" s="31" t="inlineStr">
         <is>
-          <t>HZ-012</t>
+          <t>HZ-012
+HZ-008</t>
         </is>
       </c>
       <c r="E55" s="32" t="n">
@@ -13559,6 +13640,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-008: the driver believes control was released by the brake or cancel while the item still acts</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -13599,7 +13706,8 @@
       </c>
       <c r="D69" s="31" t="inlineStr">
         <is>
-          <t>HZ-012</t>
+          <t>HZ-012
+HZ-008</t>
         </is>
       </c>
       <c r="E69" s="32" t="n">
@@ -16122,6 +16230,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-005: stock ACC and item acceleration requests combine on the bus</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -16164,7 +16298,8 @@
         <is>
           <t>HZ-011
 HZ-002
-HZ-006</t>
+HZ-006
+HZ-005</t>
         </is>
       </c>
       <c r="E82" s="32" t="n">
@@ -16299,7 +16434,7 @@
       <c r="R82" s="37" t="inlineStr"/>
       <c r="S82" s="37" t="inlineStr"/>
     </row>
-    <row r="83" ht="102" customHeight="1">
+    <row r="83" ht="142.5" customHeight="1">
       <c r="A83" s="39" t="n"/>
       <c r="B83" s="39" t="n"/>
       <c r="C83" s="39" t="n"/>
@@ -17319,7 +17454,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.21 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -22991,7 +23126,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.20 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.21 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
SFM-038 / SFM-ACT-023: the override EPS warning chimes but never escalates
Correction from the FSC session: steerTempUnavailableSilent is a
LOW-priority warning with a prompt chime and no soft disable
(events.py:516-521), not silent. The defect is that it stays latched
while the EPS fault lasts, so a long fault after an override or at
standstill never reaches the take-over request. Failure mode, C1,
SFM-ACT-023 and the BE-2.08 note reworded; the action now names the
lead question DQ-342. No rating changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -17744,7 +17744,7 @@
       <c r="R90" s="45" t="inlineStr"/>
       <c r="S90" s="45" t="inlineStr"/>
     </row>
-    <row r="91" ht="114" customHeight="1">
+    <row r="91" ht="168" customHeight="1">
       <c r="A91" s="30" t="inlineStr">
         <is>
           <r>
@@ -17858,7 +17858,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>steerTempUnavailable shown silently, steerSaturated raised late or not at all, or the panda's EPS-fault flag not acted on</t>
+            <t>steerTempUnavailable not escalated to a take-over request, steerSaturated raised late or not at all, or the panda's EPS-fault flag not acted on</t>
           </r>
         </is>
       </c>
@@ -17889,7 +17889,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Warning of a lateral-control fault or limit late, silent or missing</t>
+            <t>Warning of a lateral-control fault or limit late, not escalated or missing</t>
           </r>
         </is>
       </c>
@@ -17906,7 +17906,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>After any driver steering input in the last 1.5 s, a temporary EPS fault raises only steerTempUnavailableSilent (a small WARNING with no soft disable), and the warning stays silent for as long as the fault lasts (car_events.py:162-177; T-25, GAP-03)</t>
+            <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
           </r>
         </is>
       </c>
@@ -17972,7 +17972,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Warn audibly and with a take-over request on every EPS fault while engaged, with no silent variant after a recent override (car_events.py steerTempUnavailableSilent), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+            <t>Escalate every EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE), instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py:162-177; behaviour change queued for the lead by the FSC session as DQ-342), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
           </r>
         </is>
       </c>
@@ -17986,7 +17986,7 @@
       <c r="R91" s="37" t="inlineStr"/>
       <c r="S91" s="37" t="inlineStr"/>
     </row>
-    <row r="92" ht="114" customHeight="1">
+    <row r="92" ht="168" customHeight="1">
       <c r="A92" s="38" t="n"/>
       <c r="B92" s="38" t="n"/>
       <c r="C92" s="38" t="n"/>
@@ -18072,7 +18072,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Warn audibly and with a take-over request on every EPS fault while engaged, with no silent variant after a recent override (car_events.py steerTempUnavailableSilent), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+            <t>Escalate every EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE), instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py:162-177; behaviour change queued for the lead by the FSC session as DQ-342), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
           </r>
         </is>
       </c>
@@ -19225,7 +19225,7 @@
       <c r="H22" s="61" t="inlineStr"/>
       <c r="I22" s="61" t="inlineStr"/>
     </row>
-    <row r="23" ht="73.5" customHeight="1">
+    <row r="23" ht="100.5" customHeight="1">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>SFM-ACT-023</t>
@@ -19238,7 +19238,7 @@
       </c>
       <c r="C23" s="61" t="inlineStr">
         <is>
-          <t>Warn audibly and with a take-over request on every EPS fault while engaged, with no silent variant after a recent override (car_events.py steerTempUnavailableSilent), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+          <t>Escalate every EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE), instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py:162-177; behaviour change queued for the lead by the FSC session as DQ-342), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
         </is>
       </c>
       <c r="D23" s="61" t="inlineStr"/>
@@ -24296,10 +24296,10 @@
       <c r="O73" s="37" t="inlineStr"/>
       <c r="P73" s="37" t="inlineStr"/>
     </row>
-    <row r="74" ht="100.5" customHeight="1">
+    <row r="74" ht="141" customHeight="1">
       <c r="A74" s="34" t="inlineStr">
         <is>
-          <t>SFM-038 · Warning of a lateral-control fault or limit late, silent or missing</t>
+          <t>SFM-038 · Warning of a lateral-control fault or limit late, not escalated or missing</t>
         </is>
       </c>
       <c r="B74" s="35" t="n">
@@ -24312,7 +24312,7 @@
       </c>
       <c r="D74" s="34" t="inlineStr">
         <is>
-          <t>After any driver steering input in the last 1.5 s, a temporary EPS fault raises only steerTempUnavailableSilent (a small WARNING with no soft disable), and the warning stays silent for as long as the fault lasts (car_events.py:162-177; T-25, GAP-03)</t>
+          <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
         </is>
       </c>
       <c r="E74" s="64" t="inlineStr">
@@ -24335,7 +24335,7 @@
     <row r="75" ht="114" customHeight="1">
       <c r="A75" s="34" t="inlineStr">
         <is>
-          <t>SFM-038 · Warning of a lateral-control fault or limit late, silent or missing</t>
+          <t>SFM-038 · Warning of a lateral-control fault or limit late, not escalated or missing</t>
         </is>
       </c>
       <c r="B75" s="35" t="n">
@@ -24371,7 +24371,7 @@
     <row r="76" ht="127.5" customHeight="1">
       <c r="A76" s="34" t="inlineStr">
         <is>
-          <t>SFM-038 · Warning of a lateral-control fault or limit late, silent or missing</t>
+          <t>SFM-038 · Warning of a lateral-control fault or limit late, not escalated or missing</t>
         </is>
       </c>
       <c r="B76" s="35" t="n">

</xml_diff>

<commit_message>
System FMEA rev 0.24: apply DQ-365 A to SFM-ACT-005
The lead decided the zero-awareness reaction (DQ-365, option A, which
absorbs DQ-340): stop in the lane, hold the vehicle, and lock out
re-engagement until the driver responds, specified in TSR-633
(WP-S-02 v0.26, #151). SFM-ACT-005 moves from decision_pending to open
and names TSR-633 and the preliminary WP-S-04 v0.12 §3.8.4 time. The
SFM-025 note no longer says the decision is open. Not implemented at
BL-005, so SFM-025.C1 keeps O 8, D 9, M 10. Review exports regenerated;
they no longer cite DQ-340. Merge after #151.

AI-drafted; for the lead's review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -261,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -396,9 +396,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -823,7 +820,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.23 · draft</t>
+          <t>0.24 · draft</t>
         </is>
       </c>
     </row>
@@ -12333,7 +12330,7 @@
       <c r="R62" s="45" t="inlineStr"/>
       <c r="S62" s="45" t="inlineStr"/>
     </row>
-    <row r="63" ht="195" customHeight="1">
+    <row r="63" ht="249" customHeight="1">
       <c r="A63" s="51" t="inlineStr">
         <is>
           <r>
@@ -12605,13 +12602,13 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided. The requirement is TSR-633 (terminal reaction, ASIL A proposed) with TSR-611 (WP-S-02 §12.3a); the reaction is lead decision DQ-340. The H-09 FTTI is not yet set, so the timing rows of WP-S-04 §3.8.4 cannot be compared</t>
-          </r>
-        </is>
-      </c>
-      <c r="O63" s="57" t="inlineStr">
-        <is>
-          <t>decision pending</t>
+            <t>Implement the reaction when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005), the safe state of SG-010 (WP-C-03 SG-08, ASIL A; DQ-205). Decided by the lead (DQ-365, option A, 2026-10-16) and specified in TSR-633 (WP-S-02 v0.26) with TSR-611; keep the lane and decelerate in lane to a standstill with the terminal alert sounding, hold the vehicle stopped, and lock out re-engagement and resumption until the driver responds. WP-S-04 v0.12 §3.8.4 gives a preliminary time to the reaction (18 s vision, 30 s wheel-touch from loss of attention; OI-11); SFM-025.C1 is re-rated once TSR-633 is implemented and that time is confirmed</t>
+          </r>
+        </is>
+      </c>
+      <c r="O63" s="48" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
       <c r="P63" s="40" t="inlineStr"/>
@@ -14215,7 +14212,7 @@
       <c r="L71" s="35" t="n">
         <v>4</v>
       </c>
-      <c r="M71" s="58" t="inlineStr">
+      <c r="M71" s="57" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -17156,7 +17153,7 @@
           </r>
         </is>
       </c>
-      <c r="O86" s="59" t="inlineStr">
+      <c r="O86" s="58" t="inlineStr">
         <is>
           <t>decision pending</t>
         </is>
@@ -18404,7 +18401,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.23 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.24 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -18434,79 +18431,79 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="B1" s="60" t="inlineStr">
+      <c r="B1" s="59" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="C1" s="60" t="inlineStr">
+      <c r="C1" s="59" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="60" t="inlineStr">
+      <c r="D1" s="59" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E1" s="60" t="inlineStr">
+      <c r="E1" s="59" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="60" t="inlineStr">
+      <c r="F1" s="59" t="inlineStr">
         <is>
           <t>Causes</t>
         </is>
       </c>
-      <c r="G1" s="60" t="inlineStr">
+      <c r="G1" s="59" t="inlineStr">
         <is>
           <t>Revised S/O/D</t>
         </is>
       </c>
-      <c r="H1" s="60" t="inlineStr">
+      <c r="H1" s="59" t="inlineStr">
         <is>
           <t>Revised AP</t>
         </is>
       </c>
-      <c r="I1" s="60" t="inlineStr">
+      <c r="I1" s="59" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
     </row>
     <row r="2" ht="127.5" customHeight="1">
-      <c r="A2" s="61" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-001</t>
         </is>
       </c>
-      <c r="B2" s="61" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C2" s="61" t="inlineStr">
+      <c r="C2" s="60" t="inlineStr">
         <is>
           <t>Derive steering and acceleration envelopes from measurements on the reference vehicle and set the panda limits from them, independently of the SoC limits (same as SWF-ACT-003, FSC FOI-001)</t>
         </is>
       </c>
-      <c r="D2" s="61" t="inlineStr">
+      <c r="D2" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E2" s="61" t="inlineStr">
+      <c r="E2" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F2" s="61" t="inlineStr">
+      <c r="F2" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
@@ -18519,37 +18516,37 @@
 SFM-029.C2</t>
         </is>
       </c>
-      <c r="G2" s="61" t="inlineStr"/>
-      <c r="H2" s="61" t="inlineStr"/>
-      <c r="I2" s="61" t="inlineStr"/>
+      <c r="G2" s="60" t="inlineStr"/>
+      <c r="H2" s="60" t="inlineStr"/>
+      <c r="I2" s="60" t="inlineStr"/>
     </row>
     <row r="3" ht="168" customHeight="1">
-      <c r="A3" s="61" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-002</t>
         </is>
       </c>
-      <c r="B3" s="61" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C3" s="61" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
         </is>
       </c>
-      <c r="D3" s="61" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E3" s="61" t="inlineStr">
+      <c r="E3" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F3" s="61" t="inlineStr">
+      <c r="F3" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C4
 SFM-004.C3
@@ -18565,37 +18562,37 @@
 SFM-037.C3</t>
         </is>
       </c>
-      <c r="G3" s="61" t="inlineStr"/>
-      <c r="H3" s="61" t="inlineStr"/>
-      <c r="I3" s="61" t="inlineStr"/>
+      <c r="G3" s="60" t="inlineStr"/>
+      <c r="H3" s="60" t="inlineStr"/>
+      <c r="I3" s="60" t="inlineStr"/>
     </row>
     <row r="4" ht="343.5" customHeight="1">
-      <c r="A4" s="61" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-003</t>
         </is>
       </c>
-      <c r="B4" s="61" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C4" s="61" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
         </is>
       </c>
-      <c r="D4" s="61" t="inlineStr">
+      <c r="D4" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E4" s="61" t="inlineStr">
+      <c r="E4" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F4" s="61" t="inlineStr">
+      <c r="F4" s="60" t="inlineStr">
         <is>
           <t>SFM-003.C1
 SFM-003.C2
@@ -18624,72 +18621,72 @@
 SFM-033.C3</t>
         </is>
       </c>
-      <c r="G4" s="61" t="inlineStr"/>
-      <c r="H4" s="61" t="inlineStr"/>
-      <c r="I4" s="61" t="inlineStr"/>
+      <c r="G4" s="60" t="inlineStr"/>
+      <c r="H4" s="60" t="inlineStr"/>
+      <c r="I4" s="60" t="inlineStr"/>
     </row>
-    <row r="5" ht="114" customHeight="1">
-      <c r="A5" s="61" t="inlineStr">
+    <row r="5" ht="154.5" customHeight="1">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-005</t>
         </is>
       </c>
-      <c r="B5" s="61" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C5" s="61" t="inlineStr">
-        <is>
-          <t>Decide in the FSC how the item reacts when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005) and implement the decision. DQ-205 (answered) makes this the safe state of SG-010 (WP-C-03 SG-08, ASIL A); the reaction itself is still to be decided. The requirement is TSR-633 (terminal reaction, ASIL A proposed) with TSR-611 (WP-S-02 §12.3a); the reaction is lead decision DQ-340. The H-09 FTTI is not yet set, so the timing rows of WP-S-04 §3.8.4 cannot be compared</t>
-        </is>
-      </c>
-      <c r="D5" s="61" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
+        <is>
+          <t>Implement the reaction when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005), the safe state of SG-010 (WP-C-03 SG-08, ASIL A; DQ-205). Decided by the lead (DQ-365, option A, 2026-10-16) and specified in TSR-633 (WP-S-02 v0.26) with TSR-611; keep the lane and decelerate in lane to a standstill with the terminal alert sounding, hold the vehicle stopped, and lock out re-engagement and resumption until the driver responds. WP-S-04 v0.12 §3.8.4 gives a preliminary time to the reaction (18 s vision, 30 s wheel-touch from loss of attention; OI-11); SFM-025.C1 is re-rated once TSR-633 is implemented and that time is confirmed</t>
+        </is>
+      </c>
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E5" s="61" t="inlineStr">
-        <is>
-          <t>decision pending</t>
-        </is>
-      </c>
-      <c r="F5" s="61" t="inlineStr">
+      <c r="E5" s="60" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F5" s="60" t="inlineStr">
         <is>
           <t>SFM-025.C1</t>
         </is>
       </c>
-      <c r="G5" s="61" t="inlineStr"/>
-      <c r="H5" s="61" t="inlineStr"/>
-      <c r="I5" s="61" t="inlineStr"/>
+      <c r="G5" s="60" t="inlineStr"/>
+      <c r="H5" s="60" t="inlineStr"/>
+      <c r="I5" s="60" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-006</t>
         </is>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C6" s="61" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>Establish on the reference car which stock TSS2 functions (PCS/AEB, FCW) remain available with LionDriver installed and longitudinal control enabled, and verify the stock pre-collision path after installation (PFMEA PFM-014)</t>
         </is>
       </c>
-      <c r="D6" s="61" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E6" s="61" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F6" s="61" t="inlineStr">
+      <c r="F6" s="60" t="inlineStr">
         <is>
           <t>SFM-010.C2
 SFM-033.C1
@@ -18697,37 +18694,37 @@
 SFM-036.C2</t>
         </is>
       </c>
-      <c r="G6" s="61" t="inlineStr"/>
-      <c r="H6" s="61" t="inlineStr"/>
-      <c r="I6" s="61" t="inlineStr"/>
+      <c r="G6" s="60" t="inlineStr"/>
+      <c r="H6" s="60" t="inlineStr"/>
+      <c r="I6" s="60" t="inlineStr"/>
     </row>
     <row r="7" ht="73.5" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-007</t>
         </is>
       </c>
-      <c r="B7" s="61" t="inlineStr">
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C7" s="61" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>Supervise the alert channels: treat loss of ui or soundd liveness, or a stale displayed state, as a fault that escalates (audible fallback, disengagement) instead of continuing silently</t>
         </is>
       </c>
-      <c r="D7" s="61" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E7" s="61" t="inlineStr">
+      <c r="E7" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F7" s="61" t="inlineStr">
+      <c r="F7" s="60" t="inlineStr">
         <is>
           <t>SFM-015.C1
 SFM-026.C1
@@ -18736,76 +18733,76 @@
 SFM-028.C1</t>
         </is>
       </c>
-      <c r="G7" s="61" t="inlineStr"/>
-      <c r="H7" s="61" t="inlineStr"/>
-      <c r="I7" s="61" t="inlineStr"/>
+      <c r="G7" s="60" t="inlineStr"/>
+      <c r="H7" s="60" t="inlineStr"/>
+      <c r="I7" s="60" t="inlineStr"/>
     </row>
     <row r="8" ht="73.5" customHeight="1">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-008</t>
         </is>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>Allow engagement only when the fingerprint, CarParams and panda safety parameter match the reference configuration AC-001 (refuse fuzzy matches in the reference build); see PFMEA PFM-013</t>
         </is>
       </c>
-      <c r="D8" s="61" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E8" s="61" t="inlineStr">
+      <c r="E8" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F8" s="61" t="inlineStr">
+      <c r="F8" s="60" t="inlineStr">
         <is>
           <t>SFM-032.C1</t>
         </is>
       </c>
-      <c r="G8" s="61" t="inlineStr"/>
-      <c r="H8" s="61" t="inlineStr"/>
-      <c r="I8" s="61" t="inlineStr">
+      <c r="G8" s="60" t="inlineStr"/>
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr">
         <is>
           <t>BL-005: the reference build is the default (LionDriver #36), the panda accepts only TOYOTA parameter 73 (reference_lock.h) and pandad configures a car mode only on a reference panda (#41). Fuzzy fingerprint matches are still accepted on the host (SFM-032.C1)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="100.5" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-009</t>
         </is>
       </c>
-      <c r="B9" s="61" t="inlineStr">
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t>prevention</t>
         </is>
       </c>
-      <c r="C9" s="61" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>Produce SOTIF / ISO PAS 8800 evidence for the neural-network elements (driving model, lead detection, driver monitoring model) per WP-V-02..04, including fault-induced inputs (corrupted or stale frames)</t>
         </is>
       </c>
-      <c r="D9" s="61" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E9" s="61" t="inlineStr">
+      <c r="E9" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F9" s="61" t="inlineStr">
+      <c r="F9" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C2
 SFM-003.C3
@@ -18816,37 +18813,37 @@
 SFM-022.C2</t>
         </is>
       </c>
-      <c r="G9" s="61" t="inlineStr"/>
-      <c r="H9" s="61" t="inlineStr"/>
-      <c r="I9" s="61" t="inlineStr"/>
+      <c r="G9" s="60" t="inlineStr"/>
+      <c r="H9" s="60" t="inlineStr"/>
+      <c r="I9" s="60" t="inlineStr"/>
     </row>
     <row r="10" ht="73.5" customHeight="1">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-010</t>
         </is>
       </c>
-      <c r="B10" s="61" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C10" s="61" t="inlineStr">
+      <c r="C10" s="60" t="inlineStr">
         <is>
           <t>Justify every SOFT_DISABLE reaction and debounce against the FTTI (WP-S-04) and alert at once when the panda withdraws authority while engaged (controlsMismatch debounce)</t>
         </is>
       </c>
-      <c r="D10" s="61" t="inlineStr">
+      <c r="D10" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E10" s="61" t="inlineStr">
+      <c r="E10" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F10" s="61" t="inlineStr">
+      <c r="F10" s="60" t="inlineStr">
         <is>
           <t>SFM-014.C2
 SFM-015.C2
@@ -18854,408 +18851,408 @@
 SFM-016.C2</t>
         </is>
       </c>
-      <c r="G10" s="61" t="inlineStr"/>
-      <c r="H10" s="61" t="inlineStr"/>
-      <c r="I10" s="61" t="inlineStr">
+      <c r="G10" s="60" t="inlineStr"/>
+      <c r="H10" s="60" t="inlineStr"/>
+      <c r="I10" s="60" t="inlineStr">
         <is>
           <t>controlsMismatch debounce cut from 200 cumulative samples (~2 s) to 2 consecutive samples, at most 0.5 s (change-2026-10-13-host-supervision.md); credited at BL-005 (SFM-015.C2 M 6). FTTI justification of SOFT_DISABLE reactions open</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-011</t>
         </is>
       </c>
-      <c r="B11" s="61" t="inlineStr">
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C11" s="61" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
         <is>
           <t>Alert the driver when stock cruise stays engaged while the item is disengaged (cruiseMismatch has no alert at BL-004)</t>
         </is>
       </c>
-      <c r="D11" s="61" t="inlineStr">
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E11" s="62" t="inlineStr">
+      <c r="E11" s="61" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F11" s="61" t="inlineStr">
+      <c r="F11" s="60" t="inlineStr">
         <is>
           <t>SFM-021.C1
 SFM-021.C2</t>
         </is>
       </c>
-      <c r="G11" s="61" t="inlineStr"/>
-      <c r="H11" s="61" t="inlineStr"/>
-      <c r="I11" s="61" t="inlineStr">
+      <c r="G11" s="60" t="inlineStr"/>
+      <c r="H11" s="60" t="inlineStr"/>
+      <c r="I11" s="60" t="inlineStr">
         <is>
           <t>cruiseMismatch now alerts after 1 s (change-2026-10-13-host-supervision.md); see SWF-ACT-034</t>
         </is>
       </c>
     </row>
     <row r="12" ht="73.5" customHeight="1">
-      <c r="A12" s="61" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-012</t>
         </is>
       </c>
-      <c r="B12" s="61" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C12" s="61" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>Measure on the HIL bench and the reference car (WP-V-05) how the panda reacts to over-limit and not-engaged steering and acceleration frames and to driver brake, gas and cancel inputs, and what the EPS and PCM do when frames are refused; re-rate the MSR rows from code-derived to measured timing</t>
         </is>
       </c>
-      <c r="D12" s="61" t="inlineStr"/>
-      <c r="E12" s="61" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F12" s="61" t="inlineStr"/>
-      <c r="G12" s="61" t="inlineStr"/>
-      <c r="H12" s="61" t="inlineStr"/>
-      <c r="I12" s="61" t="inlineStr"/>
+      <c r="F12" s="60" t="inlineStr"/>
+      <c r="G12" s="60" t="inlineStr"/>
+      <c r="H12" s="60" t="inlineStr"/>
+      <c r="I12" s="60" t="inlineStr"/>
     </row>
     <row r="13" ht="87" customHeight="1">
-      <c r="A13" s="61" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-013</t>
         </is>
       </c>
-      <c r="B13" s="61" t="inlineStr">
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C13" s="61" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert. The requirement is TSR-630, within 0.3 s (WP-S-02 §12.3a; WP-S-04 T-32, not implemented)</t>
         </is>
       </c>
-      <c r="D13" s="61" t="inlineStr"/>
-      <c r="E13" s="61" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr"/>
+      <c r="E13" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F13" s="61" t="inlineStr"/>
-      <c r="G13" s="61" t="inlineStr"/>
-      <c r="H13" s="61" t="inlineStr"/>
-      <c r="I13" s="61" t="inlineStr"/>
+      <c r="F13" s="60" t="inlineStr"/>
+      <c r="G13" s="60" t="inlineStr"/>
+      <c r="H13" s="60" t="inlineStr"/>
+      <c r="I13" s="60" t="inlineStr"/>
     </row>
     <row r="14" ht="46.5" customHeight="1">
-      <c r="A14" s="61" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-014</t>
         </is>
       </c>
-      <c r="B14" s="61" t="inlineStr">
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C14" s="61" t="inlineStr">
+      <c r="C14" s="60" t="inlineStr">
         <is>
           <t>Specify in the TSC a steering-direction plausibility monitor (commanded torque sign against measured yaw rate and lane-relative lateral motion), or justify its absence against HZ-003</t>
         </is>
       </c>
-      <c r="D14" s="61" t="inlineStr"/>
-      <c r="E14" s="61" t="inlineStr">
+      <c r="D14" s="60" t="inlineStr"/>
+      <c r="E14" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F14" s="61" t="inlineStr"/>
-      <c r="G14" s="61" t="inlineStr"/>
-      <c r="H14" s="61" t="inlineStr"/>
-      <c r="I14" s="61" t="inlineStr"/>
+      <c r="F14" s="60" t="inlineStr"/>
+      <c r="G14" s="60" t="inlineStr"/>
+      <c r="H14" s="60" t="inlineStr"/>
+      <c r="I14" s="60" t="inlineStr"/>
     </row>
     <row r="15" ht="100.5" customHeight="1">
-      <c r="A15" s="61" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-015</t>
         </is>
       </c>
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C15" s="61" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>Detect stale commands and inputs within the SG-01 FTTI: command-frame freshness in the MCU with an active zero frame (TSR-408, TSR-109) and frozen-content and age checks on model outputs in controlsd (TSR-602, TSR-631, AIR-17)</t>
         </is>
       </c>
-      <c r="D15" s="61" t="inlineStr"/>
-      <c r="E15" s="61" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr"/>
+      <c r="E15" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F15" s="61" t="inlineStr"/>
-      <c r="G15" s="61" t="inlineStr"/>
-      <c r="H15" s="61" t="inlineStr"/>
-      <c r="I15" s="61" t="inlineStr">
+      <c r="F15" s="60" t="inlineStr"/>
+      <c r="G15" s="60" t="inlineStr"/>
+      <c r="H15" s="60" t="inlineStr"/>
+      <c r="I15" s="60" t="inlineStr">
         <is>
           <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3). The frozen-content check is TSR-631, with the age taken from the source timestamp (WP-S-02 §12.3a)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="73.5" customHeight="1">
-      <c r="A16" s="61" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-016</t>
         </is>
       </c>
-      <c r="B16" s="61" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C16" s="61" t="inlineStr">
+      <c r="C16" s="60" t="inlineStr">
         <is>
           <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue. Requirements: TSR-304 (timing tied to the SG-05 budget) and TSR-628 (WP-S-02 §12.3a)</t>
         </is>
       </c>
-      <c r="D16" s="61" t="inlineStr"/>
-      <c r="E16" s="61" t="inlineStr">
+      <c r="D16" s="60" t="inlineStr"/>
+      <c r="E16" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F16" s="61" t="inlineStr"/>
-      <c r="G16" s="61" t="inlineStr"/>
-      <c r="H16" s="61" t="inlineStr"/>
-      <c r="I16" s="61" t="inlineStr"/>
+      <c r="F16" s="60" t="inlineStr"/>
+      <c r="G16" s="60" t="inlineStr"/>
+      <c r="H16" s="60" t="inlineStr"/>
+      <c r="I16" s="60" t="inlineStr"/>
     </row>
     <row r="17" ht="87" customHeight="1">
-      <c r="A17" s="61" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-017</t>
         </is>
       </c>
-      <c r="B17" s="61" t="inlineStr">
+      <c r="B17" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>Add WP-S-04 FTTI rows for the warning paths without one (insufficient lateral control, late or insufficient braking warnings, SG-008 unintended engagement, driver monitoring), so these mechanisms can be compared with a time budget</t>
         </is>
       </c>
-      <c r="D17" s="61" t="inlineStr"/>
-      <c r="E17" s="62" t="inlineStr">
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="61" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F17" s="61" t="inlineStr"/>
-      <c r="G17" s="61" t="inlineStr"/>
-      <c r="H17" s="61" t="inlineStr"/>
-      <c r="I17" s="61" t="inlineStr">
+      <c r="F17" s="60" t="inlineStr"/>
+      <c r="G17" s="60" t="inlineStr"/>
+      <c r="H17" s="60" t="inlineStr"/>
+      <c r="I17" s="60" t="inlineStr">
         <is>
           <t>WP-S-04 v0.7 §3.7 (four rows) and §3.8, with T-30 to T-33. Rev 0.15 compares SFM-004, SFM-010.C2/C3, SFM-012.C1 and SFM-013.C1/C2 with them. Driver monitoring (SFM-022.C3, SFM-025.C1) waits for the H-09 FTTI (§3.8.4); follow-up is SFM-ACT-005. Late warnings found: SFM-ACT-021 (lateral) and SFM-ACT-022 (braking)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="100.5" customHeight="1">
-      <c r="A18" s="61" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-018</t>
         </is>
       </c>
-      <c r="B18" s="61" t="inlineStr">
+      <c r="B18" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr">
+      <c r="C18" s="60" t="inlineStr">
         <is>
           <t>Detect silent loss of the actuation path: report forwarded and refused TX frames from the panda, and compare EPS and PCM acceptance (LKA_STATE, ACC status) with the commands, warning within the SG-02/06 1 s budget</t>
         </is>
       </c>
-      <c r="D18" s="61" t="inlineStr"/>
-      <c r="E18" s="61" t="inlineStr">
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="60" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F18" s="61" t="inlineStr"/>
-      <c r="G18" s="61" t="inlineStr"/>
-      <c r="H18" s="61" t="inlineStr"/>
-      <c r="I18" s="61" t="inlineStr">
+      <c r="F18" s="60" t="inlineStr"/>
+      <c r="G18" s="60" t="inlineStr"/>
+      <c r="H18" s="60" t="inlineStr"/>
+      <c r="I18" s="60" t="inlineStr">
         <is>
           <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1). Requirements: TSR-632 (per-ID transmitted and refused counts), TSR-626(d)/(e) (EPS and PCM acceptance status) and TSR-615, warning within 1 s (WP-S-02 §12.3a)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="61" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-019</t>
         </is>
       </c>
-      <c r="B19" s="61" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C19" s="61" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
         </is>
       </c>
-      <c r="D19" s="61" t="inlineStr"/>
-      <c r="E19" s="61" t="inlineStr">
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F19" s="61" t="inlineStr">
+      <c r="F19" s="60" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
 SFM-002.C4</t>
         </is>
       </c>
-      <c r="G19" s="61" t="inlineStr"/>
-      <c r="H19" s="61" t="inlineStr"/>
-      <c r="I19" s="61" t="inlineStr"/>
+      <c r="G19" s="60" t="inlineStr"/>
+      <c r="H19" s="60" t="inlineStr"/>
+      <c r="I19" s="60" t="inlineStr"/>
     </row>
     <row r="20" ht="73.5" customHeight="1">
-      <c r="A20" s="61" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-020</t>
         </is>
       </c>
-      <c r="B20" s="61" t="inlineStr">
+      <c r="B20" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C20" s="61" t="inlineStr">
+      <c r="C20" s="60" t="inlineStr">
         <is>
           <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
         </is>
       </c>
-      <c r="D20" s="61" t="inlineStr"/>
-      <c r="E20" s="61" t="inlineStr">
+      <c r="D20" s="60" t="inlineStr"/>
+      <c r="E20" s="60" t="inlineStr">
         <is>
           <t>decision pending</t>
         </is>
       </c>
-      <c r="F20" s="61" t="inlineStr">
+      <c r="F20" s="60" t="inlineStr">
         <is>
           <t>SFM-036.C1</t>
         </is>
       </c>
-      <c r="G20" s="61" t="inlineStr"/>
-      <c r="H20" s="61" t="inlineStr"/>
-      <c r="I20" s="61" t="inlineStr"/>
+      <c r="G20" s="60" t="inlineStr"/>
+      <c r="H20" s="60" t="inlineStr"/>
+      <c r="I20" s="60" t="inlineStr"/>
     </row>
     <row r="21" ht="73.5" customHeight="1">
-      <c r="A21" s="61" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-021</t>
         </is>
       </c>
-      <c r="B21" s="61" t="inlineStr">
+      <c r="B21" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C21" s="61" t="inlineStr">
+      <c r="C21" s="60" t="inlineStr">
         <is>
           <t>Make the insufficient-lateral-control warning timely (WP-S-04 §3.8.1): warn before the deficit has lasted 0.4 s, for example from the planned curvature against the envelope, or keep the deficit at or below about 0.5 m/s² through the steering limits and the ODD curve bound (WP-S-04 OI-2). A change to the ODD bound is a lead decision</t>
         </is>
       </c>
-      <c r="D21" s="61" t="inlineStr"/>
-      <c r="E21" s="61" t="inlineStr">
+      <c r="D21" s="60" t="inlineStr"/>
+      <c r="E21" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F21" s="61" t="inlineStr">
+      <c r="F21" s="60" t="inlineStr">
         <is>
           <t>SFM-038.C3</t>
         </is>
       </c>
-      <c r="G21" s="61" t="inlineStr"/>
-      <c r="H21" s="61" t="inlineStr"/>
-      <c r="I21" s="61" t="inlineStr"/>
+      <c r="G21" s="60" t="inlineStr"/>
+      <c r="H21" s="60" t="inlineStr"/>
+      <c r="I21" s="60" t="inlineStr"/>
     </row>
     <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="61" t="inlineStr">
+      <c r="A22" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-022</t>
         </is>
       </c>
-      <c r="B22" s="61" t="inlineStr">
+      <c r="B22" s="60" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C22" s="61" t="inlineStr">
+      <c r="C22" s="60" t="inlineStr">
         <is>
           <t>Measure the FCW onset after a lead brakes hard (WP-S-04 T-31, M-12) and compare it with the §3.8.2 budget (about 0.6 s at a 1.0 s gap). For pipeline lag (SFM-012.C1), detect it within that budget or show that the FCW path does not depend on the lagging process</t>
         </is>
       </c>
-      <c r="D22" s="61" t="inlineStr"/>
-      <c r="E22" s="61" t="inlineStr">
+      <c r="D22" s="60" t="inlineStr"/>
+      <c r="E22" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F22" s="61" t="inlineStr"/>
-      <c r="G22" s="61" t="inlineStr"/>
-      <c r="H22" s="61" t="inlineStr"/>
-      <c r="I22" s="61" t="inlineStr"/>
+      <c r="F22" s="60" t="inlineStr"/>
+      <c r="G22" s="60" t="inlineStr"/>
+      <c r="H22" s="60" t="inlineStr"/>
+      <c r="I22" s="60" t="inlineStr"/>
     </row>
     <row r="23" ht="100.5" customHeight="1">
-      <c r="A23" s="61" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-023</t>
         </is>
       </c>
-      <c r="B23" s="61" t="inlineStr">
+      <c r="B23" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C23" s="61" t="inlineStr">
+      <c r="C23" s="60" t="inlineStr">
         <is>
           <t>Escalate every EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE), instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py:162-177; behaviour change queued for the lead by the FSC session as DQ-342), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
         </is>
       </c>
-      <c r="D23" s="61" t="inlineStr"/>
-      <c r="E23" s="61" t="inlineStr">
+      <c r="D23" s="60" t="inlineStr"/>
+      <c r="E23" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F23" s="61" t="inlineStr">
+      <c r="F23" s="60" t="inlineStr">
         <is>
           <t>SFM-038.C1
 SFM-038.C2</t>
         </is>
       </c>
-      <c r="G23" s="61" t="inlineStr"/>
-      <c r="H23" s="61" t="inlineStr"/>
-      <c r="I23" s="61" t="inlineStr"/>
+      <c r="G23" s="60" t="inlineStr"/>
+      <c r="H23" s="60" t="inlineStr"/>
+      <c r="I23" s="60" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I23"/>
@@ -19280,50 +19277,50 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Element</t>
         </is>
       </c>
-      <c r="B1" s="60" t="inlineStr">
+      <c r="B1" s="59" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="60" t="inlineStr">
+      <c r="C1" s="59" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="D1" s="60" t="inlineStr">
+      <c r="D1" s="59" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="E1" s="60" t="inlineStr">
+      <c r="E1" s="59" t="inlineStr">
         <is>
           <t>Functions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="222" customHeight="1">
-      <c r="A2" s="61" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="B2" s="61" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
         </is>
       </c>
-      <c r="C2" s="61" t="inlineStr">
+      <c r="C2" s="60" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D2" s="61" t="inlineStr"/>
-      <c r="E2" s="61" t="inlineStr">
+      <c r="D2" s="60" t="inlineStr"/>
+      <c r="E2" s="60" t="inlineStr">
         <is>
           <t>SFM-FN-001: F1 Lateral control: request steering torque from the EPS to keep the vehicle in its lane while engaged
 SFM-FN-002: F2 Longitudinal control: request acceleration/deceleration to hold set speed and follow leads while engaged
@@ -19337,398 +19334,398 @@
       </c>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="61" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="B3" s="61" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">    comma 3X device</t>
         </is>
       </c>
-      <c r="C3" s="61" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="D3" s="61" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E3" s="61" t="inlineStr"/>
+      <c r="E3" s="60" t="inlineStr"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="61" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-003</t>
         </is>
       </c>
-      <c r="B4" s="61" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Integrated panda (CAN interface and safety model)</t>
         </is>
       </c>
-      <c r="C4" s="61" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>subsystem</t>
         </is>
       </c>
-      <c r="D4" s="61" t="inlineStr">
+      <c r="D4" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E4" s="61" t="inlineStr"/>
+      <c r="E4" s="60" t="inlineStr"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-004</t>
         </is>
       </c>
-      <c r="B5" s="61" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">    Harness (Toyota A connector, harness box, comma power v3)</t>
         </is>
       </c>
-      <c r="C5" s="61" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
         <is>
           <t>component</t>
         </is>
       </c>
-      <c r="D5" s="61" t="inlineStr">
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E5" s="61" t="inlineStr"/>
+      <c r="E5" s="60" t="inlineStr"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-010</t>
         </is>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Perception (camerad, modeld)</t>
         </is>
       </c>
-      <c r="C6" s="61" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D6" s="61" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E6" s="61" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-011</t>
         </is>
       </c>
-      <c r="B7" s="61" t="inlineStr">
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Localization and calibration (locationd, calibrationd, paramsd, torqued)</t>
         </is>
       </c>
-      <c r="C7" s="61" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D7" s="61" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E7" s="61" t="inlineStr"/>
+      <c r="E7" s="60" t="inlineStr"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-012</t>
         </is>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Planning (plannerd, radard)</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D8" s="61" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E8" s="61" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-013</t>
         </is>
       </c>
-      <c r="B9" s="61" t="inlineStr">
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Control (controlsd, lateral/longitudinal controllers)</t>
         </is>
       </c>
-      <c r="C9" s="61" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D9" s="61" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E9" s="61" t="inlineStr"/>
+      <c r="E9" s="60" t="inlineStr"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-014</t>
         </is>
       </c>
-      <c r="B10" s="61" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Supervision (selfdrived state machine, events, alert manager)</t>
         </is>
       </c>
-      <c r="C10" s="61" t="inlineStr">
+      <c r="C10" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D10" s="61" t="inlineStr">
+      <c r="D10" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E10" s="61" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-015</t>
         </is>
       </c>
-      <c r="B11" s="61" t="inlineStr">
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Driver monitoring (dmonitoringmodeld, dmonitoringd)</t>
         </is>
       </c>
-      <c r="C11" s="61" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D11" s="61" t="inlineStr">
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E11" s="61" t="inlineStr"/>
+      <c r="E11" s="60" t="inlineStr"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="61" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-016</t>
         </is>
       </c>
-      <c r="B12" s="61" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Car interface (card, car_events, opendbc Toyota port)</t>
         </is>
       </c>
-      <c r="C12" s="61" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D12" s="61" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E12" s="61" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="61" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-017</t>
         </is>
       </c>
-      <c r="B13" s="61" t="inlineStr">
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Panda daemon (pandad)</t>
         </is>
       </c>
-      <c r="C13" s="61" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D13" s="61" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E13" s="61" t="inlineStr"/>
+      <c r="E13" s="60" t="inlineStr"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="61" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-018</t>
         </is>
       </c>
-      <c r="B14" s="61" t="inlineStr">
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        HMI (ui, soundd)</t>
         </is>
       </c>
-      <c r="C14" s="61" t="inlineStr">
+      <c r="C14" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D14" s="61" t="inlineStr">
+      <c r="D14" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E14" s="61" t="inlineStr"/>
+      <c r="E14" s="60" t="inlineStr"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="61" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-019</t>
         </is>
       </c>
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">        Platform (manager, messaging, hardwared, OS)</t>
         </is>
       </c>
-      <c r="C15" s="61" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D15" s="61" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E15" s="61" t="inlineStr"/>
+      <c r="E15" s="60" t="inlineStr"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="61" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-030</t>
         </is>
       </c>
-      <c r="B16" s="61" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>Toyota EPS</t>
         </is>
       </c>
-      <c r="C16" s="61" t="inlineStr">
+      <c r="C16" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D16" s="61" t="inlineStr"/>
-      <c r="E16" s="61" t="inlineStr"/>
+      <c r="D16" s="60" t="inlineStr"/>
+      <c r="E16" s="60" t="inlineStr"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="61" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-031</t>
         </is>
       </c>
-      <c r="B17" s="61" t="inlineStr">
+      <c r="B17" s="60" t="inlineStr">
         <is>
           <t>Toyota powertrain and brake control (receives ACC acceleration requests)</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D17" s="61" t="inlineStr"/>
-      <c r="E17" s="61" t="inlineStr"/>
+      <c r="D17" s="60" t="inlineStr"/>
+      <c r="E17" s="60" t="inlineStr"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="61" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-032</t>
         </is>
       </c>
-      <c r="B18" s="61" t="inlineStr">
+      <c r="B18" s="60" t="inlineStr">
         <is>
           <t>Toyota stock ADAS camera (TSS2)</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr">
+      <c r="C18" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D18" s="61" t="inlineStr"/>
-      <c r="E18" s="61" t="inlineStr"/>
+      <c r="D18" s="60" t="inlineStr"/>
+      <c r="E18" s="60" t="inlineStr"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="61" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-033</t>
         </is>
       </c>
-      <c r="B19" s="61" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>Vehicle CAN buses and 12 V supply</t>
         </is>
       </c>
-      <c r="C19" s="61" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D19" s="61" t="inlineStr"/>
-      <c r="E19" s="61" t="inlineStr"/>
+      <c r="D19" s="60" t="inlineStr"/>
+      <c r="E19" s="60" t="inlineStr"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="61" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr">
         <is>
           <t>SFM-SE-034</t>
         </is>
       </c>
-      <c r="B20" s="61" t="inlineStr">
+      <c r="B20" s="60" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C20" s="61" t="inlineStr">
+      <c r="C20" s="60" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D20" s="61" t="inlineStr"/>
-      <c r="E20" s="61" t="inlineStr"/>
+      <c r="D20" s="60" t="inlineStr"/>
+      <c r="E20" s="60" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E20"/>
@@ -19764,7 +19761,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>FMEA-MSR (monitoring and system response, msr-plan.md): S, F, M and MSR AP per rating-tables.md §7 (RT-2). The MSR AP table is provisional until the handbook table is transcribed (decision register DQ-207). Exempt causes are rated in the FMEA named in the reason.</t>
         </is>
@@ -22521,7 +22518,7 @@
           <t>Device power loss (12 V interruption, harness connector)</t>
         </is>
       </c>
-      <c r="E44" s="64" t="inlineStr">
+      <c r="E44" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-012.C1)</t>
         </is>
@@ -23242,7 +23239,7 @@
       </c>
       <c r="N55" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-005 · decision pending</t>
+          <t>SFM-ACT-005 · open</t>
         </is>
       </c>
       <c r="O55" s="37" t="inlineStr"/>
@@ -23304,7 +23301,7 @@
       </c>
       <c r="N56" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-005 · decision pending</t>
+          <t>SFM-ACT-005 · open</t>
         </is>
       </c>
       <c r="O56" s="37" t="inlineStr"/>
@@ -23643,7 +23640,7 @@
           <t>Panda MCU hardware fault (see DFMEA/FMEDA)</t>
         </is>
       </c>
-      <c r="E62" s="64" t="inlineStr">
+      <c r="E62" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-001.C1)</t>
         </is>
@@ -23803,7 +23800,7 @@
           <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
         </is>
       </c>
-      <c r="E65" s="64" t="inlineStr">
+      <c r="E65" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-010.C1)</t>
         </is>
@@ -23839,7 +23836,7 @@
           <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
         </is>
       </c>
-      <c r="E66" s="64" t="inlineStr">
+      <c r="E66" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-011.C1)</t>
         </is>
@@ -24315,7 +24312,7 @@
           <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
         </is>
       </c>
-      <c r="E74" s="64" t="inlineStr">
+      <c r="E74" s="63" t="inlineStr">
         <is>
           <t>Exempt: The cause is a defect of the warning path itself; its effect on detecting the lateral loss is rated in the MSR rows of SFM-004.C2 and SFM-005 (msr-plan §3)</t>
         </is>
@@ -24351,7 +24348,7 @@
           <t>pandad publishes the panda fields epsFault and requestsRejected (pandad.cc:137-138), but no SoC process reads them (txRateExceeded is read, TSR-615), so a panda-side EPS-fault refusal reaches the driver only through the panda siren and the stock EPS path (SW FMEA SWF-025 notes)</t>
         </is>
       </c>
-      <c r="E75" s="64" t="inlineStr">
+      <c r="E75" s="63" t="inlineStr">
         <is>
           <t>Exempt: The cause is a defect of the warning path itself; the panda siren that remains is rated on SFM-005 and in the DFMEA (msr-plan §3)</t>
         </is>
@@ -24387,7 +24384,7 @@
           <t>steerSaturated needs the controller saturated, a desired lateral acceleration above 1.0 m/s², an undershoot above 1.2x and no steering input for 2 s (selfdrived.py:465-479), and the controller reports saturation only after 0.4 s (latcontrol.py, T-30); a gradual deficit therefore warns late or not at all (WP-S-04 §3.8.1)</t>
         </is>
       </c>
-      <c r="E76" s="64" t="inlineStr">
+      <c r="E76" s="63" t="inlineStr">
         <is>
           <t>Exempt: The cause is the timing of the warning itself; it is rated as M 8 in the MSR rows of SFM-004.C1-C3 (rev 0.15, WP-S-04 §3.8.1)</t>
         </is>
@@ -24418,7 +24415,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.23 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.24 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.25: SFM-ACT-023 completed for the code (#174, DQ-342 A)
The lighter EPS-fault prompt after an override or at standstill now lasts
at most 1.5 s, then the take-over request (TSR-607 (b)); 6 unit tests in
CI, not verified on the vehicle. SFM-ACT-023 now covers SFM-038.C1 only
and carries predicted ratings (O 5, D 4, AP H); C1 keeps its BL-005
ratings until the next baseline. The host part (epsFault and
requestsRejected, SFM-038.C2) moves to the new open SFM-ACT-024.
AI-drafted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$93</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$76</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
@@ -261,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -410,6 +410,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -820,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.24 · draft</t>
+          <t>0.25 · draft</t>
         </is>
       </c>
     </row>
@@ -949,7 +952,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>22 (20)</t>
+          <t>23 (20)</t>
         </is>
       </c>
     </row>
@@ -17741,7 +17744,7 @@
       <c r="R90" s="45" t="inlineStr"/>
       <c r="S90" s="45" t="inlineStr"/>
     </row>
-    <row r="91" ht="168" customHeight="1">
+    <row r="91" ht="154.5" customHeight="1">
       <c r="A91" s="30" t="inlineStr">
         <is>
           <r>
@@ -17969,21 +17972,29 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Escalate every EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE), instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py:162-177; behaviour change queued for the lead by the FSC session as DQ-342), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
-          </r>
-        </is>
-      </c>
-      <c r="O91" s="47" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="P91" s="33" t="inlineStr"/>
-      <c r="Q91" s="33" t="inlineStr"/>
+            <t>Escalate a temporary EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE) instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py; lead decision DQ-342, option A: the lighter prompt for at most 1.5 s, then the take-over request; TSR-607 (b)). SFM-038.C1; FTA BE-2.08</t>
+          </r>
+        </is>
+      </c>
+      <c r="O91" s="54" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="P91" s="33" t="inlineStr">
+        <is>
+          <t>10/5/4</t>
+        </is>
+      </c>
+      <c r="Q91" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
       <c r="R91" s="37" t="inlineStr"/>
       <c r="S91" s="37" t="inlineStr"/>
     </row>
-    <row r="92" ht="168" customHeight="1">
+    <row r="92" ht="141" customHeight="1">
       <c r="A92" s="38" t="n"/>
       <c r="B92" s="38" t="n"/>
       <c r="C92" s="38" t="n"/>
@@ -18060,16 +18071,16 @@
               <color rgb="001F4E8C"/>
               <sz val="9"/>
             </rPr>
-            <t xml:space="preserve">SFM-ACT-023 · design change
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="001B2430"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Escalate every EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE), instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py:162-177; behaviour change queued for the lead by the FSC session as DQ-342), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+            <t xml:space="preserve">SFM-ACT-024 · monitoring
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)): raise the take-over request when the panda reports an EPS fault or refused steering frames while lateral control is engaged, within the SG-02 1 s budget, instead of relying on the panda siren alone. Split from SFM-ACT-023 (rev 0.25). SFM-038.C2; FTA BE-2.08</t>
           </r>
         </is>
       </c>
@@ -18401,7 +18412,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.24 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.25 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -18416,7 +18427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19222,7 +19233,7 @@
       <c r="H22" s="60" t="inlineStr"/>
       <c r="I22" s="60" t="inlineStr"/>
     </row>
-    <row r="23" ht="100.5" customHeight="1">
+    <row r="23" ht="141" customHeight="1">
       <c r="A23" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-023</t>
@@ -19235,27 +19246,69 @@
       </c>
       <c r="C23" s="60" t="inlineStr">
         <is>
-          <t>Escalate every EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE), instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py:162-177; behaviour change queued for the lead by the FSC session as DQ-342), and act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)). SFM-038.C1, C2; FTA BE-2.08</t>
+          <t>Escalate a temporary EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE) instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py; lead decision DQ-342, option A: the lighter prompt for at most 1.5 s, then the take-over request; TSR-607 (b)). SFM-038.C1; FTA BE-2.08</t>
         </is>
       </c>
       <c r="D23" s="60" t="inlineStr"/>
-      <c r="E23" s="60" t="inlineStr">
+      <c r="E23" s="61" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F23" s="60" t="inlineStr">
+        <is>
+          <t>SFM-038.C1</t>
+        </is>
+      </c>
+      <c r="G23" s="60" t="inlineStr">
+        <is>
+          <t>10/5/4</t>
+        </is>
+      </c>
+      <c r="H23" s="62" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="I23" s="60" t="inlineStr">
+        <is>
+          <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Not in BL-005, so SFM-038.C1 keeps O 8, D 10 until the next baseline; revised ratings below are a prediction (as SWF-ACT-025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="87" customHeight="1">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>SFM-ACT-024</t>
+        </is>
+      </c>
+      <c r="B24" s="60" t="inlineStr">
+        <is>
+          <t>monitoring</t>
+        </is>
+      </c>
+      <c r="C24" s="60" t="inlineStr">
+        <is>
+          <t>Act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)): raise the take-over request when the panda reports an EPS fault or refused steering frames while lateral control is engaged, within the SG-02 1 s budget, instead of relying on the panda siren alone. Split from SFM-ACT-023 (rev 0.25). SFM-038.C2; FTA BE-2.08</t>
+        </is>
+      </c>
+      <c r="D24" s="60" t="inlineStr"/>
+      <c r="E24" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F23" s="60" t="inlineStr">
-        <is>
-          <t>SFM-038.C1
-SFM-038.C2</t>
-        </is>
-      </c>
-      <c r="G23" s="60" t="inlineStr"/>
-      <c r="H23" s="60" t="inlineStr"/>
-      <c r="I23" s="60" t="inlineStr"/>
+      <c r="F24" s="60" t="inlineStr">
+        <is>
+          <t>SFM-038.C2</t>
+        </is>
+      </c>
+      <c r="G24" s="60" t="inlineStr"/>
+      <c r="H24" s="60" t="inlineStr"/>
+      <c r="I24" s="60" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I23"/>
+  <autoFilter ref="A1:I24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19761,7 +19814,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>FMEA-MSR (monitoring and system response, msr-plan.md): S, F, M and MSR AP per rating-tables.md §7 (RT-2). The MSR AP table is provisional until the handbook table is transcribed (decision register DQ-207). Exempt causes are rated in the FMEA named in the reason.</t>
         </is>
@@ -22518,7 +22571,7 @@
           <t>Device power loss (12 V interruption, harness connector)</t>
         </is>
       </c>
-      <c r="E44" s="63" t="inlineStr">
+      <c r="E44" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-012.C1)</t>
         </is>
@@ -23640,7 +23693,7 @@
           <t>Panda MCU hardware fault (see DFMEA/FMEDA)</t>
         </is>
       </c>
-      <c r="E62" s="63" t="inlineStr">
+      <c r="E62" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-001.C1)</t>
         </is>
@@ -23800,7 +23853,7 @@
           <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
         </is>
       </c>
-      <c r="E65" s="63" t="inlineStr">
+      <c r="E65" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-010.C1)</t>
         </is>
@@ -23836,7 +23889,7 @@
           <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
         </is>
       </c>
-      <c r="E66" s="63" t="inlineStr">
+      <c r="E66" s="64" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-011.C1)</t>
         </is>
@@ -24312,7 +24365,7 @@
           <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
         </is>
       </c>
-      <c r="E74" s="63" t="inlineStr">
+      <c r="E74" s="64" t="inlineStr">
         <is>
           <t>Exempt: The cause is a defect of the warning path itself; its effect on detecting the lateral loss is rated in the MSR rows of SFM-004.C2 and SFM-005 (msr-plan §3)</t>
         </is>
@@ -24348,7 +24401,7 @@
           <t>pandad publishes the panda fields epsFault and requestsRejected (pandad.cc:137-138), but no SoC process reads them (txRateExceeded is read, TSR-615), so a panda-side EPS-fault refusal reaches the driver only through the panda siren and the stock EPS path (SW FMEA SWF-025 notes)</t>
         </is>
       </c>
-      <c r="E75" s="63" t="inlineStr">
+      <c r="E75" s="64" t="inlineStr">
         <is>
           <t>Exempt: The cause is a defect of the warning path itself; the panda siren that remains is rated on SFM-005 and in the DFMEA (msr-plan §3)</t>
         </is>
@@ -24384,7 +24437,7 @@
           <t>steerSaturated needs the controller saturated, a desired lateral acceleration above 1.0 m/s², an undershoot above 1.2x and no steering input for 2 s (selfdrived.py:465-479), and the controller reports saturation only after 0.4 s (latcontrol.py, T-30); a gradual deficit therefore warns late or not at all (WP-S-04 §3.8.1)</t>
         </is>
       </c>
-      <c r="E76" s="63" t="inlineStr">
+      <c r="E76" s="64" t="inlineStr">
         <is>
           <t>Exempt: The cause is the timing of the warning itself; it is rated as M 8 in the MSR rows of SFM-004.C1-C3 (rev 0.15, WP-S-04 §3.8.1)</t>
         </is>
@@ -24415,7 +24468,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.24 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.25 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Baseline BL-006 proposed; System FMEA rev 0.27 moves to BL-006
BL-006: liondriver-dev c61e31b (#186), panda 0a7da85, opendbc 62b89a3.
Adds over BL-005 the EPS-fault prompt limit (TSR-607 (b)/(c)), opendbc
#15-#18 (ATC-20, DQ-079/080, SM-F1, wrong-length RX fault) and the
panda relay-malfunction latch (DFA DM-25).

System FMEA rev 0.27 at BL-006: SFM-038.C1 O 8 -> 5, D 10 -> 4 (AP H),
with `previous` keeping the BL-005 rating; SFM-ACT-023 credited.
Evidence only on SFM-013.C1/C2 and SFM-017.C1; mechanism text on
SFM-029 and SFM-034. The other analyses stay on their baselines.
Stacked on #185. AI-drafted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.26 · draft</t>
+          <t>0.27 · draft</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>BL-005</t>
+          <t>BL-006</t>
         </is>
       </c>
     </row>
@@ -18015,7 +18015,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
+            <t>The lighter EPS-fault prompt (steerTempUnavailableSilent, a LOW-priority WARNING with a chime and no soft disable, events.py:516-521) after a recent override, at standstill or while the driver steers is not limited to 1.5 s, so a long fault does not escalate to the take-over request (car_events.py:167-185, STEER_FAULT_SILENT_FRAMES; T-25, GAP-03). Until BL-005 the prompt was latched for the whole fault by design; from BL-006 the cause is a defect of the TSR-607 (b)/(c) frame counter</t>
           </r>
         </is>
       </c>
@@ -18027,7 +18027,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Upstream openpilot design choice (a softer alert after an override); no LionDriver requirement on it</t>
+            <t>• TSR-607 (b)/(c) implemented in car_events.py (#174, f350f5b; DQ-342 A, DQ-366 A): the lighter prompt is allowed for the first 150 frames of the fault only; ruff and ty in fork CI; impact record change-2026-10-17-eps-fault-escalation.md. Not reviewed independently</t>
           </r>
           <r>
             <rPr>
@@ -18041,22 +18041,31 @@
         </is>
       </c>
       <c r="J92" s="35" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K92" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="008A5A00"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• No LionDriver test targets this cause</t>
-          </r>
-        </is>
-      </c>
-      <c r="L92" s="46" t="n">
-        <v>10</v>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• test_steer_fault_warning.py (7 tests: silent window, no recent override, escalation after an override, at standstill, after releasing the wheel, a returning fault, a short fault while holding), run by the CI test runner; 4 of the #174 tests fail on the BL-005 code. Not proven by mutation; not verified on the vehicle (impact record OI-1)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/car/tests/test_steer_fault_warning.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L92" s="35" t="n">
+        <v>4</v>
       </c>
       <c r="M92" s="36" t="inlineStr">
         <is>
@@ -18521,7 +18530,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.26 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.27 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -19346,7 +19355,7 @@
       <c r="H22" s="60" t="inlineStr"/>
       <c r="I22" s="60" t="inlineStr"/>
     </row>
-    <row r="23" ht="141" customHeight="1">
+    <row r="23" ht="154.5" customHeight="1">
       <c r="A23" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-023</t>
@@ -19385,7 +19394,7 @@
       </c>
       <c r="I23" s="60" t="inlineStr">
         <is>
-          <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Not in BL-005, so SFM-038.C1 keeps O 8, D 10 until the next baseline; revised ratings below are a prediction (as SWF-ACT-025)</t>
+          <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Credited at BL-006 (System FMEA rev 0.27): SFM-038.C1 O 8 -&gt; 5, D 10 -&gt; 4, AP stays H (S 10); f350f5b adds TSR-607 (c) for a fault while the driver steers</t>
         </is>
       </c>
     </row>
@@ -24495,7 +24504,7 @@
       <c r="O74" s="37" t="inlineStr"/>
       <c r="P74" s="37" t="inlineStr"/>
     </row>
-    <row r="75" ht="141" customHeight="1">
+    <row r="75" ht="195" customHeight="1">
       <c r="A75" s="34" t="inlineStr">
         <is>
           <t>SFM-038 · Warning of a lateral-control fault or limit late, not escalated or missing</t>
@@ -24511,7 +24520,7 @@
       </c>
       <c r="D75" s="34" t="inlineStr">
         <is>
-          <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
+          <t>The lighter EPS-fault prompt (steerTempUnavailableSilent, a LOW-priority WARNING with a chime and no soft disable, events.py:516-521) after a recent override, at standstill or while the driver steers is not limited to 1.5 s, so a long fault does not escalate to the take-over request (car_events.py:167-185, STEER_FAULT_SILENT_FRAMES; T-25, GAP-03). Until BL-005 the prompt was latched for the whole fault by design; from BL-006 the cause is a defect of the TSR-607 (b)/(c) frame counter</t>
         </is>
       </c>
       <c r="E75" s="64" t="inlineStr">
@@ -24617,7 +24626,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.26 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.27 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
SFM-038.C1 links SW FMEA SWF-088 (#187); merge #185 head and liondriver-dev
SWF-088 (EPS-fault warning held at the low-priority prompt) is the SW
FMEA counterpart of SFM-038.C1. The SW FMEA still rates it at BL-005
(O 8, D 10); this row is rated at BL-006, so the inherited-rating check
warns until the SW FMEA moves to BL-006 (rationale says so).
Generated outputs regenerated after the merge.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.26 · draft</t>
+          <t>0.27 · draft</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>BL-005</t>
+          <t>BL-006</t>
         </is>
       </c>
     </row>
@@ -18015,7 +18015,16 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
+            <t>The lighter EPS-fault prompt (steerTempUnavailableSilent, a LOW-priority WARNING with a chime and no soft disable, events.py:516-521) after a recent override, at standstill or while the driver steers is not limited to 1.5 s, so a long fault does not escalate to the take-over request (car_events.py:167-185, STEER_FAULT_SILENT_FRAMES; T-25, GAP-03). Until BL-005 the prompt was latched for the whole fault by design; from BL-006 the cause is a defect of the TSR-607 (b)/(c) frame counter</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+linked: SWF-088</t>
           </r>
         </is>
       </c>
@@ -18027,7 +18036,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Upstream openpilot design choice (a softer alert after an override); no LionDriver requirement on it</t>
+            <t>• TSR-607 (b)/(c) implemented in car_events.py (#174, f350f5b; DQ-342 A, DQ-366 A): the lighter prompt is allowed for the first 150 frames of the fault only; ruff and ty in fork CI; impact record change-2026-10-17-eps-fault-escalation.md. Not reviewed independently</t>
           </r>
           <r>
             <rPr>
@@ -18041,22 +18050,31 @@
         </is>
       </c>
       <c r="J92" s="35" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K92" s="34" t="inlineStr">
         <is>
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="008A5A00"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• No LionDriver test targets this cause</t>
-          </r>
-        </is>
-      </c>
-      <c r="L92" s="46" t="n">
-        <v>10</v>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• test_steer_fault_warning.py (7 tests: silent window, no recent override, escalation after an override, at standstill, after releasing the wheel, a returning fault, a short fault while holding), run by the CI test runner; 4 of the #174 tests fail on the BL-005 code. Not proven by mutation; not verified on the vehicle (impact record OI-1)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/car/tests/test_steer_fault_warning.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="L92" s="35" t="n">
+        <v>4</v>
       </c>
       <c r="M92" s="36" t="inlineStr">
         <is>
@@ -18521,7 +18539,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.26 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.27 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -19346,7 +19364,7 @@
       <c r="H22" s="60" t="inlineStr"/>
       <c r="I22" s="60" t="inlineStr"/>
     </row>
-    <row r="23" ht="141" customHeight="1">
+    <row r="23" ht="154.5" customHeight="1">
       <c r="A23" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-023</t>
@@ -19385,7 +19403,7 @@
       </c>
       <c r="I23" s="60" t="inlineStr">
         <is>
-          <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Not in BL-005, so SFM-038.C1 keeps O 8, D 10 until the next baseline; revised ratings below are a prediction (as SWF-ACT-025)</t>
+          <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Credited at BL-006 (System FMEA rev 0.27): SFM-038.C1 O 8 -&gt; 5, D 10 -&gt; 4, AP stays H (S 10); f350f5b adds TSR-607 (c) for a fault while the driver steers</t>
         </is>
       </c>
     </row>
@@ -24495,7 +24513,7 @@
       <c r="O74" s="37" t="inlineStr"/>
       <c r="P74" s="37" t="inlineStr"/>
     </row>
-    <row r="75" ht="141" customHeight="1">
+    <row r="75" ht="195" customHeight="1">
       <c r="A75" s="34" t="inlineStr">
         <is>
           <t>SFM-038 · Warning of a lateral-control fault or limit late, not escalated or missing</t>
@@ -24511,7 +24529,7 @@
       </c>
       <c r="D75" s="34" t="inlineStr">
         <is>
-          <t>After any driver steering input in the last 1.5 s, or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent (a LOW-priority WARNING with a prompt chime and no soft disable, events.py:516-521), and it stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; T-25, GAP-03)</t>
+          <t>The lighter EPS-fault prompt (steerTempUnavailableSilent, a LOW-priority WARNING with a chime and no soft disable, events.py:516-521) after a recent override, at standstill or while the driver steers is not limited to 1.5 s, so a long fault does not escalate to the take-over request (car_events.py:167-185, STEER_FAULT_SILENT_FRAMES; T-25, GAP-03). Until BL-005 the prompt was latched for the whole fault by design; from BL-006 the cause is a defect of the TSR-607 (b)/(c) frame counter</t>
         </is>
       </c>
       <c r="E75" s="64" t="inlineStr">
@@ -24617,7 +24635,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.26 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.27 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
SFM-038.C1 D 8, not D 4: the EPS-fault tests are not yet proven by mutation
Rating tables D 8 (targeted test, not proven) applies, as the SW FMEA
rates every host row; D 4 needs a proven method. O 5, AP H unchanged.
SFM-ACT-023 revised D and evidence corrected; a car_events.py mutation
run (planned with SWF-ACT-077) would support D 4 later. Raised by the
SW FMEA session via the coordinator.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -17853,7 +17853,7 @@
       <c r="R91" s="45" t="inlineStr"/>
       <c r="S91" s="45" t="inlineStr"/>
     </row>
-    <row r="92" ht="154.5" customHeight="1">
+    <row r="92" ht="168" customHeight="1">
       <c r="A92" s="30" t="inlineStr">
         <is>
           <r>
@@ -18060,7 +18060,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_steer_fault_warning.py (7 tests: silent window, no recent override, escalation after an override, at standstill, after releasing the wheel, a returning fault, a short fault while holding), run by the CI test runner; 4 of the #174 tests fail on the BL-005 code. Not proven by mutation; not verified on the vehicle (impact record OI-1)</t>
+            <t>• test_steer_fault_warning.py (7 tests: silent window, no recent override, escalation after an override, at standstill, after releasing the wheel, a returning fault, a short fault while holding), run by the CI test runner; 4 of the #174 tests fail on the BL-005 code. Targeted but not proven by mutation, so D 8 (RT-2); not verified on the vehicle (impact record OI-1)</t>
           </r>
           <r>
             <rPr>
@@ -18074,7 +18074,7 @@
         </is>
       </c>
       <c r="L92" s="35" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M92" s="36" t="inlineStr">
         <is>
@@ -18110,7 +18110,7 @@
       </c>
       <c r="P92" s="33" t="inlineStr">
         <is>
-          <t>10/5/4</t>
+          <t>10/5/8</t>
         </is>
       </c>
       <c r="Q92" s="36" t="inlineStr">
@@ -19364,7 +19364,7 @@
       <c r="H22" s="60" t="inlineStr"/>
       <c r="I22" s="60" t="inlineStr"/>
     </row>
-    <row r="23" ht="154.5" customHeight="1">
+    <row r="23" ht="195" customHeight="1">
       <c r="A23" s="60" t="inlineStr">
         <is>
           <t>SFM-ACT-023</t>
@@ -19393,7 +19393,7 @@
       </c>
       <c r="G23" s="60" t="inlineStr">
         <is>
-          <t>10/5/4</t>
+          <t>10/5/8</t>
         </is>
       </c>
       <c r="H23" s="62" t="inlineStr">
@@ -19403,7 +19403,7 @@
       </c>
       <c r="I23" s="60" t="inlineStr">
         <is>
-          <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Credited at BL-006 (System FMEA rev 0.27): SFM-038.C1 O 8 -&gt; 5, D 10 -&gt; 4, AP stays H (S 10); f350f5b adds TSR-607 (c) for a fault while the driver steers</t>
+          <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Credited at BL-006 (System FMEA rev 0.27): SFM-038.C1 O 8 -&gt; 5, D 10 -&gt; 8, AP stays H (S 10): the tests are targeted but not proven by mutation, so D 8 rather than the D 4 predicted below (rating tables D 8; a car_events.py mutation run, planned with SWF-ACT-077, would support D 4); f350f5b adds TSR-607 (c) for a fault while the driver steers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
System FMEA rev 0.28: SFM-034 latch mechanism cites SWF-090
The BL-006 relay-malfunction latch line on SFM-034 now names its SW FMEA
failure mode, SWF-090 (#196, O 3 D 4 at BL-006). SWF-088 is O 5 D 8 at
BL-006, matching SFM-038.C1, so the inherited-rating warnings are gone.
No rating change. AI-drafted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.27 · draft</t>
+          <t>0.28 · draft</t>
         </is>
       </c>
     </row>
@@ -18539,7 +18539,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.27 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.28 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -24635,7 +24635,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.27 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.28 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.29: SFM-ACT-020 open per DQ-300 A (stand down during stock AEB)
The lead decided DQ-300 option A on 2026-10-18: while the car reports
a stock PCS/AEB event, LionDriver requests zero acceleration; the
AOU-04R vehicle test still runs. SFM-ACT-020 moves from
decision_pending to open with that behaviour; SFM-036 notes updated.
Not implemented at BL-006, so SFM-036 keeps its ratings. AI-drafted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -261,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -399,9 +399,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -823,7 +820,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.28 · draft</t>
+          <t>0.29 · draft</t>
         </is>
       </c>
     </row>
@@ -17033,7 +17030,7 @@
       <c r="R86" s="45" t="inlineStr"/>
       <c r="S86" s="45" t="inlineStr"/>
     </row>
-    <row r="87" ht="127.5" customHeight="1">
+    <row r="87" ht="141" customHeight="1">
       <c r="A87" s="30" t="inlineStr">
         <is>
           <r>
@@ -17261,13 +17258,13 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
-          </r>
-        </is>
-      </c>
-      <c r="O87" s="58" t="inlineStr">
-        <is>
-          <t>decision pending</t>
+            <t>Stand down during stock AEB: while the car reports a stock PCS/AEB event (stockAeb), LionDriver requests zero acceleration, so stock AEB does not depend on PCM arbitration alone (AOU-04R). Lead decision DQ-300, option A (2026-10-18); the AOU-04R vehicle test still runs. Code change with the implementation-spec session; not in BL-006, so SFM-036 keeps its ratings</t>
+          </r>
+        </is>
+      </c>
+      <c r="O87" s="47" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
       <c r="P87" s="33" t="inlineStr"/>
@@ -18539,7 +18536,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.28 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.29 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -18569,79 +18566,79 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="59" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="B1" s="59" t="inlineStr">
+      <c r="B1" s="58" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="C1" s="59" t="inlineStr">
+      <c r="C1" s="58" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="59" t="inlineStr">
+      <c r="D1" s="58" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E1" s="59" t="inlineStr">
+      <c r="E1" s="58" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="59" t="inlineStr">
+      <c r="F1" s="58" t="inlineStr">
         <is>
           <t>Causes</t>
         </is>
       </c>
-      <c r="G1" s="59" t="inlineStr">
+      <c r="G1" s="58" t="inlineStr">
         <is>
           <t>Revised S/O/D</t>
         </is>
       </c>
-      <c r="H1" s="59" t="inlineStr">
+      <c r="H1" s="58" t="inlineStr">
         <is>
           <t>Revised AP</t>
         </is>
       </c>
-      <c r="I1" s="59" t="inlineStr">
+      <c r="I1" s="58" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
     </row>
     <row r="2" ht="127.5" customHeight="1">
-      <c r="A2" s="60" t="inlineStr">
+      <c r="A2" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-001</t>
         </is>
       </c>
-      <c r="B2" s="60" t="inlineStr">
+      <c r="B2" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C2" s="60" t="inlineStr">
+      <c r="C2" s="59" t="inlineStr">
         <is>
           <t>Derive steering and acceleration envelopes from measurements on the reference vehicle and set the panda limits from them, independently of the SoC limits (same as SWF-ACT-003, FSC FOI-001)</t>
         </is>
       </c>
-      <c r="D2" s="60" t="inlineStr">
+      <c r="D2" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E2" s="60" t="inlineStr">
+      <c r="E2" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F2" s="60" t="inlineStr">
+      <c r="F2" s="59" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
@@ -18654,37 +18651,37 @@
 SFM-029.C2</t>
         </is>
       </c>
-      <c r="G2" s="60" t="inlineStr"/>
-      <c r="H2" s="60" t="inlineStr"/>
-      <c r="I2" s="60" t="inlineStr"/>
+      <c r="G2" s="59" t="inlineStr"/>
+      <c r="H2" s="59" t="inlineStr"/>
+      <c r="I2" s="59" t="inlineStr"/>
     </row>
     <row r="3" ht="168" customHeight="1">
-      <c r="A3" s="60" t="inlineStr">
+      <c r="A3" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-002</t>
         </is>
       </c>
-      <c r="B3" s="60" t="inlineStr">
+      <c r="B3" s="59" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C3" s="60" t="inlineStr">
+      <c r="C3" s="59" t="inlineStr">
         <is>
           <t>Requirements-based tests for the host safety-relevant functions (selfdrived, controlsd, pandad, car interface, locationd bounds, monitoring policy), proven by mutation or fault injection and run as a CI gate (see SWF host actions)</t>
         </is>
       </c>
-      <c r="D3" s="60" t="inlineStr">
+      <c r="D3" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E3" s="60" t="inlineStr">
+      <c r="E3" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F3" s="60" t="inlineStr">
+      <c r="F3" s="59" t="inlineStr">
         <is>
           <t>SFM-002.C4
 SFM-004.C3
@@ -18700,37 +18697,37 @@
 SFM-037.C3</t>
         </is>
       </c>
-      <c r="G3" s="60" t="inlineStr"/>
-      <c r="H3" s="60" t="inlineStr"/>
-      <c r="I3" s="60" t="inlineStr"/>
+      <c r="G3" s="59" t="inlineStr"/>
+      <c r="H3" s="59" t="inlineStr"/>
+      <c r="I3" s="59" t="inlineStr"/>
     </row>
     <row r="4" ht="343.5" customHeight="1">
-      <c r="A4" s="60" t="inlineStr">
+      <c r="A4" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-003</t>
         </is>
       </c>
-      <c r="B4" s="60" t="inlineStr">
+      <c r="B4" s="59" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C4" s="60" t="inlineStr">
+      <c r="C4" s="59" t="inlineStr">
         <is>
           <t>Execute system integration and vehicle verification on the reference car (WP-S-08, WP-S-09) and the HIL bench (D-04): steering sign and torque response, EPS and powertrain interface behaviour (lockouts, ignored requests), brake, accelerator and cancel paths, intercept-switch and harness faults, 12 V interruptions, alert latency and audibility, CPU-load soak</t>
         </is>
       </c>
-      <c r="D4" s="60" t="inlineStr">
+      <c r="D4" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E4" s="60" t="inlineStr">
+      <c r="E4" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F4" s="60" t="inlineStr">
+      <c r="F4" s="59" t="inlineStr">
         <is>
           <t>SFM-003.C1
 SFM-003.C2
@@ -18759,72 +18756,72 @@
 SFM-033.C3</t>
         </is>
       </c>
-      <c r="G4" s="60" t="inlineStr"/>
-      <c r="H4" s="60" t="inlineStr"/>
-      <c r="I4" s="60" t="inlineStr"/>
+      <c r="G4" s="59" t="inlineStr"/>
+      <c r="H4" s="59" t="inlineStr"/>
+      <c r="I4" s="59" t="inlineStr"/>
     </row>
     <row r="5" ht="154.5" customHeight="1">
-      <c r="A5" s="60" t="inlineStr">
+      <c r="A5" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-005</t>
         </is>
       </c>
-      <c r="B5" s="60" t="inlineStr">
+      <c r="B5" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C5" s="60" t="inlineStr">
+      <c r="C5" s="59" t="inlineStr">
         <is>
           <t>Implement the reaction when driver awareness reaches zero (driverUnresponsive3 / driverDistracted3 have no disable reaction at BL-004 or BL-005), the safe state of SG-010 (WP-C-03 SG-08, ASIL A; DQ-205). Decided by the lead (DQ-365, option A, 2026-10-16) and specified in TSR-633 (WP-S-02 v0.26) with TSR-611; keep the lane and decelerate in lane to a standstill with the terminal alert sounding, hold the vehicle stopped, and lock out re-engagement and resumption until the driver responds. WP-S-04 v0.12 §3.8.4 gives a preliminary time to the reaction (18 s vision, 30 s wheel-touch from loss of attention; OI-11); SFM-025.C1 is re-rated once TSR-633 is implemented and that time is confirmed</t>
         </is>
       </c>
-      <c r="D5" s="60" t="inlineStr">
+      <c r="D5" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E5" s="60" t="inlineStr">
+      <c r="E5" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F5" s="60" t="inlineStr">
+      <c r="F5" s="59" t="inlineStr">
         <is>
           <t>SFM-025.C1</t>
         </is>
       </c>
-      <c r="G5" s="60" t="inlineStr"/>
-      <c r="H5" s="60" t="inlineStr"/>
-      <c r="I5" s="60" t="inlineStr"/>
+      <c r="G5" s="59" t="inlineStr"/>
+      <c r="H5" s="59" t="inlineStr"/>
+      <c r="I5" s="59" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-006</t>
         </is>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="59" t="inlineStr">
         <is>
           <t>detection</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>Establish on the reference car which stock TSS2 functions (PCS/AEB, FCW) remain available with LionDriver installed and longitudinal control enabled, and verify the stock pre-collision path after installation (PFMEA PFM-014)</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E6" s="60" t="inlineStr">
+      <c r="E6" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F6" s="60" t="inlineStr">
+      <c r="F6" s="59" t="inlineStr">
         <is>
           <t>SFM-010.C2
 SFM-033.C1
@@ -18832,37 +18829,37 @@
 SFM-036.C2</t>
         </is>
       </c>
-      <c r="G6" s="60" t="inlineStr"/>
-      <c r="H6" s="60" t="inlineStr"/>
-      <c r="I6" s="60" t="inlineStr"/>
+      <c r="G6" s="59" t="inlineStr"/>
+      <c r="H6" s="59" t="inlineStr"/>
+      <c r="I6" s="59" t="inlineStr"/>
     </row>
     <row r="7" ht="73.5" customHeight="1">
-      <c r="A7" s="60" t="inlineStr">
+      <c r="A7" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-007</t>
         </is>
       </c>
-      <c r="B7" s="60" t="inlineStr">
+      <c r="B7" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C7" s="60" t="inlineStr">
+      <c r="C7" s="59" t="inlineStr">
         <is>
           <t>Supervise the alert channels: treat loss of ui or soundd liveness, or a stale displayed state, as a fault that escalates (audible fallback, disengagement) instead of continuing silently</t>
         </is>
       </c>
-      <c r="D7" s="60" t="inlineStr">
+      <c r="D7" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E7" s="60" t="inlineStr">
+      <c r="E7" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F7" s="60" t="inlineStr">
+      <c r="F7" s="59" t="inlineStr">
         <is>
           <t>SFM-015.C1
 SFM-026.C1
@@ -18871,76 +18868,76 @@
 SFM-028.C1</t>
         </is>
       </c>
-      <c r="G7" s="60" t="inlineStr"/>
-      <c r="H7" s="60" t="inlineStr"/>
-      <c r="I7" s="60" t="inlineStr"/>
+      <c r="G7" s="59" t="inlineStr"/>
+      <c r="H7" s="59" t="inlineStr"/>
+      <c r="I7" s="59" t="inlineStr"/>
     </row>
     <row r="8" ht="73.5" customHeight="1">
-      <c r="A8" s="60" t="inlineStr">
+      <c r="A8" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-008</t>
         </is>
       </c>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="B8" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C8" s="60" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
           <t>Allow engagement only when the fingerprint, CarParams and panda safety parameter match the reference configuration AC-001 (refuse fuzzy matches in the reference build); see PFMEA PFM-013</t>
         </is>
       </c>
-      <c r="D8" s="60" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E8" s="60" t="inlineStr">
+      <c r="E8" s="59" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F8" s="60" t="inlineStr">
+      <c r="F8" s="59" t="inlineStr">
         <is>
           <t>SFM-032.C1</t>
         </is>
       </c>
-      <c r="G8" s="60" t="inlineStr"/>
-      <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr">
+      <c r="G8" s="59" t="inlineStr"/>
+      <c r="H8" s="59" t="inlineStr"/>
+      <c r="I8" s="59" t="inlineStr">
         <is>
           <t>BL-005: the reference build is the default (LionDriver #36), the panda accepts only TOYOTA parameter 73 (reference_lock.h) and pandad configures a car mode only on a reference panda (#41). Fuzzy fingerprint matches are still accepted on the host (SFM-032.C1)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="100.5" customHeight="1">
-      <c r="A9" s="60" t="inlineStr">
+      <c r="A9" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-009</t>
         </is>
       </c>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="B9" s="59" t="inlineStr">
         <is>
           <t>prevention</t>
         </is>
       </c>
-      <c r="C9" s="60" t="inlineStr">
+      <c r="C9" s="59" t="inlineStr">
         <is>
           <t>Produce SOTIF / ISO PAS 8800 evidence for the neural-network elements (driving model, lead detection, driver monitoring model) per WP-V-02..04, including fault-induced inputs (corrupted or stale frames)</t>
         </is>
       </c>
-      <c r="D9" s="60" t="inlineStr">
+      <c r="D9" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E9" s="60" t="inlineStr">
+      <c r="E9" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F9" s="60" t="inlineStr">
+      <c r="F9" s="59" t="inlineStr">
         <is>
           <t>SFM-002.C2
 SFM-003.C3
@@ -18951,37 +18948,37 @@
 SFM-022.C2</t>
         </is>
       </c>
-      <c r="G9" s="60" t="inlineStr"/>
-      <c r="H9" s="60" t="inlineStr"/>
-      <c r="I9" s="60" t="inlineStr"/>
+      <c r="G9" s="59" t="inlineStr"/>
+      <c r="H9" s="59" t="inlineStr"/>
+      <c r="I9" s="59" t="inlineStr"/>
     </row>
     <row r="10" ht="73.5" customHeight="1">
-      <c r="A10" s="60" t="inlineStr">
+      <c r="A10" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-010</t>
         </is>
       </c>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B10" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr">
         <is>
           <t>Justify every SOFT_DISABLE reaction and debounce against the FTTI (WP-S-04) and alert at once when the panda withdraws authority while engaged (controlsMismatch debounce)</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E10" s="60" t="inlineStr">
+      <c r="E10" s="59" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F10" s="60" t="inlineStr">
+      <c r="F10" s="59" t="inlineStr">
         <is>
           <t>SFM-014.C2
 SFM-015.C2
@@ -18989,454 +18986,454 @@
 SFM-016.C2</t>
         </is>
       </c>
-      <c r="G10" s="60" t="inlineStr"/>
-      <c r="H10" s="60" t="inlineStr"/>
-      <c r="I10" s="60" t="inlineStr">
+      <c r="G10" s="59" t="inlineStr"/>
+      <c r="H10" s="59" t="inlineStr"/>
+      <c r="I10" s="59" t="inlineStr">
         <is>
           <t>controlsMismatch debounce cut from 200 cumulative samples (~2 s) to 2 consecutive samples, at most 0.5 s (change-2026-10-13-host-supervision.md); credited at BL-005 (SFM-015.C2 M 6). FTTI justification of SOFT_DISABLE reactions open</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="60" t="inlineStr">
+      <c r="A11" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-011</t>
         </is>
       </c>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="B11" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C11" s="60" t="inlineStr">
+      <c r="C11" s="59" t="inlineStr">
         <is>
           <t>Alert the driver when stock cruise stays engaged while the item is disengaged (cruiseMismatch has no alert at BL-004)</t>
         </is>
       </c>
-      <c r="D11" s="60" t="inlineStr">
+      <c r="D11" s="59" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E11" s="61" t="inlineStr">
+      <c r="E11" s="60" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F11" s="60" t="inlineStr">
+      <c r="F11" s="59" t="inlineStr">
         <is>
           <t>SFM-021.C1
 SFM-021.C2</t>
         </is>
       </c>
-      <c r="G11" s="60" t="inlineStr"/>
-      <c r="H11" s="60" t="inlineStr"/>
-      <c r="I11" s="60" t="inlineStr">
+      <c r="G11" s="59" t="inlineStr"/>
+      <c r="H11" s="59" t="inlineStr"/>
+      <c r="I11" s="59" t="inlineStr">
         <is>
           <t>cruiseMismatch now alerts after 1 s (change-2026-10-13-host-supervision.md); see SWF-ACT-034</t>
         </is>
       </c>
     </row>
     <row r="12" ht="73.5" customHeight="1">
-      <c r="A12" s="60" t="inlineStr">
+      <c r="A12" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-012</t>
         </is>
       </c>
-      <c r="B12" s="60" t="inlineStr">
+      <c r="B12" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C12" s="59" t="inlineStr">
         <is>
           <t>Measure on the HIL bench and the reference car (WP-V-05) how the panda reacts to over-limit and not-engaged steering and acceleration frames and to driver brake, gas and cancel inputs, and what the EPS and PCM do when frames are refused; re-rate the MSR rows from code-derived to measured timing</t>
         </is>
       </c>
-      <c r="D12" s="60" t="inlineStr"/>
-      <c r="E12" s="60" t="inlineStr">
+      <c r="D12" s="59" t="inlineStr"/>
+      <c r="E12" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F12" s="60" t="inlineStr"/>
-      <c r="G12" s="60" t="inlineStr"/>
-      <c r="H12" s="60" t="inlineStr"/>
-      <c r="I12" s="60" t="inlineStr"/>
+      <c r="F12" s="59" t="inlineStr"/>
+      <c r="G12" s="59" t="inlineStr"/>
+      <c r="H12" s="59" t="inlineStr"/>
+      <c r="I12" s="59" t="inlineStr"/>
     </row>
     <row r="13" ht="87" customHeight="1">
-      <c r="A13" s="60" t="inlineStr">
+      <c r="A13" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-013</t>
         </is>
       </c>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C13" s="60" t="inlineStr">
+      <c r="C13" s="59" t="inlineStr">
         <is>
           <t>Check on the host, within the SG-01 FTTI, that the panda reports controls_allowed false while the item is disengaged (the reverse of the controlsMismatch check, which at BL-005 still covers only engaged with authority withdrawn), with a disable and an alert. The requirement is TSR-630, within 0.3 s (WP-S-02 §12.3a; WP-S-04 T-32, not implemented)</t>
         </is>
       </c>
-      <c r="D13" s="60" t="inlineStr"/>
-      <c r="E13" s="60" t="inlineStr">
+      <c r="D13" s="59" t="inlineStr"/>
+      <c r="E13" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F13" s="60" t="inlineStr"/>
-      <c r="G13" s="60" t="inlineStr"/>
-      <c r="H13" s="60" t="inlineStr"/>
-      <c r="I13" s="60" t="inlineStr"/>
+      <c r="F13" s="59" t="inlineStr"/>
+      <c r="G13" s="59" t="inlineStr"/>
+      <c r="H13" s="59" t="inlineStr"/>
+      <c r="I13" s="59" t="inlineStr"/>
     </row>
     <row r="14" ht="46.5" customHeight="1">
-      <c r="A14" s="60" t="inlineStr">
+      <c r="A14" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-014</t>
         </is>
       </c>
-      <c r="B14" s="60" t="inlineStr">
+      <c r="B14" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C14" s="60" t="inlineStr">
+      <c r="C14" s="59" t="inlineStr">
         <is>
           <t>Specify in the TSC a steering-direction plausibility monitor (commanded torque sign against measured yaw rate and lane-relative lateral motion), or justify its absence against HZ-003</t>
         </is>
       </c>
-      <c r="D14" s="60" t="inlineStr"/>
-      <c r="E14" s="60" t="inlineStr">
+      <c r="D14" s="59" t="inlineStr"/>
+      <c r="E14" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F14" s="60" t="inlineStr"/>
-      <c r="G14" s="60" t="inlineStr"/>
-      <c r="H14" s="60" t="inlineStr"/>
-      <c r="I14" s="60" t="inlineStr"/>
+      <c r="F14" s="59" t="inlineStr"/>
+      <c r="G14" s="59" t="inlineStr"/>
+      <c r="H14" s="59" t="inlineStr"/>
+      <c r="I14" s="59" t="inlineStr"/>
     </row>
     <row r="15" ht="100.5" customHeight="1">
-      <c r="A15" s="60" t="inlineStr">
+      <c r="A15" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-015</t>
         </is>
       </c>
-      <c r="B15" s="60" t="inlineStr">
+      <c r="B15" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C15" s="60" t="inlineStr">
+      <c r="C15" s="59" t="inlineStr">
         <is>
           <t>Detect stale commands and inputs within the SG-01 FTTI: command-frame freshness in the MCU with an active zero frame (TSR-408, TSR-109) and frozen-content and age checks on model outputs in controlsd (TSR-602, TSR-631, AIR-17)</t>
         </is>
       </c>
-      <c r="D15" s="60" t="inlineStr"/>
-      <c r="E15" s="60" t="inlineStr">
+      <c r="D15" s="59" t="inlineStr"/>
+      <c r="E15" s="59" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F15" s="60" t="inlineStr"/>
-      <c r="G15" s="60" t="inlineStr"/>
-      <c r="H15" s="60" t="inlineStr"/>
-      <c r="I15" s="60" t="inlineStr">
+      <c r="F15" s="59" t="inlineStr"/>
+      <c r="G15" s="59" t="inlineStr"/>
+      <c r="H15" s="59" t="inlineStr"/>
+      <c r="I15" s="59" t="inlineStr">
         <is>
           <t>BL-005: command-frame arrival in the MCU (TSR-408, 50 ms STEERING_LKA, reference build by default) and input age checks in controlsd (TSR-602) are in. Open: the active zero frame (TSR-109), a frozen-content check on model outputs, and stale data with fresh timestamps (SFM-006.C1 to C3). The frozen-content check is TSR-631, with the age taken from the source timestamp (WP-S-02 §12.3a)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="73.5" customHeight="1">
-      <c r="A16" s="60" t="inlineStr">
+      <c r="A16" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-016</t>
         </is>
       </c>
-      <c r="B16" s="60" t="inlineStr">
+      <c r="B16" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C16" s="60" t="inlineStr">
+      <c r="C16" s="59" t="inlineStr">
         <is>
           <t>Supervise driver override in the panda: driver steering torque above the override threshold limits or revokes lateral authority within the SG-05 0.2 s budget (TSR-304). Behaviour decided by the lead (DQ-053, option A): back off on override and show a cue. Requirements: TSR-304 (timing tied to the SG-05 budget) and TSR-628 (WP-S-02 §12.3a)</t>
         </is>
       </c>
-      <c r="D16" s="60" t="inlineStr"/>
-      <c r="E16" s="60" t="inlineStr">
+      <c r="D16" s="59" t="inlineStr"/>
+      <c r="E16" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F16" s="60" t="inlineStr">
+      <c r="F16" s="59" t="inlineStr">
         <is>
           <t>SFM-018.C3</t>
         </is>
       </c>
-      <c r="G16" s="60" t="inlineStr"/>
-      <c r="H16" s="60" t="inlineStr"/>
-      <c r="I16" s="60" t="inlineStr"/>
+      <c r="G16" s="59" t="inlineStr"/>
+      <c r="H16" s="59" t="inlineStr"/>
+      <c r="I16" s="59" t="inlineStr"/>
     </row>
     <row r="17" ht="87" customHeight="1">
-      <c r="A17" s="60" t="inlineStr">
+      <c r="A17" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-017</t>
         </is>
       </c>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="B17" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C17" s="60" t="inlineStr">
+      <c r="C17" s="59" t="inlineStr">
         <is>
           <t>Add WP-S-04 FTTI rows for the warning paths without one (insufficient lateral control, late or insufficient braking warnings, SG-008 unintended engagement, driver monitoring), so these mechanisms can be compared with a time budget</t>
         </is>
       </c>
-      <c r="D17" s="60" t="inlineStr"/>
-      <c r="E17" s="61" t="inlineStr">
+      <c r="D17" s="59" t="inlineStr"/>
+      <c r="E17" s="60" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F17" s="60" t="inlineStr"/>
-      <c r="G17" s="60" t="inlineStr"/>
-      <c r="H17" s="60" t="inlineStr"/>
-      <c r="I17" s="60" t="inlineStr">
+      <c r="F17" s="59" t="inlineStr"/>
+      <c r="G17" s="59" t="inlineStr"/>
+      <c r="H17" s="59" t="inlineStr"/>
+      <c r="I17" s="59" t="inlineStr">
         <is>
           <t>WP-S-04 v0.7 §3.7 (four rows) and §3.8, with T-30 to T-33. Rev 0.15 compares SFM-004, SFM-010.C2/C3, SFM-012.C1 and SFM-013.C1/C2 with them. Driver monitoring (SFM-022.C3, SFM-025.C1) waits for the H-09 FTTI (§3.8.4); follow-up is SFM-ACT-005. Late warnings found: SFM-ACT-021 (lateral) and SFM-ACT-022 (braking)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="100.5" customHeight="1">
-      <c r="A18" s="60" t="inlineStr">
+      <c r="A18" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-018</t>
         </is>
       </c>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="B18" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C18" s="60" t="inlineStr">
+      <c r="C18" s="59" t="inlineStr">
         <is>
           <t>Detect silent loss of the actuation path: report forwarded and refused TX frames from the panda, and compare EPS and PCM acceptance (LKA_STATE, ACC status) with the commands, warning within the SG-02/06 1 s budget</t>
         </is>
       </c>
-      <c r="D18" s="60" t="inlineStr"/>
-      <c r="E18" s="60" t="inlineStr">
+      <c r="D18" s="59" t="inlineStr"/>
+      <c r="E18" s="59" t="inlineStr">
         <is>
           <t>in progress</t>
         </is>
       </c>
-      <c r="F18" s="60" t="inlineStr"/>
-      <c r="G18" s="60" t="inlineStr"/>
-      <c r="H18" s="60" t="inlineStr"/>
-      <c r="I18" s="60" t="inlineStr">
+      <c r="F18" s="59" t="inlineStr"/>
+      <c r="G18" s="59" t="inlineStr"/>
+      <c r="H18" s="59" t="inlineStr"/>
+      <c r="I18" s="59" t="inlineStr">
         <is>
           <t>BL-005: frames that stop reaching the panda are detected (TSR-408) and alerted within 0.5 s (TSR-621), credited on SFM-005.C2 and SFM-011.C2. Open: frames that reach the panda but are not accepted by the EPS or PCM (SFM-005.C1, SFM-011.C1). Requirements: TSR-632 (per-ID transmitted and refused counts), TSR-626(d)/(e) (EPS and PCM acceptance status) and TSR-615, warning within 1 s (WP-S-02 §12.3a)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="60" t="inlineStr">
+      <c r="A19" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-019</t>
         </is>
       </c>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="B19" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="59" t="inlineStr">
         <is>
           <t>Revoke lateral authority in the panda when it rejects a steering frame while authority is granted, and keep it revoked until a new valid engagement (TSR-108; lead decision DQ-060, option A). At BL-005 the frame is dropped and only the host disengages (pandaTxBlocked)</t>
         </is>
       </c>
-      <c r="D19" s="60" t="inlineStr"/>
-      <c r="E19" s="60" t="inlineStr">
+      <c r="D19" s="59" t="inlineStr"/>
+      <c r="E19" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F19" s="60" t="inlineStr">
+      <c r="F19" s="59" t="inlineStr">
         <is>
           <t>SFM-002.C1
 SFM-002.C2
 SFM-002.C4</t>
         </is>
       </c>
-      <c r="G19" s="60" t="inlineStr"/>
-      <c r="H19" s="60" t="inlineStr"/>
-      <c r="I19" s="60" t="inlineStr"/>
+      <c r="G19" s="59" t="inlineStr"/>
+      <c r="H19" s="59" t="inlineStr"/>
+      <c r="I19" s="59" t="inlineStr"/>
     </row>
-    <row r="20" ht="73.5" customHeight="1">
-      <c r="A20" s="60" t="inlineStr">
+    <row r="20" ht="87" customHeight="1">
+      <c r="A20" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-020</t>
         </is>
       </c>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="B20" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
-        <is>
-          <t>React to a stock PCS event on the longitudinal command (for example a neutral or zero acceleration request, or a longitudinal disable, while stockAeb is set), so stock AEB does not depend on PCM arbitration alone (AOU-04R); or keep today's behaviour and rely on the AOU-04R vehicle test. Lead decision DQ-300</t>
-        </is>
-      </c>
-      <c r="D20" s="60" t="inlineStr"/>
-      <c r="E20" s="60" t="inlineStr">
-        <is>
-          <t>decision pending</t>
-        </is>
-      </c>
-      <c r="F20" s="60" t="inlineStr">
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>Stand down during stock AEB: while the car reports a stock PCS/AEB event (stockAeb), LionDriver requests zero acceleration, so stock AEB does not depend on PCM arbitration alone (AOU-04R). Lead decision DQ-300, option A (2026-10-18); the AOU-04R vehicle test still runs. Code change with the implementation-spec session; not in BL-006, so SFM-036 keeps its ratings</t>
+        </is>
+      </c>
+      <c r="D20" s="59" t="inlineStr"/>
+      <c r="E20" s="59" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F20" s="59" t="inlineStr">
         <is>
           <t>SFM-036.C1</t>
         </is>
       </c>
-      <c r="G20" s="60" t="inlineStr"/>
-      <c r="H20" s="60" t="inlineStr"/>
-      <c r="I20" s="60" t="inlineStr"/>
+      <c r="G20" s="59" t="inlineStr"/>
+      <c r="H20" s="59" t="inlineStr"/>
+      <c r="I20" s="59" t="inlineStr"/>
     </row>
     <row r="21" ht="73.5" customHeight="1">
-      <c r="A21" s="60" t="inlineStr">
+      <c r="A21" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-021</t>
         </is>
       </c>
-      <c r="B21" s="60" t="inlineStr">
+      <c r="B21" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C21" s="60" t="inlineStr">
+      <c r="C21" s="59" t="inlineStr">
         <is>
           <t>Make the insufficient-lateral-control warning timely (WP-S-04 §3.8.1): warn before the deficit has lasted 0.4 s, for example from the planned curvature against the envelope, or keep the deficit at or below about 0.5 m/s² through the steering limits and the ODD curve bound (WP-S-04 OI-2). A change to the ODD bound is a lead decision</t>
         </is>
       </c>
-      <c r="D21" s="60" t="inlineStr"/>
-      <c r="E21" s="60" t="inlineStr">
+      <c r="D21" s="59" t="inlineStr"/>
+      <c r="E21" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F21" s="60" t="inlineStr">
+      <c r="F21" s="59" t="inlineStr">
         <is>
           <t>SFM-038.C3</t>
         </is>
       </c>
-      <c r="G21" s="60" t="inlineStr"/>
-      <c r="H21" s="60" t="inlineStr"/>
-      <c r="I21" s="60" t="inlineStr"/>
+      <c r="G21" s="59" t="inlineStr"/>
+      <c r="H21" s="59" t="inlineStr"/>
+      <c r="I21" s="59" t="inlineStr"/>
     </row>
     <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="60" t="inlineStr">
+      <c r="A22" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-022</t>
         </is>
       </c>
-      <c r="B22" s="60" t="inlineStr">
+      <c r="B22" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C22" s="60" t="inlineStr">
+      <c r="C22" s="59" t="inlineStr">
         <is>
           <t>Measure the FCW onset after a lead brakes hard (WP-S-04 T-31, M-12) and compare it with the §3.8.2 budget (about 0.6 s at a 1.0 s gap). For pipeline lag (SFM-012.C1), detect it within that budget or show that the FCW path does not depend on the lagging process</t>
         </is>
       </c>
-      <c r="D22" s="60" t="inlineStr"/>
-      <c r="E22" s="60" t="inlineStr">
+      <c r="D22" s="59" t="inlineStr"/>
+      <c r="E22" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F22" s="60" t="inlineStr"/>
-      <c r="G22" s="60" t="inlineStr"/>
-      <c r="H22" s="60" t="inlineStr"/>
-      <c r="I22" s="60" t="inlineStr"/>
+      <c r="F22" s="59" t="inlineStr"/>
+      <c r="G22" s="59" t="inlineStr"/>
+      <c r="H22" s="59" t="inlineStr"/>
+      <c r="I22" s="59" t="inlineStr"/>
     </row>
     <row r="23" ht="195" customHeight="1">
-      <c r="A23" s="60" t="inlineStr">
+      <c r="A23" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-023</t>
         </is>
       </c>
-      <c r="B23" s="60" t="inlineStr">
+      <c r="B23" s="59" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C23" s="60" t="inlineStr">
+      <c r="C23" s="59" t="inlineStr">
         <is>
           <t>Escalate a temporary EPS fault that lasts while engaged to the take-over request (steerTempUnavailable, SOFT_DISABLE) instead of keeping the low-priority steerTempUnavailableSilent prompt latched after a recent override or at standstill (car_events.py; lead decision DQ-342, option A: the lighter prompt for at most 1.5 s, then the take-over request; TSR-607 (b)). SFM-038.C1; FTA BE-2.08</t>
         </is>
       </c>
-      <c r="D23" s="60" t="inlineStr"/>
-      <c r="E23" s="61" t="inlineStr">
+      <c r="D23" s="59" t="inlineStr"/>
+      <c r="E23" s="60" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F23" s="60" t="inlineStr">
+      <c r="F23" s="59" t="inlineStr">
         <is>
           <t>SFM-038.C1</t>
         </is>
       </c>
-      <c r="G23" s="60" t="inlineStr">
+      <c r="G23" s="59" t="inlineStr">
         <is>
           <t>10/5/8</t>
         </is>
       </c>
-      <c r="H23" s="62" t="inlineStr">
+      <c r="H23" s="61" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="I23" s="60" t="inlineStr">
+      <c r="I23" s="59" t="inlineStr">
         <is>
           <t>Merged in jherrodthomas/LionDriver#174 (7158a9a): STEER_FAULT_SILENT_FRAMES in car_events.py limits the lighter prompt to the first 1.5 s of the fault; selfdrive/car/tests/test_steer_fault_warning.py, 6 tests run in CI, 4 of them fail on the old code. Impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Unit-tested only: not verified on the vehicle (impact OI-1) and not reviewed independently. Credited at BL-006 (System FMEA rev 0.27): SFM-038.C1 O 8 -&gt; 5, D 10 -&gt; 8, AP stays H (S 10): the tests are targeted but not proven by mutation, so D 8 rather than the D 4 predicted below (rating tables D 8; a car_events.py mutation run, planned with SWF-ACT-077, would support D 4); f350f5b adds TSR-607 (c) for a fault while the driver steers</t>
         </is>
       </c>
     </row>
     <row r="24" ht="87" customHeight="1">
-      <c r="A24" s="60" t="inlineStr">
+      <c r="A24" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-024</t>
         </is>
       </c>
-      <c r="B24" s="60" t="inlineStr">
+      <c r="B24" s="59" t="inlineStr">
         <is>
           <t>monitoring</t>
         </is>
       </c>
-      <c r="C24" s="60" t="inlineStr">
+      <c r="C24" s="59" t="inlineStr">
         <is>
           <t>Act on the panda fields epsFault and requestsRejected on the host (TSR-626(d), TSR-516(b)): raise the take-over request when the panda reports an EPS fault or refused steering frames while lateral control is engaged, within the SG-02 1 s budget, instead of relying on the panda siren alone. Split from SFM-ACT-023 (rev 0.25). SFM-038.C2; FTA BE-2.08</t>
         </is>
       </c>
-      <c r="D24" s="60" t="inlineStr"/>
-      <c r="E24" s="60" t="inlineStr">
+      <c r="D24" s="59" t="inlineStr"/>
+      <c r="E24" s="59" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F24" s="60" t="inlineStr">
+      <c r="F24" s="59" t="inlineStr">
         <is>
           <t>SFM-038.C2</t>
         </is>
       </c>
-      <c r="G24" s="60" t="inlineStr"/>
-      <c r="H24" s="60" t="inlineStr"/>
-      <c r="I24" s="60" t="inlineStr"/>
+      <c r="G24" s="59" t="inlineStr"/>
+      <c r="H24" s="59" t="inlineStr"/>
+      <c r="I24" s="59" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I24"/>
@@ -19461,50 +19458,50 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="59" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Element</t>
         </is>
       </c>
-      <c r="B1" s="59" t="inlineStr">
+      <c r="B1" s="58" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="59" t="inlineStr">
+      <c r="C1" s="58" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="D1" s="59" t="inlineStr">
+      <c r="D1" s="58" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="E1" s="59" t="inlineStr">
+      <c r="E1" s="58" t="inlineStr">
         <is>
           <t>Functions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="222" customHeight="1">
-      <c r="A2" s="60" t="inlineStr">
+      <c r="A2" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="B2" s="60" t="inlineStr">
+      <c r="B2" s="59" t="inlineStr">
         <is>
           <t>LionDriver item (L2 ACC + ALC + driver monitoring)</t>
         </is>
       </c>
-      <c r="C2" s="60" t="inlineStr">
+      <c r="C2" s="59" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D2" s="60" t="inlineStr"/>
-      <c r="E2" s="60" t="inlineStr">
+      <c r="D2" s="59" t="inlineStr"/>
+      <c r="E2" s="59" t="inlineStr">
         <is>
           <t>SFM-FN-001: F1 Lateral control: request steering torque from the EPS to keep the vehicle in its lane while engaged
 SFM-FN-002: F2 Longitudinal control: request acceleration/deceleration to hold set speed and follow leads while engaged
@@ -19518,398 +19515,398 @@
       </c>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="60" t="inlineStr">
+      <c r="A3" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="B3" s="60" t="inlineStr">
+      <c r="B3" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">    comma 3X device</t>
         </is>
       </c>
-      <c r="C3" s="60" t="inlineStr">
+      <c r="C3" s="59" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="D3" s="60" t="inlineStr">
+      <c r="D3" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E3" s="60" t="inlineStr"/>
+      <c r="E3" s="59" t="inlineStr"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="60" t="inlineStr">
+      <c r="A4" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-003</t>
         </is>
       </c>
-      <c r="B4" s="60" t="inlineStr">
+      <c r="B4" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Integrated panda (CAN interface and safety model)</t>
         </is>
       </c>
-      <c r="C4" s="60" t="inlineStr">
+      <c r="C4" s="59" t="inlineStr">
         <is>
           <t>subsystem</t>
         </is>
       </c>
-      <c r="D4" s="60" t="inlineStr">
+      <c r="D4" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E4" s="60" t="inlineStr"/>
+      <c r="E4" s="59" t="inlineStr"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="60" t="inlineStr">
+      <c r="A5" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-004</t>
         </is>
       </c>
-      <c r="B5" s="60" t="inlineStr">
+      <c r="B5" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">    Harness (Toyota A connector, harness box, comma power v3)</t>
         </is>
       </c>
-      <c r="C5" s="60" t="inlineStr">
+      <c r="C5" s="59" t="inlineStr">
         <is>
           <t>component</t>
         </is>
       </c>
-      <c r="D5" s="60" t="inlineStr">
+      <c r="D5" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-001</t>
         </is>
       </c>
-      <c r="E5" s="60" t="inlineStr"/>
+      <c r="E5" s="59" t="inlineStr"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-010</t>
         </is>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Perception (camerad, modeld)</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E6" s="60" t="inlineStr"/>
+      <c r="E6" s="59" t="inlineStr"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="60" t="inlineStr">
+      <c r="A7" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-011</t>
         </is>
       </c>
-      <c r="B7" s="60" t="inlineStr">
+      <c r="B7" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Localization and calibration (locationd, calibrationd, paramsd, torqued)</t>
         </is>
       </c>
-      <c r="C7" s="60" t="inlineStr">
+      <c r="C7" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D7" s="60" t="inlineStr">
+      <c r="D7" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E7" s="60" t="inlineStr"/>
+      <c r="E7" s="59" t="inlineStr"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="60" t="inlineStr">
+      <c r="A8" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-012</t>
         </is>
       </c>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="B8" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Planning (plannerd, radard)</t>
         </is>
       </c>
-      <c r="C8" s="60" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D8" s="60" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E8" s="60" t="inlineStr"/>
+      <c r="E8" s="59" t="inlineStr"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="60" t="inlineStr">
+      <c r="A9" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-013</t>
         </is>
       </c>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="B9" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Control (controlsd, lateral/longitudinal controllers)</t>
         </is>
       </c>
-      <c r="C9" s="60" t="inlineStr">
+      <c r="C9" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D9" s="60" t="inlineStr">
+      <c r="D9" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E9" s="60" t="inlineStr"/>
+      <c r="E9" s="59" t="inlineStr"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="60" t="inlineStr">
+      <c r="A10" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-014</t>
         </is>
       </c>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B10" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Supervision (selfdrived state machine, events, alert manager)</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E10" s="60" t="inlineStr"/>
+      <c r="E10" s="59" t="inlineStr"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="60" t="inlineStr">
+      <c r="A11" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-015</t>
         </is>
       </c>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="B11" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Driver monitoring (dmonitoringmodeld, dmonitoringd)</t>
         </is>
       </c>
-      <c r="C11" s="60" t="inlineStr">
+      <c r="C11" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D11" s="60" t="inlineStr">
+      <c r="D11" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E11" s="60" t="inlineStr"/>
+      <c r="E11" s="59" t="inlineStr"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="60" t="inlineStr">
+      <c r="A12" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-016</t>
         </is>
       </c>
-      <c r="B12" s="60" t="inlineStr">
+      <c r="B12" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Car interface (card, car_events, opendbc Toyota port)</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C12" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D12" s="60" t="inlineStr">
+      <c r="D12" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E12" s="60" t="inlineStr"/>
+      <c r="E12" s="59" t="inlineStr"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="60" t="inlineStr">
+      <c r="A13" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-017</t>
         </is>
       </c>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Panda daemon (pandad)</t>
         </is>
       </c>
-      <c r="C13" s="60" t="inlineStr">
+      <c r="C13" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D13" s="60" t="inlineStr">
+      <c r="D13" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E13" s="60" t="inlineStr"/>
+      <c r="E13" s="59" t="inlineStr"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="60" t="inlineStr">
+      <c r="A14" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-018</t>
         </is>
       </c>
-      <c r="B14" s="60" t="inlineStr">
+      <c r="B14" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        HMI (ui, soundd)</t>
         </is>
       </c>
-      <c r="C14" s="60" t="inlineStr">
+      <c r="C14" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D14" s="60" t="inlineStr">
+      <c r="D14" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E14" s="60" t="inlineStr"/>
+      <c r="E14" s="59" t="inlineStr"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="60" t="inlineStr">
+      <c r="A15" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-019</t>
         </is>
       </c>
-      <c r="B15" s="60" t="inlineStr">
+      <c r="B15" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">        Platform (manager, messaging, hardwared, OS)</t>
         </is>
       </c>
-      <c r="C15" s="60" t="inlineStr">
+      <c r="C15" s="59" t="inlineStr">
         <is>
           <t>sw_element</t>
         </is>
       </c>
-      <c r="D15" s="60" t="inlineStr">
+      <c r="D15" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-002</t>
         </is>
       </c>
-      <c r="E15" s="60" t="inlineStr"/>
+      <c r="E15" s="59" t="inlineStr"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="60" t="inlineStr">
+      <c r="A16" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-030</t>
         </is>
       </c>
-      <c r="B16" s="60" t="inlineStr">
+      <c r="B16" s="59" t="inlineStr">
         <is>
           <t>Toyota EPS</t>
         </is>
       </c>
-      <c r="C16" s="60" t="inlineStr">
+      <c r="C16" s="59" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D16" s="60" t="inlineStr"/>
-      <c r="E16" s="60" t="inlineStr"/>
+      <c r="D16" s="59" t="inlineStr"/>
+      <c r="E16" s="59" t="inlineStr"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="60" t="inlineStr">
+      <c r="A17" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-031</t>
         </is>
       </c>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="B17" s="59" t="inlineStr">
         <is>
           <t>Toyota powertrain and brake control (receives ACC acceleration requests)</t>
         </is>
       </c>
-      <c r="C17" s="60" t="inlineStr">
+      <c r="C17" s="59" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D17" s="60" t="inlineStr"/>
-      <c r="E17" s="60" t="inlineStr"/>
+      <c r="D17" s="59" t="inlineStr"/>
+      <c r="E17" s="59" t="inlineStr"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="60" t="inlineStr">
+      <c r="A18" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-032</t>
         </is>
       </c>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="B18" s="59" t="inlineStr">
         <is>
           <t>Toyota stock ADAS camera (TSS2)</t>
         </is>
       </c>
-      <c r="C18" s="60" t="inlineStr">
+      <c r="C18" s="59" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D18" s="60" t="inlineStr"/>
-      <c r="E18" s="60" t="inlineStr"/>
+      <c r="D18" s="59" t="inlineStr"/>
+      <c r="E18" s="59" t="inlineStr"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="60" t="inlineStr">
+      <c r="A19" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-033</t>
         </is>
       </c>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="B19" s="59" t="inlineStr">
         <is>
           <t>Vehicle CAN buses and 12 V supply</t>
         </is>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="59" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D19" s="60" t="inlineStr"/>
-      <c r="E19" s="60" t="inlineStr"/>
+      <c r="D19" s="59" t="inlineStr"/>
+      <c r="E19" s="59" t="inlineStr"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="60" t="inlineStr">
+      <c r="A20" s="59" t="inlineStr">
         <is>
           <t>SFM-SE-034</t>
         </is>
       </c>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="B20" s="59" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
+      <c r="C20" s="59" t="inlineStr">
         <is>
           <t>external</t>
         </is>
       </c>
-      <c r="D20" s="60" t="inlineStr"/>
-      <c r="E20" s="60" t="inlineStr"/>
+      <c r="D20" s="59" t="inlineStr"/>
+      <c r="E20" s="59" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E20"/>
@@ -19945,7 +19942,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>FMEA-MSR (monitoring and system response, msr-plan.md): S, F, M and MSR AP per rating-tables.md §7 (RT-2). The MSR AP table is provisional until the handbook table is transcribed (decision register DQ-207). Exempt causes are rated in the FMEA named in the reason.</t>
         </is>
@@ -22702,7 +22699,7 @@
           <t>Device power loss (12 V interruption, harness connector)</t>
         </is>
       </c>
-      <c r="E44" s="64" t="inlineStr">
+      <c r="E44" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-012.C1)</t>
         </is>
@@ -22996,7 +22993,7 @@
           <t>The panda envelope passes STEERING_LKA torque that opposes the driver while the driver overrides: the Toyota LKA check covers magnitude, rate and measured-torque error only, and STEER_TORQUE_DRIVER is used only on the LTA path (toyota.h:298-310, 421-424; GAP-02). TSR-304 is not implemented in either build, so only the host 500-unit cut-off (C1, C2) stops the torque</t>
         </is>
       </c>
-      <c r="E49" s="64" t="inlineStr">
+      <c r="E49" s="63" t="inlineStr">
         <is>
           <t>Exempt: The cause is the missing panda override supervision itself, which is the MSR mechanism of C1 and C2; its absence is rated there as M 10 (msr-plan §3)</t>
         </is>
@@ -23860,7 +23857,7 @@
           <t>Panda MCU hardware fault (see DFMEA/FMEDA)</t>
         </is>
       </c>
-      <c r="E63" s="64" t="inlineStr">
+      <c r="E63" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-001.C1)</t>
         </is>
@@ -24020,7 +24017,7 @@
           <t>Switch U1 or U2 stuck in intercept, its IN input damaged high or driven high, its pull-down R2/R3 open, or the switches damaged by box supply transients (DG419LE, RR-2026-010)</t>
         </is>
       </c>
-      <c r="E66" s="64" t="inlineStr">
+      <c r="E66" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-010.C1)</t>
         </is>
@@ -24056,7 +24053,7 @@
           <t>Switch stuck in pass-through, or the SBU1 drive lost, held low or too low to change the switch over (5 V drive against VL = VIN)</t>
         </is>
       </c>
-      <c r="E67" s="64" t="inlineStr">
+      <c r="E67" s="63" t="inlineStr">
         <is>
           <t>Exempt: Hardware cause; rated once in the DFMEA (DFM-011.C1)</t>
         </is>
@@ -24250,7 +24247,7 @@
       </c>
       <c r="N70" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-020 · decision pending</t>
+          <t>SFM-ACT-020 · open</t>
         </is>
       </c>
       <c r="O70" s="37" t="inlineStr"/>
@@ -24312,7 +24309,7 @@
       </c>
       <c r="N71" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-020 · decision pending</t>
+          <t>SFM-ACT-020 · open</t>
         </is>
       </c>
       <c r="O71" s="37" t="inlineStr"/>
@@ -24532,7 +24529,7 @@
           <t>The lighter EPS-fault prompt (steerTempUnavailableSilent, a LOW-priority WARNING with a chime and no soft disable, events.py:516-521) after a recent override, at standstill or while the driver steers is not limited to 1.5 s, so a long fault does not escalate to the take-over request (car_events.py:167-185, STEER_FAULT_SILENT_FRAMES; T-25, GAP-03). Until BL-005 the prompt was latched for the whole fault by design; from BL-006 the cause is a defect of the TSR-607 (b)/(c) frame counter</t>
         </is>
       </c>
-      <c r="E75" s="64" t="inlineStr">
+      <c r="E75" s="63" t="inlineStr">
         <is>
           <t>Exempt: The cause is a defect of the warning path itself; its effect on detecting the lateral loss is rated in the MSR rows of SFM-004.C2 and SFM-005 (msr-plan §3)</t>
         </is>
@@ -24568,7 +24565,7 @@
           <t>pandad publishes the panda fields epsFault and requestsRejected (pandad.cc:137-138), but no SoC process reads them (txRateExceeded is read, TSR-615), so a panda-side EPS-fault refusal reaches the driver only through the panda siren and the stock EPS path (SW FMEA SWF-025 notes)</t>
         </is>
       </c>
-      <c r="E76" s="64" t="inlineStr">
+      <c r="E76" s="63" t="inlineStr">
         <is>
           <t>Exempt: The cause is a defect of the warning path itself; the panda siren that remains is rated on SFM-005 and in the DFMEA (msr-plan §3)</t>
         </is>
@@ -24604,7 +24601,7 @@
           <t>steerSaturated needs the controller saturated, a desired lateral acceleration above 1.0 m/s², an undershoot above 1.2x and no steering input for 2 s (selfdrived.py:465-479), and the controller reports saturation only after 0.4 s (latcontrol.py, T-30); a gradual deficit therefore warns late or not at all (WP-S-04 §3.8.1)</t>
         </is>
       </c>
-      <c r="E77" s="64" t="inlineStr">
+      <c r="E77" s="63" t="inlineStr">
         <is>
           <t>Exempt: The cause is the timing of the warning itself; it is rated as M 8 in the MSR rows of SFM-004.C1-C3 (rev 0.15, WP-S-04 §3.8.1)</t>
         </is>
@@ -24635,7 +24632,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.28 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.29 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.31: SFM-ACT-020 completed for the host code (#292)
SFM-ACT-020 (DQ-300 A, stand down during stock AEB) is implemented in
#292 (c045874). Evidence cites the 4 local-only unit tests (CI scons
blocked by the LFS 404), the impact record and its open items OI-1..3.
Predicted rating S10 O5 D8 AP H. The change is not in BL-006, so
SFM-036.C1 keeps O8 D10. fmea-plan v0.24. Generated outputs regenerated.
AI-drafted; not reviewed independently.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.30 · draft</t>
+          <t>0.31 · draft</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>23 (20)</t>
+          <t>23 (19)</t>
         </is>
       </c>
     </row>
@@ -17033,7 +17033,7 @@
       <c r="R86" s="45" t="inlineStr"/>
       <c r="S86" s="45" t="inlineStr"/>
     </row>
-    <row r="87" ht="141" customHeight="1">
+    <row r="87" ht="114" customHeight="1">
       <c r="A87" s="30" t="inlineStr">
         <is>
           <r>
@@ -17261,17 +17261,25 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Stand down during stock AEB: while the car reports a stock PCS/AEB event (stockAeb), LionDriver requests zero acceleration, so stock AEB does not depend on PCM arbitration alone (AOU-04R). Lead decision DQ-300, option A (2026-10-18); the AOU-04R vehicle test still runs. Code change with the implementation-spec session; not in BL-006, so SFM-036 keeps its ratings</t>
-          </r>
-        </is>
-      </c>
-      <c r="O87" s="47" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="P87" s="33" t="inlineStr"/>
-      <c r="Q87" s="33" t="inlineStr"/>
+            <t>Stand down during stock AEB: while the car reports a stock PCS/AEB event (stockAeb), LionDriver requests zero acceleration, so stock AEB does not depend on PCM arbitration alone (AOU-04R). Lead decision DQ-300, option A (2026-10-18); the AOU-04R vehicle test still runs. SFM-036.C1; FTA BE-7.13</t>
+          </r>
+        </is>
+      </c>
+      <c r="O87" s="54" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="P87" s="33" t="inlineStr">
+        <is>
+          <t>10/5/8</t>
+        </is>
+      </c>
+      <c r="Q87" s="36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
       <c r="R87" s="37" t="inlineStr"/>
       <c r="S87" s="37" t="inlineStr"/>
     </row>
@@ -18539,7 +18547,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.30 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.31 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -19275,7 +19283,7 @@
       <c r="H19" s="59" t="inlineStr"/>
       <c r="I19" s="59" t="inlineStr"/>
     </row>
-    <row r="20" ht="87" customHeight="1">
+    <row r="20" ht="235.5" customHeight="1">
       <c r="A20" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-020</t>
@@ -19288,13 +19296,13 @@
       </c>
       <c r="C20" s="59" t="inlineStr">
         <is>
-          <t>Stand down during stock AEB: while the car reports a stock PCS/AEB event (stockAeb), LionDriver requests zero acceleration, so stock AEB does not depend on PCM arbitration alone (AOU-04R). Lead decision DQ-300, option A (2026-10-18); the AOU-04R vehicle test still runs. Code change with the implementation-spec session; not in BL-006, so SFM-036 keeps its ratings</t>
+          <t>Stand down during stock AEB: while the car reports a stock PCS/AEB event (stockAeb), LionDriver requests zero acceleration, so stock AEB does not depend on PCM arbitration alone (AOU-04R). Lead decision DQ-300, option A (2026-10-18); the AOU-04R vehicle test still runs. SFM-036.C1; FTA BE-7.13</t>
         </is>
       </c>
       <c r="D20" s="59" t="inlineStr"/>
-      <c r="E20" s="59" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="E20" s="60" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="F20" s="59" t="inlineStr">
@@ -19302,9 +19310,21 @@
           <t>SFM-036.C1</t>
         </is>
       </c>
-      <c r="G20" s="59" t="inlineStr"/>
-      <c r="H20" s="59" t="inlineStr"/>
-      <c r="I20" s="59" t="inlineStr"/>
+      <c r="G20" s="59" t="inlineStr">
+        <is>
+          <t>10/5/8</t>
+        </is>
+      </c>
+      <c r="H20" s="61" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="I20" s="59" t="inlineStr">
+        <is>
+          <t>Merged in jherrodthomas/LionDriver#292 (c045874): stock_aeb_stand_down in longcontrol.py, called from controlsd.py, caps the acceleration target and the upper PID limit at 0 m/s² while stockAeb is set and keeps any braking request; selfdrive/controls/tests/test_stock_aeb.py, 4 tests, run locally only (CI scons is blocked by the LFS 404, DQ-401; cite the CI run once it re-runs). Impact record assurance/07-supporting/impact/change-2026-10-19-stock-aeb-stand-down.md. Host code only: the opendbc Toyota controller still applies its rate limit and positive terms, so the command reaches 0 about 0.4 s after +1.5 m/s² (impact OI-2); the parent TSR/SWSR are open (OI-1); not verified on the vehicle (OI-3, the AOU-04R test, also checks that stockAeb is reported during a PCS event) and not reviewed independently. Not in BL-006, so SFM-036.C1 keeps O 8 D 10 until the next baseline; the prediction below assumes targeted tests, not mutation-proven (rating tables D 8)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="73.5" customHeight="1">
       <c r="A21" s="59" t="inlineStr">
@@ -24250,7 +24270,7 @@
       </c>
       <c r="N70" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-020 · open</t>
+          <t>SFM-ACT-020 · completed</t>
         </is>
       </c>
       <c r="O70" s="37" t="inlineStr"/>
@@ -24312,7 +24332,7 @@
       </c>
       <c r="N71" s="34" t="inlineStr">
         <is>
-          <t>SFM-ACT-020 · open</t>
+          <t>SFM-ACT-020 · completed</t>
         </is>
       </c>
       <c r="O71" s="37" t="inlineStr"/>
@@ -24635,7 +24655,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.30 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.31 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
System FMEA rev 0.32: SFM-ACT-020 evidence cites CI and the opendbc cap
The LFS mirror is back. Tests run 39296172878 on liondriver-dev 6126485
passed: unit tests 1578 passed, 42 skipped, 3 xfailed, process replay
green. The runner collects every openpilot test file and prints no names,
so test_stock_aeb.py is shown to have run by collection, not by name.
The evidence also cites opendbc e233362 (#311), which closes impact OI-2,
and TSR-713 implemented (#313). Ratings unchanged; fmea-plan v0.25.
AI-drafted; not reviewed independently.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.31 · draft</t>
+          <t>0.32 · draft</t>
         </is>
       </c>
     </row>
@@ -18547,7 +18547,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.31 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.32 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -19283,7 +19283,7 @@
       <c r="H19" s="59" t="inlineStr"/>
       <c r="I19" s="59" t="inlineStr"/>
     </row>
-    <row r="20" ht="235.5" customHeight="1">
+    <row r="20" ht="343.5" customHeight="1">
       <c r="A20" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-020</t>
@@ -19322,7 +19322,7 @@
       </c>
       <c r="I20" s="59" t="inlineStr">
         <is>
-          <t>Merged in jherrodthomas/LionDriver#292 (c045874): stock_aeb_stand_down in longcontrol.py, called from controlsd.py, caps the acceleration target and the upper PID limit at 0 m/s² while stockAeb is set and keeps any braking request; selfdrive/controls/tests/test_stock_aeb.py, 4 tests, run locally only (CI scons is blocked by the LFS 404, DQ-401; cite the CI run once it re-runs). Impact record assurance/07-supporting/impact/change-2026-10-19-stock-aeb-stand-down.md. Host code only: the opendbc Toyota controller still applies its rate limit and positive terms, so the command reaches 0 about 0.4 s after +1.5 m/s² (impact OI-2); the parent TSR/SWSR are open (OI-1); not verified on the vehicle (OI-3, the AOU-04R test, also checks that stockAeb is reported during a PCS event) and not reviewed independently. Not in BL-006, so SFM-036.C1 keeps O 8 D 10 until the next baseline; the prediction below assumes targeted tests, not mutation-proven (rating tables D 8)</t>
+          <t>Merged in jherrodthomas/LionDriver#292 (c045874): stock_aeb_stand_down in longcontrol.py, called from controlsd.py, caps the acceleration target and the upper PID limit at 0 m/s² while stockAeb is set and keeps any braking request; selfdrive/controls/tests/test_stock_aeb.py, 4 tests. CI: tests run 39296172878 on liondriver-dev 6126485 (2026-10-19), unit tests job 1578 passed, 42 skipped, 3 xfailed, no failures or collection errors; process replay passed. The runner collects every openpilot/**/test_*.py and prints no test names, so the four tests are shown to have run by collection, not by name; the file has no skip. Second layer, opendbc e233362 (#311, SWSR-713h): the Toyota controller caps the 0x343 command at 0 from the first frame of the event, after its rate limit, PID and pitch compensation (impact OI-2 done); its 6 test_carcontroller.py cases ran locally only (opendbc_repo tests are not in the openpilot runner). Impact records assurance/07-supporting/impact/change-2026-10-19-stock-aeb-stand-down.md and change-2026-10-19-pin-e233362.md. TSR-713 and FSR-07.07 implemented (#313). Not verified on the vehicle (OI-3, the AOU-04R test, also checks that stockAeb is reported during a PCS event) and not reviewed independently. Not in BL-006, so SFM-036.C1 keeps O 8 D 10 until the next baseline; the prediction below assumes targeted tests, not mutation-proven (rating tables D 8)</t>
         </is>
       </c>
     </row>
@@ -24655,7 +24655,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.31 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.32 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
SFM-ACT-020: fix YAML quoting broken by c3ad0c6
An apostrophe in a single-quoted evidence string closed it early, so the
FMEA tools could not parse system-fmea.yaml. Reworded; regenerated; ci.sh
FAIL=0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -19283,7 +19283,7 @@
       <c r="H19" s="59" t="inlineStr"/>
       <c r="I19" s="59" t="inlineStr"/>
     </row>
-    <row r="20" ht="343.5" customHeight="1">
+    <row r="20" ht="384" customHeight="1">
       <c r="A20" s="59" t="inlineStr">
         <is>
           <t>SFM-ACT-020</t>
@@ -19322,7 +19322,7 @@
       </c>
       <c r="I20" s="59" t="inlineStr">
         <is>
-          <t>Merged in jherrodthomas/LionDriver#292 (c045874): stock_aeb_stand_down in longcontrol.py, called from controlsd.py, caps the acceleration target and the upper PID limit at 0 m/s² while stockAeb is set and keeps any braking request; selfdrive/controls/tests/test_stock_aeb.py, 4 tests. CI: tests run 39296172878 on liondriver-dev 6126485 (2026-10-19), unit tests job 1578 passed, 42 skipped, 3 xfailed, no failures or collection errors; process replay passed. The runner collects every openpilot/**/test_*.py and prints no test names, so the four tests are shown to have run by collection, not by name; the file has no skip. Second layer, opendbc e233362 (#311, SWSR-713h): the Toyota controller caps the 0x343 command at 0 from the first frame of the event, after its rate limit, PID and pitch compensation (impact OI-2 done); its 6 test_carcontroller.py cases ran locally only (opendbc_repo tests are not in the openpilot runner). Impact records assurance/07-supporting/impact/change-2026-10-19-stock-aeb-stand-down.md and change-2026-10-19-pin-e233362.md. TSR-713 and FSR-07.07 implemented (#313). Not verified on the vehicle (OI-3, the AOU-04R test, also checks that stockAeb is reported during a PCS event) and not reviewed independently. Not in BL-006, so SFM-036.C1 keeps O 8 D 10 until the next baseline; the prediction below assumes targeted tests, not mutation-proven (rating tables D 8)</t>
+          <t>Merged in jherrodthomas/LionDriver#292 (c045874): stock_aeb_stand_down in longcontrol.py, called from controlsd.py, caps the acceleration target and the upper PID limit at 0 m/s² while stockAeb is set and keeps any braking request; selfdrive/controls/tests/test_stock_aeb.py, 4 tests. CI: tests run 39296172878 on liondriver-dev 6126485 (2026-10-19), unit tests job 1578 passed, 42 skipped, 3 xfailed, no failures or collection errors; process replay passed. The runner collects every openpilot/**/test_*.py and prints no test names, so the four tests are shown to have run by collection, not by name; the file has no skip. Second layer, opendbc e233362 (#311, SWSR-713h): the Toyota controller caps the 0x343 command at 0 from the first frame of the event, after its rate limit, PID and pitch compensation (impact OI-2 done); its 6 test_carcontroller.py cases ran locally (pin record). The openpilot runner does not run opendbc_repo tests; tests.yml in the opendbc fork triggers on pull requests, but a CI run on jherrodthomas/opendbc#20 is not confirmed here (the pin record says none). Impact records assurance/07-supporting/impact/change-2026-10-19-stock-aeb-stand-down.md and change-2026-10-19-pin-e233362.md. TSR-713 and FSR-07.07 implemented (#313). Not verified on the vehicle (OI-3, the AOU-04R test, also checks that stockAeb is reported during a PCS event) and not reviewed independently. Not in BL-006, so SFM-036.C1 keeps O 8 D 10 until the next baseline; the prediction below assumes targeted tests, not mutation-proven (rating tables D 8)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
System FMEA rev 0.33: SFM-005.C2 and SFM-006.C1 record the panda siren on a SoC stall
From the FSC/TSC routes walk (#395). Since panda 8a69ccf (DQ-404 A, kept in
f4803c5) the panda sounds its own siren when it revokes authority because
command frames stopped (TSR-516(b)). The plant model F-04b at panda f4803c5
shows the siren at 0.25 s. Both causes now say so in their mechanism and
evidence. The change is after BL-006, so no rating changes. fmea-plan v0.29.
AI-drafted; not reviewed independently.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/system-fmea-review.xlsx
@@ -823,7 +823,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.32 · draft</t>
+          <t>0.33 · draft</t>
         </is>
       </c>
     </row>
@@ -18547,7 +18547,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.32 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · rev 0.33 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -21030,7 +21030,7 @@
       <c r="O17" s="37" t="inlineStr"/>
       <c r="P17" s="37" t="inlineStr"/>
     </row>
-    <row r="18" ht="141" customHeight="1">
+    <row r="18" ht="195" customHeight="1">
       <c r="A18" s="34" t="inlineStr">
         <is>
           <t>SFM-005 · Loss of lateral control without driver alert</t>
@@ -21051,7 +21051,7 @@
       </c>
       <c r="E18" s="34" t="inlineStr">
         <is>
-          <t>BL-005: when no STEERING_LKA frame reaches the panda for 50 ms while authority is granted, the 100 Hz safety task clears controls_allowed (tx_arrival_ok, safety.h; TSR-408). pandad keeps publishing pandaStates, so selfdrived sees controlsAllowed false on the next sample and raises controlsMismatch after 2 consecutive samples, at most 0.5 s after the first mismatched frame (TSR-621). At BL-004 only the EPS drop-out path existed (about 3.5 s)</t>
+          <t>BL-005: when no STEERING_LKA frame reaches the panda for 50 ms while authority is granted, the 100 Hz safety task clears controls_allowed (tx_arrival_ok, safety.h; TSR-408). pandad keeps publishing pandaStates, so selfdrived sees controlsAllowed false on the next sample and raises controlsMismatch after 2 consecutive samples, at most 0.5 s after the first mismatched frame (TSR-621). At BL-004 only the EPS drop-out path existed (about 3.5 s). After BL-006 (panda 8a69ccf, DQ-404 A; kept in f4803c5) the panda also sounds its own siren on this revocation, independent of the SoC (TSR-516(b)); not in BL-006, so the rating below does not credit it</t>
         </is>
       </c>
       <c r="F18" s="34" t="inlineStr">
@@ -21160,7 +21160,7 @@
       <c r="O19" s="37" t="inlineStr"/>
       <c r="P19" s="37" t="inlineStr"/>
     </row>
-    <row r="20" ht="100.5" customHeight="1">
+    <row r="20" ht="127.5" customHeight="1">
       <c r="A20" s="34" t="inlineStr">
         <is>
           <t>SFM-006 · Lateral command frozen at last value</t>
@@ -21191,7 +21191,7 @@
       </c>
       <c r="G20" s="34" t="inlineStr">
         <is>
-          <t>Last torque command held about 0.1 s, then LKA frames stop and assist decays over about 2 s. The driver is now warned within about 0.66 s, but the actuation reaction is still beyond the 0.5 s FTTI</t>
+          <t>Last torque command held about 0.1 s, then LKA frames stop and assist decays over about 2 s. The driver is now warned within about 0.66 s (after BL-006 the panda siren comes first, about 0.25 s after the last frame, DQ-404), but the actuation reaction is still beyond the 0.5 s FTTI</t>
         </is>
       </c>
       <c r="H20" s="35" t="n">
@@ -24655,7 +24655,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.32 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSystem FMEA — LionDriver L2 ACC/ALC item · FMEA-MSR · rev 0.33 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>